<commit_message>
Limit competitor list to 20 sites
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01GGxzKXyeNbw77cRhpGHusQ
</commit_message>
<xml_diff>
--- a/out/analiz_konkurentov_reiginmed.xlsx
+++ b/out/analiz_konkurentov_reiginmed.xlsx
@@ -11,7 +11,7 @@
     <sheet name="Технический лист" sheetId="6" state="hidden" r:id="rId6"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Анализ конкурентов'!$A$1:$V$44</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Анализ конкурентов'!$A$1:$V$23</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -3019,7 +3019,7 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:X44"/>
+  <dimension ref="A1:X23"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.63" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
     <col width="3.13" customWidth="1" style="354" min="1" max="1"/>
@@ -4181,7 +4181,7 @@
       </c>
       <c r="B20" s="28" t="inlineStr">
         <is>
-          <t>https://vendem.ru/</t>
+          <t>https://intelmed.ru/</t>
         </is>
       </c>
       <c r="C20" s="31">
@@ -4201,12 +4201,8 @@
       <c r="K20" s="131" t="n"/>
       <c r="L20" s="40" t="n"/>
       <c r="M20" s="41" t="n"/>
-      <c r="N20" s="42" t="n">
-        <v>876</v>
-      </c>
-      <c r="O20" s="255" t="n">
-        <v>13675</v>
-      </c>
+      <c r="N20" s="42" t="n"/>
+      <c r="O20" s="255" t="n"/>
       <c r="P20" s="44" t="n"/>
       <c r="Q20" s="311" t="n"/>
       <c r="R20" s="46">
@@ -4226,7 +4222,7 @@
       <c r="W20" s="50" t="n"/>
       <c r="X20" s="262" t="inlineStr">
         <is>
-          <t>Слабый конкурент</t>
+          <t>Более широкий конкурент</t>
         </is>
       </c>
     </row>
@@ -4237,7 +4233,7 @@
       </c>
       <c r="B21" s="28" t="inlineStr">
         <is>
-          <t>https://redsrus.ru/</t>
+          <t>https://kriptomed.ru/</t>
         </is>
       </c>
       <c r="C21" s="31">
@@ -4257,12 +4253,8 @@
       <c r="K21" s="131" t="n"/>
       <c r="L21" s="40" t="n"/>
       <c r="M21" s="41" t="n"/>
-      <c r="N21" s="42" t="n">
-        <v>858</v>
-      </c>
-      <c r="O21" s="255" t="n">
-        <v>8125</v>
-      </c>
+      <c r="N21" s="42" t="n"/>
+      <c r="O21" s="255" t="n"/>
       <c r="P21" s="44" t="n"/>
       <c r="Q21" s="311" t="n"/>
       <c r="R21" s="46">
@@ -4282,7 +4274,7 @@
       <c r="W21" s="50" t="n"/>
       <c r="X21" s="262" t="inlineStr">
         <is>
-          <t>Слабый конкурент</t>
+          <t>Более широкий конкурент</t>
         </is>
       </c>
     </row>
@@ -4291,56 +4283,84 @@
         <f>IMAGE(C22)</f>
         <v/>
       </c>
-      <c r="B22" s="28" t="inlineStr">
-        <is>
-          <t>https://lmed.ru/</t>
-        </is>
-      </c>
-      <c r="C22" s="31">
-        <f>"https://www.google.com/s2/favicons?domain="&amp;B22</f>
-        <v/>
-      </c>
-      <c r="D22" s="31">
-        <f>"https://a.pr-cy.ru/"&amp;IF(ISERROR(FIND("//www.",B22)),MID(B22,FIND(":",B22,4)+3,FIND("/",B22,9)-FIND(":",B22,4)-3),MID(B22,FIND(":",B22,4)+7,FIND("/",B22,9)-FIND(":",B22,4)-7))&amp;"/"</f>
-        <v/>
-      </c>
-      <c r="E22" s="33" t="n"/>
-      <c r="F22" s="34" t="n"/>
-      <c r="G22" s="35" t="n"/>
-      <c r="H22" s="36" t="n"/>
-      <c r="I22" s="37" t="n"/>
-      <c r="J22" s="38" t="n"/>
-      <c r="K22" s="131" t="n"/>
-      <c r="L22" s="40" t="n"/>
-      <c r="M22" s="41" t="n"/>
-      <c r="N22" s="42" t="n">
-        <v>698</v>
-      </c>
-      <c r="O22" s="255" t="n">
-        <v>6957</v>
-      </c>
-      <c r="P22" s="44" t="n"/>
-      <c r="Q22" s="311" t="n"/>
-      <c r="R22" s="46">
-        <f>IFERROR(N22/O22,"")</f>
-        <v/>
-      </c>
-      <c r="S22" s="46">
-        <f>IFERROR(P22/Q22,"")</f>
-        <v/>
-      </c>
-      <c r="T22" s="47" t="n"/>
-      <c r="U22" s="48" t="n"/>
-      <c r="V22" s="49">
-        <f>IFERROR(U22/T22,"")</f>
-        <v/>
-      </c>
-      <c r="W22" s="50" t="n"/>
-      <c r="X22" s="262" t="inlineStr">
-        <is>
-          <t>Слабый конкурент</t>
-        </is>
-      </c>
+      <c r="B22" s="340" t="inlineStr">
+        <is>
+          <t>Медиана (по лидерам)</t>
+        </is>
+      </c>
+      <c r="C22" s="340" t="n"/>
+      <c r="D22" s="340" t="n"/>
+      <c r="E22" s="336">
+        <f>IFERROR(MEDIAN(E2:E21),"")</f>
+        <v/>
+      </c>
+      <c r="F22" s="337">
+        <f>IFERROR(MEDIAN(F2:F21),"")</f>
+        <v/>
+      </c>
+      <c r="G22" s="337">
+        <f>IFERROR(MEDIAN(G2:G21),"")</f>
+        <v/>
+      </c>
+      <c r="H22" s="337">
+        <f>IFERROR(MEDIAN(H2:H21),"")</f>
+        <v/>
+      </c>
+      <c r="I22" s="338">
+        <f>IFERROR(MEDIAN(I2:I21),"")</f>
+        <v/>
+      </c>
+      <c r="J22" s="337">
+        <f>IFERROR(MEDIAN(J2:J21),"")</f>
+        <v/>
+      </c>
+      <c r="K22" s="339" t="n"/>
+      <c r="L22" s="337">
+        <f>IFERROR(MEDIAN(L2:L21),"")</f>
+        <v/>
+      </c>
+      <c r="M22" s="340" t="n"/>
+      <c r="N22" s="337">
+        <f t="array" ref="N22">MEDIAN(IF(X2:X21=" Лидер",N2:N21))</f>
+        <v/>
+      </c>
+      <c r="O22" s="337">
+        <f t="array" ref="O22">MEDIAN(IF(X2:X21=" Лидер",O2:O21))</f>
+        <v/>
+      </c>
+      <c r="P22" s="337">
+        <f>IFERROR(MEDIAN(P2:P21),"")</f>
+        <v/>
+      </c>
+      <c r="Q22" s="337">
+        <f>IFERROR(MEDIAN(Q2:Q21),"")</f>
+        <v/>
+      </c>
+      <c r="R22" s="341">
+        <f>N22/O22</f>
+        <v/>
+      </c>
+      <c r="S22" s="341">
+        <f>IFERROR(MEDIAN(S2:S21),"")</f>
+        <v/>
+      </c>
+      <c r="T22" s="336">
+        <f>IFERROR(MEDIAN(T2:T21),"")</f>
+        <v/>
+      </c>
+      <c r="U22" s="337">
+        <f>IFERROR(MEDIAN(U2:U21),"")</f>
+        <v/>
+      </c>
+      <c r="V22" s="337">
+        <f>IFERROR(MEDIAN(V2:V21),"")</f>
+        <v/>
+      </c>
+      <c r="W22" s="338">
+        <f>IFERROR(MEDIAN(W2:W21),"")</f>
+        <v/>
+      </c>
+      <c r="X22" s="340" t="n"/>
     </row>
     <row r="23">
       <c r="A23" s="26">
@@ -4349,34 +4369,30 @@
       </c>
       <c r="B23" s="28" t="inlineStr">
         <is>
-          <t>https://medfregat.ru/</t>
-        </is>
-      </c>
-      <c r="C23" s="31">
+          <t>https://reiginmed.ru/</t>
+        </is>
+      </c>
+      <c r="C23" s="342">
         <f>"https://www.google.com/s2/favicons?domain="&amp;B23</f>
         <v/>
       </c>
-      <c r="D23" s="31">
+      <c r="D23" s="342">
         <f>"https://a.pr-cy.ru/"&amp;IF(ISERROR(FIND("//www.",B23)),MID(B23,FIND(":",B23,4)+3,FIND("/",B23,9)-FIND(":",B23,4)-3),MID(B23,FIND(":",B23,4)+7,FIND("/",B23,9)-FIND(":",B23,4)-7))&amp;"/"</f>
         <v/>
       </c>
-      <c r="E23" s="33" t="n"/>
-      <c r="F23" s="34" t="n"/>
-      <c r="G23" s="35" t="n"/>
-      <c r="H23" s="36" t="n"/>
-      <c r="I23" s="37" t="n"/>
-      <c r="J23" s="38" t="n"/>
+      <c r="E23" s="343" t="n"/>
+      <c r="F23" s="344" t="n"/>
+      <c r="G23" s="345" t="n"/>
+      <c r="H23" s="344" t="n"/>
+      <c r="I23" s="346" t="n"/>
+      <c r="J23" s="348" t="n"/>
       <c r="K23" s="131" t="n"/>
-      <c r="L23" s="40" t="n"/>
-      <c r="M23" s="41" t="n"/>
-      <c r="N23" s="42" t="n">
-        <v>675</v>
-      </c>
-      <c r="O23" s="255" t="n">
-        <v>13742</v>
-      </c>
-      <c r="P23" s="44" t="n"/>
-      <c r="Q23" s="311" t="n"/>
+      <c r="L23" s="348" t="n"/>
+      <c r="M23" s="131" t="n"/>
+      <c r="N23" s="348" t="n"/>
+      <c r="O23" s="348" t="n"/>
+      <c r="P23" s="348" t="n"/>
+      <c r="Q23" s="348" t="n"/>
       <c r="R23" s="46">
         <f>IFERROR(N23/O23,"")</f>
         <v/>
@@ -4385,1213 +4401,21 @@
         <f>IFERROR(P23/Q23,"")</f>
         <v/>
       </c>
-      <c r="T23" s="47" t="n"/>
-      <c r="U23" s="48" t="n"/>
-      <c r="V23" s="49">
+      <c r="T23" s="349" t="n"/>
+      <c r="U23" s="350" t="n"/>
+      <c r="V23" s="351">
         <f>IFERROR(U23/T23,"")</f>
         <v/>
       </c>
-      <c r="W23" s="50" t="n"/>
-      <c r="X23" s="262" t="inlineStr">
-        <is>
-          <t>Слабый конкурент</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="26">
-        <f>IMAGE(C24)</f>
-        <v/>
-      </c>
-      <c r="B24" s="28" t="inlineStr">
-        <is>
-          <t>https://medicray.ru/</t>
-        </is>
-      </c>
-      <c r="C24" s="31">
-        <f>"https://www.google.com/s2/favicons?domain="&amp;B24</f>
-        <v/>
-      </c>
-      <c r="D24" s="31">
-        <f>"https://a.pr-cy.ru/"&amp;IF(ISERROR(FIND("//www.",B24)),MID(B24,FIND(":",B24,4)+3,FIND("/",B24,9)-FIND(":",B24,4)-3),MID(B24,FIND(":",B24,4)+7,FIND("/",B24,9)-FIND(":",B24,4)-7))&amp;"/"</f>
-        <v/>
-      </c>
-      <c r="E24" s="33" t="n"/>
-      <c r="F24" s="34" t="n"/>
-      <c r="G24" s="35" t="n"/>
-      <c r="H24" s="36" t="n"/>
-      <c r="I24" s="37" t="n"/>
-      <c r="J24" s="38" t="n"/>
-      <c r="K24" s="131" t="n"/>
-      <c r="L24" s="40" t="n"/>
-      <c r="M24" s="41" t="n"/>
-      <c r="N24" s="42" t="n">
-        <v>500</v>
-      </c>
-      <c r="O24" s="255" t="n">
-        <v>3144</v>
-      </c>
-      <c r="P24" s="44" t="n"/>
-      <c r="Q24" s="311" t="n"/>
-      <c r="R24" s="46">
-        <f>IFERROR(N24/O24,"")</f>
-        <v/>
-      </c>
-      <c r="S24" s="46">
-        <f>IFERROR(P24/Q24,"")</f>
-        <v/>
-      </c>
-      <c r="T24" s="47" t="n"/>
-      <c r="U24" s="48" t="n"/>
-      <c r="V24" s="49">
-        <f>IFERROR(U24/T24,"")</f>
-        <v/>
-      </c>
-      <c r="W24" s="50" t="n"/>
-      <c r="X24" s="262" t="inlineStr">
-        <is>
-          <t>Слабый конкурент</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" s="26">
-        <f>IMAGE(C25)</f>
-        <v/>
-      </c>
-      <c r="B25" s="28" t="inlineStr">
-        <is>
-          <t>https://vilmed.ru/</t>
-        </is>
-      </c>
-      <c r="C25" s="31">
-        <f>"https://www.google.com/s2/favicons?domain="&amp;B25</f>
-        <v/>
-      </c>
-      <c r="D25" s="31">
-        <f>"https://a.pr-cy.ru/"&amp;IF(ISERROR(FIND("//www.",B25)),MID(B25,FIND(":",B25,4)+3,FIND("/",B25,9)-FIND(":",B25,4)-3),MID(B25,FIND(":",B25,4)+7,FIND("/",B25,9)-FIND(":",B25,4)-7))&amp;"/"</f>
-        <v/>
-      </c>
-      <c r="E25" s="33" t="n"/>
-      <c r="F25" s="34" t="n"/>
-      <c r="G25" s="35" t="n"/>
-      <c r="H25" s="36" t="n"/>
-      <c r="I25" s="37" t="n"/>
-      <c r="J25" s="38" t="n"/>
-      <c r="K25" s="131" t="n"/>
-      <c r="L25" s="40" t="n"/>
-      <c r="M25" s="41" t="n"/>
-      <c r="N25" s="42" t="n">
-        <v>477</v>
-      </c>
-      <c r="O25" s="255" t="n">
-        <v>35763</v>
-      </c>
-      <c r="P25" s="44" t="n"/>
-      <c r="Q25" s="311" t="n"/>
-      <c r="R25" s="46">
-        <f>IFERROR(N25/O25,"")</f>
-        <v/>
-      </c>
-      <c r="S25" s="46">
-        <f>IFERROR(P25/Q25,"")</f>
-        <v/>
-      </c>
-      <c r="T25" s="47" t="n"/>
-      <c r="U25" s="48" t="n"/>
-      <c r="V25" s="49">
-        <f>IFERROR(U25/T25,"")</f>
-        <v/>
-      </c>
-      <c r="W25" s="50" t="n"/>
-      <c r="X25" s="262" t="inlineStr">
-        <is>
-          <t>Слабый конкурент</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" s="26">
-        <f>IMAGE(C26)</f>
-        <v/>
-      </c>
-      <c r="B26" s="28" t="inlineStr">
-        <is>
-          <t>https://teh-med.ru/</t>
-        </is>
-      </c>
-      <c r="C26" s="31">
-        <f>"https://www.google.com/s2/favicons?domain="&amp;B26</f>
-        <v/>
-      </c>
-      <c r="D26" s="31">
-        <f>"https://a.pr-cy.ru/"&amp;IF(ISERROR(FIND("//www.",B26)),MID(B26,FIND(":",B26,4)+3,FIND("/",B26,9)-FIND(":",B26,4)-3),MID(B26,FIND(":",B26,4)+7,FIND("/",B26,9)-FIND(":",B26,4)-7))&amp;"/"</f>
-        <v/>
-      </c>
-      <c r="E26" s="33" t="n"/>
-      <c r="F26" s="34" t="n"/>
-      <c r="G26" s="35" t="n"/>
-      <c r="H26" s="36" t="n"/>
-      <c r="I26" s="37" t="n"/>
-      <c r="J26" s="38" t="n"/>
-      <c r="K26" s="131" t="n"/>
-      <c r="L26" s="40" t="n"/>
-      <c r="M26" s="41" t="n"/>
-      <c r="N26" s="42" t="n">
-        <v>467</v>
-      </c>
-      <c r="O26" s="255" t="n">
-        <v>6946</v>
-      </c>
-      <c r="P26" s="44" t="n"/>
-      <c r="Q26" s="311" t="n"/>
-      <c r="R26" s="46">
-        <f>IFERROR(N26/O26,"")</f>
-        <v/>
-      </c>
-      <c r="S26" s="46">
-        <f>IFERROR(P26/Q26,"")</f>
-        <v/>
-      </c>
-      <c r="T26" s="47" t="n"/>
-      <c r="U26" s="48" t="n"/>
-      <c r="V26" s="49">
-        <f>IFERROR(U26/T26,"")</f>
-        <v/>
-      </c>
-      <c r="W26" s="50" t="n"/>
-      <c r="X26" s="262" t="inlineStr">
-        <is>
-          <t>Слабый конкурент</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" s="26">
-        <f>IMAGE(C27)</f>
-        <v/>
-      </c>
-      <c r="B27" s="28" t="inlineStr">
-        <is>
-          <t>https://mil-nn.ru/</t>
-        </is>
-      </c>
-      <c r="C27" s="31">
-        <f>"https://www.google.com/s2/favicons?domain="&amp;B27</f>
-        <v/>
-      </c>
-      <c r="D27" s="31">
-        <f>"https://a.pr-cy.ru/"&amp;IF(ISERROR(FIND("//www.",B27)),MID(B27,FIND(":",B27,4)+3,FIND("/",B27,9)-FIND(":",B27,4)-3),MID(B27,FIND(":",B27,4)+7,FIND("/",B27,9)-FIND(":",B27,4)-7))&amp;"/"</f>
-        <v/>
-      </c>
-      <c r="E27" s="33" t="n"/>
-      <c r="F27" s="34" t="n"/>
-      <c r="G27" s="35" t="n"/>
-      <c r="H27" s="36" t="n"/>
-      <c r="I27" s="37" t="n"/>
-      <c r="J27" s="38" t="n"/>
-      <c r="K27" s="131" t="n"/>
-      <c r="L27" s="40" t="n"/>
-      <c r="M27" s="41" t="n"/>
-      <c r="N27" s="42" t="n">
-        <v>452</v>
-      </c>
-      <c r="O27" s="255" t="n">
-        <v>5620</v>
-      </c>
-      <c r="P27" s="44" t="n"/>
-      <c r="Q27" s="311" t="n"/>
-      <c r="R27" s="46">
-        <f>IFERROR(N27/O27,"")</f>
-        <v/>
-      </c>
-      <c r="S27" s="46">
-        <f>IFERROR(P27/Q27,"")</f>
-        <v/>
-      </c>
-      <c r="T27" s="47" t="n"/>
-      <c r="U27" s="48" t="n"/>
-      <c r="V27" s="49">
-        <f>IFERROR(U27/T27,"")</f>
-        <v/>
-      </c>
-      <c r="W27" s="50" t="n"/>
-      <c r="X27" s="262" t="inlineStr">
-        <is>
-          <t>Слабый конкурент</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" s="26">
-        <f>IMAGE(C28)</f>
-        <v/>
-      </c>
-      <c r="B28" s="28" t="inlineStr">
-        <is>
-          <t>https://medakt.ru/</t>
-        </is>
-      </c>
-      <c r="C28" s="31">
-        <f>"https://www.google.com/s2/favicons?domain="&amp;B28</f>
-        <v/>
-      </c>
-      <c r="D28" s="31">
-        <f>"https://a.pr-cy.ru/"&amp;IF(ISERROR(FIND("//www.",B28)),MID(B28,FIND(":",B28,4)+3,FIND("/",B28,9)-FIND(":",B28,4)-3),MID(B28,FIND(":",B28,4)+7,FIND("/",B28,9)-FIND(":",B28,4)-7))&amp;"/"</f>
-        <v/>
-      </c>
-      <c r="E28" s="33" t="n"/>
-      <c r="F28" s="34" t="n"/>
-      <c r="G28" s="35" t="n"/>
-      <c r="H28" s="36" t="n"/>
-      <c r="I28" s="37" t="n"/>
-      <c r="J28" s="38" t="n"/>
-      <c r="K28" s="131" t="n"/>
-      <c r="L28" s="40" t="n"/>
-      <c r="M28" s="41" t="n"/>
-      <c r="N28" s="42" t="n">
-        <v>424</v>
-      </c>
-      <c r="O28" s="255" t="n">
-        <v>4993</v>
-      </c>
-      <c r="P28" s="44" t="n"/>
-      <c r="Q28" s="311" t="n"/>
-      <c r="R28" s="46">
-        <f>IFERROR(N28/O28,"")</f>
-        <v/>
-      </c>
-      <c r="S28" s="46">
-        <f>IFERROR(P28/Q28,"")</f>
-        <v/>
-      </c>
-      <c r="T28" s="47" t="n"/>
-      <c r="U28" s="48" t="n"/>
-      <c r="V28" s="49">
-        <f>IFERROR(U28/T28,"")</f>
-        <v/>
-      </c>
-      <c r="W28" s="50" t="n"/>
-      <c r="X28" s="262" t="inlineStr">
-        <is>
-          <t>Слабый конкурент</t>
-        </is>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" s="26">
-        <f>IMAGE(C29)</f>
-        <v/>
-      </c>
-      <c r="B29" s="28" t="inlineStr">
-        <is>
-          <t>https://salusmed.spb.ru/</t>
-        </is>
-      </c>
-      <c r="C29" s="31">
-        <f>"https://www.google.com/s2/favicons?domain="&amp;B29</f>
-        <v/>
-      </c>
-      <c r="D29" s="31">
-        <f>"https://a.pr-cy.ru/"&amp;IF(ISERROR(FIND("//www.",B29)),MID(B29,FIND(":",B29,4)+3,FIND("/",B29,9)-FIND(":",B29,4)-3),MID(B29,FIND(":",B29,4)+7,FIND("/",B29,9)-FIND(":",B29,4)-7))&amp;"/"</f>
-        <v/>
-      </c>
-      <c r="E29" s="33" t="n"/>
-      <c r="F29" s="34" t="n"/>
-      <c r="G29" s="35" t="n"/>
-      <c r="H29" s="36" t="n"/>
-      <c r="I29" s="37" t="n"/>
-      <c r="J29" s="38" t="n"/>
-      <c r="K29" s="131" t="n"/>
-      <c r="L29" s="40" t="n"/>
-      <c r="M29" s="41" t="n"/>
-      <c r="N29" s="42" t="n">
-        <v>404</v>
-      </c>
-      <c r="O29" s="255" t="n">
-        <v>15980</v>
-      </c>
-      <c r="P29" s="44" t="n"/>
-      <c r="Q29" s="311" t="n"/>
-      <c r="R29" s="46">
-        <f>IFERROR(N29/O29,"")</f>
-        <v/>
-      </c>
-      <c r="S29" s="46">
-        <f>IFERROR(P29/Q29,"")</f>
-        <v/>
-      </c>
-      <c r="T29" s="47" t="n"/>
-      <c r="U29" s="48" t="n"/>
-      <c r="V29" s="49">
-        <f>IFERROR(U29/T29,"")</f>
-        <v/>
-      </c>
-      <c r="W29" s="50" t="n"/>
-      <c r="X29" s="262" t="inlineStr">
-        <is>
-          <t>Слабый конкурент</t>
-        </is>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" s="26">
-        <f>IMAGE(C30)</f>
-        <v/>
-      </c>
-      <c r="B30" s="28" t="inlineStr">
-        <is>
-          <t>https://gm-med.ru/</t>
-        </is>
-      </c>
-      <c r="C30" s="31">
-        <f>"https://www.google.com/s2/favicons?domain="&amp;B30</f>
-        <v/>
-      </c>
-      <c r="D30" s="31">
-        <f>"https://a.pr-cy.ru/"&amp;IF(ISERROR(FIND("//www.",B30)),MID(B30,FIND(":",B30,4)+3,FIND("/",B30,9)-FIND(":",B30,4)-3),MID(B30,FIND(":",B30,4)+7,FIND("/",B30,9)-FIND(":",B30,4)-7))&amp;"/"</f>
-        <v/>
-      </c>
-      <c r="E30" s="33" t="n"/>
-      <c r="F30" s="34" t="n"/>
-      <c r="G30" s="35" t="n"/>
-      <c r="H30" s="36" t="n"/>
-      <c r="I30" s="37" t="n"/>
-      <c r="J30" s="38" t="n"/>
-      <c r="K30" s="131" t="n"/>
-      <c r="L30" s="40" t="n"/>
-      <c r="M30" s="41" t="n"/>
-      <c r="N30" s="42" t="n">
-        <v>259</v>
-      </c>
-      <c r="O30" s="255" t="n">
-        <v>6245</v>
-      </c>
-      <c r="P30" s="44" t="n"/>
-      <c r="Q30" s="311" t="n"/>
-      <c r="R30" s="46">
-        <f>IFERROR(N30/O30,"")</f>
-        <v/>
-      </c>
-      <c r="S30" s="46">
-        <f>IFERROR(P30/Q30,"")</f>
-        <v/>
-      </c>
-      <c r="T30" s="47" t="n"/>
-      <c r="U30" s="48" t="n"/>
-      <c r="V30" s="49">
-        <f>IFERROR(U30/T30,"")</f>
-        <v/>
-      </c>
-      <c r="W30" s="50" t="n"/>
-      <c r="X30" s="262" t="inlineStr">
-        <is>
-          <t>Слабый конкурент</t>
-        </is>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" s="26">
-        <f>IMAGE(C31)</f>
-        <v/>
-      </c>
-      <c r="B31" s="28" t="inlineStr">
-        <is>
-          <t>https://medmetr.ru/</t>
-        </is>
-      </c>
-      <c r="C31" s="31">
-        <f>"https://www.google.com/s2/favicons?domain="&amp;B31</f>
-        <v/>
-      </c>
-      <c r="D31" s="31">
-        <f>"https://a.pr-cy.ru/"&amp;IF(ISERROR(FIND("//www.",B31)),MID(B31,FIND(":",B31,4)+3,FIND("/",B31,9)-FIND(":",B31,4)-3),MID(B31,FIND(":",B31,4)+7,FIND("/",B31,9)-FIND(":",B31,4)-7))&amp;"/"</f>
-        <v/>
-      </c>
-      <c r="E31" s="33" t="n"/>
-      <c r="F31" s="34" t="n"/>
-      <c r="G31" s="35" t="n"/>
-      <c r="H31" s="36" t="n"/>
-      <c r="I31" s="37" t="n"/>
-      <c r="J31" s="38" t="n"/>
-      <c r="K31" s="131" t="n"/>
-      <c r="L31" s="40" t="n"/>
-      <c r="M31" s="41" t="n"/>
-      <c r="N31" s="42" t="n">
-        <v>255</v>
-      </c>
-      <c r="O31" s="255" t="n">
-        <v>5485</v>
-      </c>
-      <c r="P31" s="44" t="n"/>
-      <c r="Q31" s="311" t="n"/>
-      <c r="R31" s="46">
-        <f>IFERROR(N31/O31,"")</f>
-        <v/>
-      </c>
-      <c r="S31" s="46">
-        <f>IFERROR(P31/Q31,"")</f>
-        <v/>
-      </c>
-      <c r="T31" s="47" t="n"/>
-      <c r="U31" s="48" t="n"/>
-      <c r="V31" s="49">
-        <f>IFERROR(U31/T31,"")</f>
-        <v/>
-      </c>
-      <c r="W31" s="50" t="n"/>
-      <c r="X31" s="262" t="inlineStr">
-        <is>
-          <t>Слабый конкурент</t>
-        </is>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" s="26">
-        <f>IMAGE(C32)</f>
-        <v/>
-      </c>
-      <c r="B32" s="28" t="inlineStr">
-        <is>
-          <t>https://gnkmed.ru/</t>
-        </is>
-      </c>
-      <c r="C32" s="31">
-        <f>"https://www.google.com/s2/favicons?domain="&amp;B32</f>
-        <v/>
-      </c>
-      <c r="D32" s="31">
-        <f>"https://a.pr-cy.ru/"&amp;IF(ISERROR(FIND("//www.",B32)),MID(B32,FIND(":",B32,4)+3,FIND("/",B32,9)-FIND(":",B32,4)-3),MID(B32,FIND(":",B32,4)+7,FIND("/",B32,9)-FIND(":",B32,4)-7))&amp;"/"</f>
-        <v/>
-      </c>
-      <c r="E32" s="33" t="n"/>
-      <c r="F32" s="34" t="n"/>
-      <c r="G32" s="35" t="n"/>
-      <c r="H32" s="36" t="n"/>
-      <c r="I32" s="37" t="n"/>
-      <c r="J32" s="38" t="n"/>
-      <c r="K32" s="131" t="n"/>
-      <c r="L32" s="40" t="n"/>
-      <c r="M32" s="41" t="n"/>
-      <c r="N32" s="42" t="n">
-        <v>229</v>
-      </c>
-      <c r="O32" s="255" t="n">
-        <v>1818</v>
-      </c>
-      <c r="P32" s="44" t="n"/>
-      <c r="Q32" s="311" t="n"/>
-      <c r="R32" s="46">
-        <f>IFERROR(N32/O32,"")</f>
-        <v/>
-      </c>
-      <c r="S32" s="46">
-        <f>IFERROR(P32/Q32,"")</f>
-        <v/>
-      </c>
-      <c r="T32" s="47" t="n"/>
-      <c r="U32" s="48" t="n"/>
-      <c r="V32" s="49">
-        <f>IFERROR(U32/T32,"")</f>
-        <v/>
-      </c>
-      <c r="W32" s="50" t="n"/>
-      <c r="X32" s="262" t="inlineStr">
-        <is>
-          <t>Слабый конкурент</t>
-        </is>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" s="26">
-        <f>IMAGE(C33)</f>
-        <v/>
-      </c>
-      <c r="B33" s="28" t="inlineStr">
-        <is>
-          <t>https://dixion.ru/</t>
-        </is>
-      </c>
-      <c r="C33" s="31">
-        <f>"https://www.google.com/s2/favicons?domain="&amp;B33</f>
-        <v/>
-      </c>
-      <c r="D33" s="31">
-        <f>"https://a.pr-cy.ru/"&amp;IF(ISERROR(FIND("//www.",B33)),MID(B33,FIND(":",B33,4)+3,FIND("/",B33,9)-FIND(":",B33,4)-3),MID(B33,FIND(":",B33,4)+7,FIND("/",B33,9)-FIND(":",B33,4)-7))&amp;"/"</f>
-        <v/>
-      </c>
-      <c r="E33" s="33" t="n"/>
-      <c r="F33" s="34" t="n"/>
-      <c r="G33" s="35" t="n"/>
-      <c r="H33" s="36" t="n"/>
-      <c r="I33" s="37" t="n"/>
-      <c r="J33" s="38" t="n"/>
-      <c r="K33" s="131" t="n"/>
-      <c r="L33" s="40" t="n"/>
-      <c r="M33" s="41" t="n"/>
-      <c r="N33" s="42" t="n">
-        <v>229</v>
-      </c>
-      <c r="O33" s="255" t="n">
-        <v>2752</v>
-      </c>
-      <c r="P33" s="44" t="n"/>
-      <c r="Q33" s="311" t="n"/>
-      <c r="R33" s="46">
-        <f>IFERROR(N33/O33,"")</f>
-        <v/>
-      </c>
-      <c r="S33" s="46">
-        <f>IFERROR(P33/Q33,"")</f>
-        <v/>
-      </c>
-      <c r="T33" s="47" t="n"/>
-      <c r="U33" s="48" t="n"/>
-      <c r="V33" s="49">
-        <f>IFERROR(U33/T33,"")</f>
-        <v/>
-      </c>
-      <c r="W33" s="50" t="n"/>
-      <c r="X33" s="262" t="inlineStr">
-        <is>
-          <t>Слабый конкурент</t>
-        </is>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" s="26">
-        <f>IMAGE(C34)</f>
-        <v/>
-      </c>
-      <c r="B34" s="28" t="inlineStr">
-        <is>
-          <t>https://lotem.ru/</t>
-        </is>
-      </c>
-      <c r="C34" s="31">
-        <f>"https://www.google.com/s2/favicons?domain="&amp;B34</f>
-        <v/>
-      </c>
-      <c r="D34" s="31">
-        <f>"https://a.pr-cy.ru/"&amp;IF(ISERROR(FIND("//www.",B34)),MID(B34,FIND(":",B34,4)+3,FIND("/",B34,9)-FIND(":",B34,4)-3),MID(B34,FIND(":",B34,4)+7,FIND("/",B34,9)-FIND(":",B34,4)-7))&amp;"/"</f>
-        <v/>
-      </c>
-      <c r="E34" s="33" t="n"/>
-      <c r="F34" s="34" t="n"/>
-      <c r="G34" s="35" t="n"/>
-      <c r="H34" s="36" t="n"/>
-      <c r="I34" s="37" t="n"/>
-      <c r="J34" s="38" t="n"/>
-      <c r="K34" s="131" t="n"/>
-      <c r="L34" s="40" t="n"/>
-      <c r="M34" s="41" t="n"/>
-      <c r="N34" s="42" t="n">
-        <v>199</v>
-      </c>
-      <c r="O34" s="255" t="n">
-        <v>1783</v>
-      </c>
-      <c r="P34" s="44" t="n"/>
-      <c r="Q34" s="311" t="n"/>
-      <c r="R34" s="46">
-        <f>IFERROR(N34/O34,"")</f>
-        <v/>
-      </c>
-      <c r="S34" s="46">
-        <f>IFERROR(P34/Q34,"")</f>
-        <v/>
-      </c>
-      <c r="T34" s="47" t="n"/>
-      <c r="U34" s="48" t="n"/>
-      <c r="V34" s="49">
-        <f>IFERROR(U34/T34,"")</f>
-        <v/>
-      </c>
-      <c r="W34" s="50" t="n"/>
-      <c r="X34" s="262" t="inlineStr">
-        <is>
-          <t>Слабый конкурент</t>
-        </is>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" s="26">
-        <f>IMAGE(C35)</f>
-        <v/>
-      </c>
-      <c r="B35" s="28" t="inlineStr">
-        <is>
-          <t>https://meditems.ru/</t>
-        </is>
-      </c>
-      <c r="C35" s="31">
-        <f>"https://www.google.com/s2/favicons?domain="&amp;B35</f>
-        <v/>
-      </c>
-      <c r="D35" s="31">
-        <f>"https://a.pr-cy.ru/"&amp;IF(ISERROR(FIND("//www.",B35)),MID(B35,FIND(":",B35,4)+3,FIND("/",B35,9)-FIND(":",B35,4)-3),MID(B35,FIND(":",B35,4)+7,FIND("/",B35,9)-FIND(":",B35,4)-7))&amp;"/"</f>
-        <v/>
-      </c>
-      <c r="E35" s="33" t="n"/>
-      <c r="F35" s="34" t="n"/>
-      <c r="G35" s="35" t="n"/>
-      <c r="H35" s="36" t="n"/>
-      <c r="I35" s="37" t="n"/>
-      <c r="J35" s="38" t="n"/>
-      <c r="K35" s="131" t="n"/>
-      <c r="L35" s="40" t="n"/>
-      <c r="M35" s="41" t="n"/>
-      <c r="N35" s="42" t="n">
-        <v>176</v>
-      </c>
-      <c r="O35" s="255" t="n">
-        <v>9245</v>
-      </c>
-      <c r="P35" s="44" t="n"/>
-      <c r="Q35" s="311" t="n"/>
-      <c r="R35" s="46">
-        <f>IFERROR(N35/O35,"")</f>
-        <v/>
-      </c>
-      <c r="S35" s="46">
-        <f>IFERROR(P35/Q35,"")</f>
-        <v/>
-      </c>
-      <c r="T35" s="47" t="n"/>
-      <c r="U35" s="48" t="n"/>
-      <c r="V35" s="49">
-        <f>IFERROR(U35/T35,"")</f>
-        <v/>
-      </c>
-      <c r="W35" s="50" t="n"/>
-      <c r="X35" s="262" t="inlineStr">
-        <is>
-          <t>Слабый конкурент</t>
-        </is>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" s="26">
-        <f>IMAGE(C36)</f>
-        <v/>
-      </c>
-      <c r="B36" s="28" t="inlineStr">
-        <is>
-          <t>https://fujitora.com/</t>
-        </is>
-      </c>
-      <c r="C36" s="31">
-        <f>"https://www.google.com/s2/favicons?domain="&amp;B36</f>
-        <v/>
-      </c>
-      <c r="D36" s="31">
-        <f>"https://a.pr-cy.ru/"&amp;IF(ISERROR(FIND("//www.",B36)),MID(B36,FIND(":",B36,4)+3,FIND("/",B36,9)-FIND(":",B36,4)-3),MID(B36,FIND(":",B36,4)+7,FIND("/",B36,9)-FIND(":",B36,4)-7))&amp;"/"</f>
-        <v/>
-      </c>
-      <c r="E36" s="33" t="n"/>
-      <c r="F36" s="34" t="n"/>
-      <c r="G36" s="35" t="n"/>
-      <c r="H36" s="36" t="n"/>
-      <c r="I36" s="37" t="n"/>
-      <c r="J36" s="38" t="n"/>
-      <c r="K36" s="131" t="n"/>
-      <c r="L36" s="40" t="n"/>
-      <c r="M36" s="41" t="n"/>
-      <c r="N36" s="42" t="n">
-        <v>148</v>
-      </c>
-      <c r="O36" s="255" t="n">
-        <v>3012</v>
-      </c>
-      <c r="P36" s="44" t="n"/>
-      <c r="Q36" s="311" t="n"/>
-      <c r="R36" s="46">
-        <f>IFERROR(N36/O36,"")</f>
-        <v/>
-      </c>
-      <c r="S36" s="46">
-        <f>IFERROR(P36/Q36,"")</f>
-        <v/>
-      </c>
-      <c r="T36" s="47" t="n"/>
-      <c r="U36" s="48" t="n"/>
-      <c r="V36" s="49">
-        <f>IFERROR(U36/T36,"")</f>
-        <v/>
-      </c>
-      <c r="W36" s="50" t="n"/>
-      <c r="X36" s="262" t="inlineStr">
-        <is>
-          <t>Слабый конкурент</t>
-        </is>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" s="26">
-        <f>IMAGE(C37)</f>
-        <v/>
-      </c>
-      <c r="B37" s="28" t="inlineStr">
-        <is>
-          <t>https://rusmedcompany.ru/</t>
-        </is>
-      </c>
-      <c r="C37" s="31">
-        <f>"https://www.google.com/s2/favicons?domain="&amp;B37</f>
-        <v/>
-      </c>
-      <c r="D37" s="31">
-        <f>"https://a.pr-cy.ru/"&amp;IF(ISERROR(FIND("//www.",B37)),MID(B37,FIND(":",B37,4)+3,FIND("/",B37,9)-FIND(":",B37,4)-3),MID(B37,FIND(":",B37,4)+7,FIND("/",B37,9)-FIND(":",B37,4)-7))&amp;"/"</f>
-        <v/>
-      </c>
-      <c r="E37" s="33" t="n"/>
-      <c r="F37" s="34" t="n"/>
-      <c r="G37" s="35" t="n"/>
-      <c r="H37" s="36" t="n"/>
-      <c r="I37" s="37" t="n"/>
-      <c r="J37" s="38" t="n"/>
-      <c r="K37" s="131" t="n"/>
-      <c r="L37" s="40" t="n"/>
-      <c r="M37" s="41" t="n"/>
-      <c r="N37" s="42" t="n">
-        <v>108</v>
-      </c>
-      <c r="O37" s="255" t="n">
-        <v>7086</v>
-      </c>
-      <c r="P37" s="44" t="n"/>
-      <c r="Q37" s="311" t="n"/>
-      <c r="R37" s="46">
-        <f>IFERROR(N37/O37,"")</f>
-        <v/>
-      </c>
-      <c r="S37" s="46">
-        <f>IFERROR(P37/Q37,"")</f>
-        <v/>
-      </c>
-      <c r="T37" s="47" t="n"/>
-      <c r="U37" s="48" t="n"/>
-      <c r="V37" s="49">
-        <f>IFERROR(U37/T37,"")</f>
-        <v/>
-      </c>
-      <c r="W37" s="50" t="n"/>
-      <c r="X37" s="262" t="inlineStr">
-        <is>
-          <t>Слабый конкурент</t>
-        </is>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" s="26">
-        <f>IMAGE(C38)</f>
-        <v/>
-      </c>
-      <c r="B38" s="28" t="inlineStr">
-        <is>
-          <t>https://gsmedicine.ru/</t>
-        </is>
-      </c>
-      <c r="C38" s="31">
-        <f>"https://www.google.com/s2/favicons?domain="&amp;B38</f>
-        <v/>
-      </c>
-      <c r="D38" s="31">
-        <f>"https://a.pr-cy.ru/"&amp;IF(ISERROR(FIND("//www.",B38)),MID(B38,FIND(":",B38,4)+3,FIND("/",B38,9)-FIND(":",B38,4)-3),MID(B38,FIND(":",B38,4)+7,FIND("/",B38,9)-FIND(":",B38,4)-7))&amp;"/"</f>
-        <v/>
-      </c>
-      <c r="E38" s="33" t="n"/>
-      <c r="F38" s="34" t="n"/>
-      <c r="G38" s="35" t="n"/>
-      <c r="H38" s="36" t="n"/>
-      <c r="I38" s="37" t="n"/>
-      <c r="J38" s="38" t="n"/>
-      <c r="K38" s="131" t="n"/>
-      <c r="L38" s="40" t="n"/>
-      <c r="M38" s="41" t="n"/>
-      <c r="N38" s="42" t="n">
-        <v>33</v>
-      </c>
-      <c r="O38" s="255" t="n">
-        <v>722</v>
-      </c>
-      <c r="P38" s="44" t="n"/>
-      <c r="Q38" s="311" t="n"/>
-      <c r="R38" s="46">
-        <f>IFERROR(N38/O38,"")</f>
-        <v/>
-      </c>
-      <c r="S38" s="46">
-        <f>IFERROR(P38/Q38,"")</f>
-        <v/>
-      </c>
-      <c r="T38" s="47" t="n"/>
-      <c r="U38" s="48" t="n"/>
-      <c r="V38" s="49">
-        <f>IFERROR(U38/T38,"")</f>
-        <v/>
-      </c>
-      <c r="W38" s="50" t="n"/>
-      <c r="X38" s="262" t="inlineStr">
-        <is>
-          <t>Слабый конкурент</t>
-        </is>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" s="26">
-        <f>IMAGE(C39)</f>
-        <v/>
-      </c>
-      <c r="B39" s="28" t="inlineStr">
-        <is>
-          <t>https://eurotech.ru/</t>
-        </is>
-      </c>
-      <c r="C39" s="31">
-        <f>"https://www.google.com/s2/favicons?domain="&amp;B39</f>
-        <v/>
-      </c>
-      <c r="D39" s="31">
-        <f>"https://a.pr-cy.ru/"&amp;IF(ISERROR(FIND("//www.",B39)),MID(B39,FIND(":",B39,4)+3,FIND("/",B39,9)-FIND(":",B39,4)-3),MID(B39,FIND(":",B39,4)+7,FIND("/",B39,9)-FIND(":",B39,4)-7))&amp;"/"</f>
-        <v/>
-      </c>
-      <c r="E39" s="33" t="n"/>
-      <c r="F39" s="34" t="n"/>
-      <c r="G39" s="35" t="n"/>
-      <c r="H39" s="36" t="n"/>
-      <c r="I39" s="37" t="n"/>
-      <c r="J39" s="38" t="n"/>
-      <c r="K39" s="131" t="n"/>
-      <c r="L39" s="40" t="n"/>
-      <c r="M39" s="41" t="n"/>
-      <c r="N39" s="42" t="n">
-        <v>17</v>
-      </c>
-      <c r="O39" s="255" t="n">
-        <v>216</v>
-      </c>
-      <c r="P39" s="44" t="n"/>
-      <c r="Q39" s="311" t="n"/>
-      <c r="R39" s="46">
-        <f>IFERROR(N39/O39,"")</f>
-        <v/>
-      </c>
-      <c r="S39" s="46">
-        <f>IFERROR(P39/Q39,"")</f>
-        <v/>
-      </c>
-      <c r="T39" s="47" t="n"/>
-      <c r="U39" s="48" t="n"/>
-      <c r="V39" s="49">
-        <f>IFERROR(U39/T39,"")</f>
-        <v/>
-      </c>
-      <c r="W39" s="50" t="n"/>
-      <c r="X39" s="262" t="inlineStr">
-        <is>
-          <t>Слабый конкурент</t>
-        </is>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" s="26">
-        <f>IMAGE(C40)</f>
-        <v/>
-      </c>
-      <c r="B40" s="28" t="inlineStr">
-        <is>
-          <t>https://ro-med.ru/</t>
-        </is>
-      </c>
-      <c r="C40" s="31">
-        <f>"https://www.google.com/s2/favicons?domain="&amp;B40</f>
-        <v/>
-      </c>
-      <c r="D40" s="31">
-        <f>"https://a.pr-cy.ru/"&amp;IF(ISERROR(FIND("//www.",B40)),MID(B40,FIND(":",B40,4)+3,FIND("/",B40,9)-FIND(":",B40,4)-3),MID(B40,FIND(":",B40,4)+7,FIND("/",B40,9)-FIND(":",B40,4)-7))&amp;"/"</f>
-        <v/>
-      </c>
-      <c r="E40" s="33" t="n"/>
-      <c r="F40" s="34" t="n"/>
-      <c r="G40" s="35" t="n"/>
-      <c r="H40" s="36" t="n"/>
-      <c r="I40" s="37" t="n"/>
-      <c r="J40" s="38" t="n"/>
-      <c r="K40" s="131" t="n"/>
-      <c r="L40" s="40" t="n"/>
-      <c r="M40" s="41" t="n"/>
-      <c r="N40" s="42" t="n">
-        <v>2</v>
-      </c>
-      <c r="O40" s="255" t="n">
-        <v>324</v>
-      </c>
-      <c r="P40" s="44" t="n"/>
-      <c r="Q40" s="311" t="n"/>
-      <c r="R40" s="46">
-        <f>IFERROR(N40/O40,"")</f>
-        <v/>
-      </c>
-      <c r="S40" s="46">
-        <f>IFERROR(P40/Q40,"")</f>
-        <v/>
-      </c>
-      <c r="T40" s="47" t="n"/>
-      <c r="U40" s="48" t="n"/>
-      <c r="V40" s="49">
-        <f>IFERROR(U40/T40,"")</f>
-        <v/>
-      </c>
-      <c r="W40" s="50" t="n"/>
-      <c r="X40" s="262" t="inlineStr">
-        <is>
-          <t>Слабый конкурент</t>
-        </is>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" s="26">
-        <f>IMAGE(C41)</f>
-        <v/>
-      </c>
-      <c r="B41" s="28" t="inlineStr">
-        <is>
-          <t>https://intelmed.ru/</t>
-        </is>
-      </c>
-      <c r="C41" s="31">
-        <f>"https://www.google.com/s2/favicons?domain="&amp;B41</f>
-        <v/>
-      </c>
-      <c r="D41" s="31">
-        <f>"https://a.pr-cy.ru/"&amp;IF(ISERROR(FIND("//www.",B41)),MID(B41,FIND(":",B41,4)+3,FIND("/",B41,9)-FIND(":",B41,4)-3),MID(B41,FIND(":",B41,4)+7,FIND("/",B41,9)-FIND(":",B41,4)-7))&amp;"/"</f>
-        <v/>
-      </c>
-      <c r="E41" s="33" t="n"/>
-      <c r="F41" s="34" t="n"/>
-      <c r="G41" s="35" t="n"/>
-      <c r="H41" s="36" t="n"/>
-      <c r="I41" s="37" t="n"/>
-      <c r="J41" s="38" t="n"/>
-      <c r="K41" s="131" t="n"/>
-      <c r="L41" s="40" t="n"/>
-      <c r="M41" s="41" t="n"/>
-      <c r="N41" s="42" t="n"/>
-      <c r="O41" s="255" t="n"/>
-      <c r="P41" s="44" t="n"/>
-      <c r="Q41" s="311" t="n"/>
-      <c r="R41" s="46">
-        <f>IFERROR(N41/O41,"")</f>
-        <v/>
-      </c>
-      <c r="S41" s="46">
-        <f>IFERROR(P41/Q41,"")</f>
-        <v/>
-      </c>
-      <c r="T41" s="47" t="n"/>
-      <c r="U41" s="48" t="n"/>
-      <c r="V41" s="49">
-        <f>IFERROR(U41/T41,"")</f>
-        <v/>
-      </c>
-      <c r="W41" s="50" t="n"/>
-      <c r="X41" s="262" t="inlineStr">
-        <is>
-          <t>Более широкий конкурент</t>
-        </is>
-      </c>
-    </row>
-    <row r="42">
-      <c r="A42" s="26">
-        <f>IMAGE(C42)</f>
-        <v/>
-      </c>
-      <c r="B42" s="28" t="inlineStr">
-        <is>
-          <t>https://kriptomed.ru/</t>
-        </is>
-      </c>
-      <c r="C42" s="31">
-        <f>"https://www.google.com/s2/favicons?domain="&amp;B42</f>
-        <v/>
-      </c>
-      <c r="D42" s="31">
-        <f>"https://a.pr-cy.ru/"&amp;IF(ISERROR(FIND("//www.",B42)),MID(B42,FIND(":",B42,4)+3,FIND("/",B42,9)-FIND(":",B42,4)-3),MID(B42,FIND(":",B42,4)+7,FIND("/",B42,9)-FIND(":",B42,4)-7))&amp;"/"</f>
-        <v/>
-      </c>
-      <c r="E42" s="33" t="n"/>
-      <c r="F42" s="34" t="n"/>
-      <c r="G42" s="35" t="n"/>
-      <c r="H42" s="36" t="n"/>
-      <c r="I42" s="37" t="n"/>
-      <c r="J42" s="38" t="n"/>
-      <c r="K42" s="131" t="n"/>
-      <c r="L42" s="40" t="n"/>
-      <c r="M42" s="41" t="n"/>
-      <c r="N42" s="42" t="n"/>
-      <c r="O42" s="255" t="n"/>
-      <c r="P42" s="44" t="n"/>
-      <c r="Q42" s="311" t="n"/>
-      <c r="R42" s="46">
-        <f>IFERROR(N42/O42,"")</f>
-        <v/>
-      </c>
-      <c r="S42" s="46">
-        <f>IFERROR(P42/Q42,"")</f>
-        <v/>
-      </c>
-      <c r="T42" s="47" t="n"/>
-      <c r="U42" s="48" t="n"/>
-      <c r="V42" s="49">
-        <f>IFERROR(U42/T42,"")</f>
-        <v/>
-      </c>
-      <c r="W42" s="50" t="n"/>
-      <c r="X42" s="262" t="inlineStr">
-        <is>
-          <t>Более широкий конкурент</t>
-        </is>
-      </c>
-    </row>
-    <row r="43">
-      <c r="A43" s="26">
-        <f>IMAGE(C43)</f>
-        <v/>
-      </c>
-      <c r="B43" s="340" t="inlineStr">
-        <is>
-          <t>Медиана (по лидерам)</t>
-        </is>
-      </c>
-      <c r="C43" s="340" t="n"/>
-      <c r="D43" s="340" t="n"/>
-      <c r="E43" s="336">
-        <f>IFERROR(MEDIAN(E2:E42),"")</f>
-        <v/>
-      </c>
-      <c r="F43" s="337">
-        <f>IFERROR(MEDIAN(F2:F42),"")</f>
-        <v/>
-      </c>
-      <c r="G43" s="337">
-        <f>IFERROR(MEDIAN(G2:G42),"")</f>
-        <v/>
-      </c>
-      <c r="H43" s="337">
-        <f>IFERROR(MEDIAN(H2:H42),"")</f>
-        <v/>
-      </c>
-      <c r="I43" s="338">
-        <f>IFERROR(MEDIAN(I2:I42),"")</f>
-        <v/>
-      </c>
-      <c r="J43" s="337">
-        <f>IFERROR(MEDIAN(J2:J42),"")</f>
-        <v/>
-      </c>
-      <c r="K43" s="339" t="n"/>
-      <c r="L43" s="337">
-        <f>IFERROR(MEDIAN(L2:L42),"")</f>
-        <v/>
-      </c>
-      <c r="M43" s="340" t="n"/>
-      <c r="N43" s="337">
-        <f t="array" ref="N43">MEDIAN(IF(X2:X42=" Лидер",N2:N42))</f>
-        <v/>
-      </c>
-      <c r="O43" s="337">
-        <f t="array" ref="O43">MEDIAN(IF(X2:X42=" Лидер",O2:O42))</f>
-        <v/>
-      </c>
-      <c r="P43" s="337">
-        <f>IFERROR(MEDIAN(P2:P42),"")</f>
-        <v/>
-      </c>
-      <c r="Q43" s="337">
-        <f>IFERROR(MEDIAN(Q2:Q42),"")</f>
-        <v/>
-      </c>
-      <c r="R43" s="341">
-        <f>N43/O43</f>
-        <v/>
-      </c>
-      <c r="S43" s="341">
-        <f>IFERROR(MEDIAN(S2:S42),"")</f>
-        <v/>
-      </c>
-      <c r="T43" s="336">
-        <f>IFERROR(MEDIAN(T2:T42),"")</f>
-        <v/>
-      </c>
-      <c r="U43" s="337">
-        <f>IFERROR(MEDIAN(U2:U42),"")</f>
-        <v/>
-      </c>
-      <c r="V43" s="337">
-        <f>IFERROR(MEDIAN(V2:V42),"")</f>
-        <v/>
-      </c>
-      <c r="W43" s="338">
-        <f>IFERROR(MEDIAN(W2:W42),"")</f>
-        <v/>
-      </c>
-      <c r="X43" s="340" t="n"/>
-    </row>
-    <row r="44">
-      <c r="A44" s="26">
-        <f>IMAGE(C44)</f>
-        <v/>
-      </c>
-      <c r="B44" s="28" t="inlineStr">
-        <is>
-          <t>https://reiginmed.ru/</t>
-        </is>
-      </c>
-      <c r="C44" s="342">
-        <f>"https://www.google.com/s2/favicons?domain="&amp;B44</f>
-        <v/>
-      </c>
-      <c r="D44" s="342">
-        <f>"https://a.pr-cy.ru/"&amp;IF(ISERROR(FIND("//www.",B44)),MID(B44,FIND(":",B44,4)+3,FIND("/",B44,9)-FIND(":",B44,4)-3),MID(B44,FIND(":",B44,4)+7,FIND("/",B44,9)-FIND(":",B44,4)-7))&amp;"/"</f>
-        <v/>
-      </c>
-      <c r="E44" s="343" t="n"/>
-      <c r="F44" s="344" t="n"/>
-      <c r="G44" s="345" t="n"/>
-      <c r="H44" s="344" t="n"/>
-      <c r="I44" s="346" t="n"/>
-      <c r="J44" s="348" t="n"/>
-      <c r="K44" s="131" t="n"/>
-      <c r="L44" s="348" t="n"/>
-      <c r="M44" s="131" t="n"/>
-      <c r="N44" s="348" t="n"/>
-      <c r="O44" s="348" t="n"/>
-      <c r="P44" s="348" t="n"/>
-      <c r="Q44" s="348" t="n"/>
-      <c r="R44" s="46">
-        <f>IFERROR(N44/O44,"")</f>
-        <v/>
-      </c>
-      <c r="S44" s="46">
-        <f>IFERROR(P44/Q44,"")</f>
-        <v/>
-      </c>
-      <c r="T44" s="349" t="n"/>
-      <c r="U44" s="350" t="n"/>
-      <c r="V44" s="351">
-        <f>IFERROR(U44/T44,"")</f>
-        <v/>
-      </c>
-      <c r="W44" s="352" t="n"/>
-      <c r="X44" s="353" t="inlineStr">
+      <c r="W23" s="352" t="n"/>
+      <c r="X23" s="353" t="inlineStr">
         <is>
           <t>Наш сайт</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:V44"/>
+  <autoFilter ref="A1:V23"/>
   <conditionalFormatting sqref="K2:K31 M2:M31">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
       <formula>"Рост"</formula>
@@ -5853,7 +4677,7 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation sqref="X2:X44" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="X2:X23" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>'Технический лист'!$A$1:$A$5</formula1>
     </dataValidation>
   </dataValidations>
@@ -5870,7 +4694,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I40"/>
+  <dimension ref="A1:I19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" style="354" min="1" max="1"/>
@@ -6522,699 +5346,6 @@
       <c r="I19" t="inlineStr">
         <is>
           <t>https://eurosmed.ru/catalog/ginekologicheskoe_oborudovanie</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" t="inlineStr">
-        <is>
-          <t>vendem.ru</t>
-        </is>
-      </c>
-      <c r="B20" t="n">
-        <v>14</v>
-      </c>
-      <c r="C20" t="n">
-        <v>1</v>
-      </c>
-      <c r="D20" t="n">
-        <v>1</v>
-      </c>
-      <c r="E20" t="n">
-        <v>55</v>
-      </c>
-      <c r="F20" t="n">
-        <v>876</v>
-      </c>
-      <c r="G20" t="n">
-        <v>2689</v>
-      </c>
-      <c r="H20" t="n">
-        <v>13675</v>
-      </c>
-      <c r="I20" t="inlineStr">
-        <is>
-          <t>https://vendem.ru/catalog/akusherstvo_i_ginekologiya</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" t="inlineStr">
-        <is>
-          <t>redsrus.ru</t>
-        </is>
-      </c>
-      <c r="B21" t="n">
-        <v>38</v>
-      </c>
-      <c r="C21" t="n">
-        <v>1</v>
-      </c>
-      <c r="D21" t="n">
-        <v>1</v>
-      </c>
-      <c r="E21" t="n">
-        <v>130</v>
-      </c>
-      <c r="F21" t="n">
-        <v>858</v>
-      </c>
-      <c r="G21" t="n">
-        <v>1959</v>
-      </c>
-      <c r="H21" t="n">
-        <v>8125</v>
-      </c>
-      <c r="I21" t="inlineStr">
-        <is>
-          <t>https://redsrus.ru/product-category/mediczinskoe-osnashhenie/mediczinskoe-oborudovanie/ginekologicheskoe</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" t="inlineStr">
-        <is>
-          <t>lmed.ru</t>
-        </is>
-      </c>
-      <c r="B22" t="n">
-        <v>28</v>
-      </c>
-      <c r="C22" t="n">
-        <v>1</v>
-      </c>
-      <c r="D22" t="n">
-        <v>2</v>
-      </c>
-      <c r="E22" t="n">
-        <v>101</v>
-      </c>
-      <c r="F22" t="n">
-        <v>698</v>
-      </c>
-      <c r="G22" t="n">
-        <v>1369</v>
-      </c>
-      <c r="H22" t="n">
-        <v>6957</v>
-      </c>
-      <c r="I22" t="inlineStr">
-        <is>
-          <t>https://lmed.ru/product-category/akusherstvo-i-ginekologiya</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" t="inlineStr">
-        <is>
-          <t>medfregat.ru</t>
-        </is>
-      </c>
-      <c r="B23" t="n">
-        <v>11</v>
-      </c>
-      <c r="C23" t="n">
-        <v>1</v>
-      </c>
-      <c r="D23" t="n">
-        <v>1</v>
-      </c>
-      <c r="E23" t="n">
-        <v>81</v>
-      </c>
-      <c r="F23" t="n">
-        <v>675</v>
-      </c>
-      <c r="G23" t="n">
-        <v>2046</v>
-      </c>
-      <c r="H23" t="n">
-        <v>13742</v>
-      </c>
-      <c r="I23" t="inlineStr">
-        <is>
-          <t>https://medfregat.ru/catalog/ginekologiya-i-urologiya</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" t="inlineStr">
-        <is>
-          <t>medicray.ru</t>
-        </is>
-      </c>
-      <c r="B24" t="n">
-        <v>19</v>
-      </c>
-      <c r="C24" t="n">
-        <v>1</v>
-      </c>
-      <c r="D24" t="n">
-        <v>0</v>
-      </c>
-      <c r="E24" t="n">
-        <v>29</v>
-      </c>
-      <c r="F24" t="n">
-        <v>500</v>
-      </c>
-      <c r="G24" t="n">
-        <v>1020</v>
-      </c>
-      <c r="H24" t="n">
-        <v>3144</v>
-      </c>
-      <c r="I24" t="inlineStr">
-        <is>
-          <t>https://medicray.ru/category/catalog-oborudovaniya/ginekologia</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" t="inlineStr">
-        <is>
-          <t>vilmed.ru</t>
-        </is>
-      </c>
-      <c r="B25" t="n">
-        <v>29</v>
-      </c>
-      <c r="C25" t="n">
-        <v>1</v>
-      </c>
-      <c r="D25" t="n">
-        <v>1</v>
-      </c>
-      <c r="E25" t="n">
-        <v>22</v>
-      </c>
-      <c r="F25" t="n">
-        <v>477</v>
-      </c>
-      <c r="G25" t="n">
-        <v>2299</v>
-      </c>
-      <c r="H25" t="n">
-        <v>35763</v>
-      </c>
-      <c r="I25" t="inlineStr">
-        <is>
-          <t>https://vilmed.ru/catalog/ginekologiya</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" t="inlineStr">
-        <is>
-          <t>teh-med.ru</t>
-        </is>
-      </c>
-      <c r="B26" t="n">
-        <v>30</v>
-      </c>
-      <c r="C26" t="n">
-        <v>1</v>
-      </c>
-      <c r="D26" t="n">
-        <v>1</v>
-      </c>
-      <c r="E26" t="n">
-        <v>89</v>
-      </c>
-      <c r="F26" t="n">
-        <v>467</v>
-      </c>
-      <c r="G26" t="n">
-        <v>1048</v>
-      </c>
-      <c r="H26" t="n">
-        <v>6946</v>
-      </c>
-      <c r="I26" t="inlineStr">
-        <is>
-          <t>https://teh-med.ru/ginekologiya_akusherstvo</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" t="inlineStr">
-        <is>
-          <t>mil-nn.ru</t>
-        </is>
-      </c>
-      <c r="B27" t="n">
-        <v>21</v>
-      </c>
-      <c r="C27" t="n">
-        <v>1</v>
-      </c>
-      <c r="D27" t="n">
-        <v>0</v>
-      </c>
-      <c r="E27" t="n">
-        <v>50</v>
-      </c>
-      <c r="F27" t="n">
-        <v>452</v>
-      </c>
-      <c r="G27" t="n">
-        <v>1286</v>
-      </c>
-      <c r="H27" t="n">
-        <v>5620</v>
-      </c>
-      <c r="I27" t="inlineStr">
-        <is>
-          <t>https://mil-nn.ru/catalog/ginekologicheskoe_oborudovanie</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" t="inlineStr">
-        <is>
-          <t>medakt.ru</t>
-        </is>
-      </c>
-      <c r="B28" t="n">
-        <v>36</v>
-      </c>
-      <c r="C28" t="n">
-        <v>1</v>
-      </c>
-      <c r="D28" t="n">
-        <v>1</v>
-      </c>
-      <c r="E28" t="n">
-        <v>77</v>
-      </c>
-      <c r="F28" t="n">
-        <v>424</v>
-      </c>
-      <c r="G28" t="n">
-        <v>943</v>
-      </c>
-      <c r="H28" t="n">
-        <v>4993</v>
-      </c>
-      <c r="I28" t="inlineStr">
-        <is>
-          <t>https://medakt.ru/catalog/akusherstvo-i-ginekologiya</t>
-        </is>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" t="inlineStr">
-        <is>
-          <t>salusmed.spb.ru</t>
-        </is>
-      </c>
-      <c r="B29" t="n">
-        <v>35</v>
-      </c>
-      <c r="C29" t="n">
-        <v>1</v>
-      </c>
-      <c r="D29" t="n">
-        <v>0</v>
-      </c>
-      <c r="E29" t="n">
-        <v>45</v>
-      </c>
-      <c r="F29" t="n">
-        <v>404</v>
-      </c>
-      <c r="G29" t="n">
-        <v>1513</v>
-      </c>
-      <c r="H29" t="n">
-        <v>15980</v>
-      </c>
-      <c r="I29" t="inlineStr">
-        <is>
-          <t>https://salusmed.spb.ru/медицинское-гинекологическое-оборудование-0</t>
-        </is>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" t="inlineStr">
-        <is>
-          <t>gm-med.ru</t>
-        </is>
-      </c>
-      <c r="B30" t="n">
-        <v>33</v>
-      </c>
-      <c r="C30" t="n">
-        <v>1</v>
-      </c>
-      <c r="D30" t="n">
-        <v>0</v>
-      </c>
-      <c r="E30" t="n">
-        <v>36</v>
-      </c>
-      <c r="F30" t="n">
-        <v>259</v>
-      </c>
-      <c r="G30" t="n">
-        <v>647</v>
-      </c>
-      <c r="H30" t="n">
-        <v>6245</v>
-      </c>
-      <c r="I30" t="inlineStr">
-        <is>
-          <t>https://gm-med.ru/catalog/akusherstvo-i-ginekologiya</t>
-        </is>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" t="inlineStr">
-        <is>
-          <t>medmetr.ru</t>
-        </is>
-      </c>
-      <c r="B31" t="n">
-        <v>32</v>
-      </c>
-      <c r="C31" t="n">
-        <v>1</v>
-      </c>
-      <c r="D31" t="n">
-        <v>0</v>
-      </c>
-      <c r="E31" t="n">
-        <v>25</v>
-      </c>
-      <c r="F31" t="n">
-        <v>255</v>
-      </c>
-      <c r="G31" t="n">
-        <v>606</v>
-      </c>
-      <c r="H31" t="n">
-        <v>5485</v>
-      </c>
-      <c r="I31" t="inlineStr">
-        <is>
-          <t>https://medmetr.ru/catalog/ginekologiia-akusherstvo</t>
-        </is>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" t="inlineStr">
-        <is>
-          <t>gnkmed.ru</t>
-        </is>
-      </c>
-      <c r="B32" t="n">
-        <v>9</v>
-      </c>
-      <c r="C32" t="n">
-        <v>1</v>
-      </c>
-      <c r="D32" t="n">
-        <v>1</v>
-      </c>
-      <c r="E32" t="n">
-        <v>24</v>
-      </c>
-      <c r="F32" t="n">
-        <v>229</v>
-      </c>
-      <c r="G32" t="n">
-        <v>504</v>
-      </c>
-      <c r="H32" t="n">
-        <v>1818</v>
-      </c>
-      <c r="I32" t="inlineStr">
-        <is>
-          <t>https://gnkmed.ru/catalog/ginekologicheskie-kombayny-otopront</t>
-        </is>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" t="inlineStr">
-        <is>
-          <t>dixion.ru</t>
-        </is>
-      </c>
-      <c r="B33" t="n">
-        <v>40</v>
-      </c>
-      <c r="C33" t="n">
-        <v>1</v>
-      </c>
-      <c r="D33" t="n">
-        <v>1</v>
-      </c>
-      <c r="E33" t="n">
-        <v>55</v>
-      </c>
-      <c r="F33" t="n">
-        <v>229</v>
-      </c>
-      <c r="G33" t="n">
-        <v>421</v>
-      </c>
-      <c r="H33" t="n">
-        <v>2752</v>
-      </c>
-      <c r="I33" t="inlineStr">
-        <is>
-          <t>https://dixion.ru/category/akusherstvo-i-ginekologiya.html</t>
-        </is>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" t="inlineStr">
-        <is>
-          <t>lotem.ru</t>
-        </is>
-      </c>
-      <c r="B34" t="n">
-        <v>43</v>
-      </c>
-      <c r="C34" t="n">
-        <v>1</v>
-      </c>
-      <c r="D34" t="n">
-        <v>0</v>
-      </c>
-      <c r="E34" t="n">
-        <v>21</v>
-      </c>
-      <c r="F34" t="n">
-        <v>199</v>
-      </c>
-      <c r="G34" t="n">
-        <v>395</v>
-      </c>
-      <c r="H34" t="n">
-        <v>1783</v>
-      </c>
-      <c r="I34" t="inlineStr">
-        <is>
-          <t>https://lotem.ru/oborudovanie/ginekologiya</t>
-        </is>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" t="inlineStr">
-        <is>
-          <t>meditems.ru</t>
-        </is>
-      </c>
-      <c r="B35" t="n">
-        <v>34</v>
-      </c>
-      <c r="C35" t="n">
-        <v>1</v>
-      </c>
-      <c r="D35" t="n">
-        <v>0</v>
-      </c>
-      <c r="E35" t="n">
-        <v>18</v>
-      </c>
-      <c r="F35" t="n">
-        <v>176</v>
-      </c>
-      <c r="G35" t="n">
-        <v>682</v>
-      </c>
-      <c r="H35" t="n">
-        <v>9245</v>
-      </c>
-      <c r="I35" t="inlineStr">
-        <is>
-          <t>https://meditems.ru/catalog/ginekologiya_i_akusherstvo</t>
-        </is>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" t="inlineStr">
-        <is>
-          <t>fujitora.com</t>
-        </is>
-      </c>
-      <c r="B36" t="n">
-        <v>42</v>
-      </c>
-      <c r="C36" t="n">
-        <v>1</v>
-      </c>
-      <c r="D36" t="n">
-        <v>0</v>
-      </c>
-      <c r="E36" t="n">
-        <v>19</v>
-      </c>
-      <c r="F36" t="n">
-        <v>148</v>
-      </c>
-      <c r="G36" t="n">
-        <v>419</v>
-      </c>
-      <c r="H36" t="n">
-        <v>3012</v>
-      </c>
-      <c r="I36" t="inlineStr">
-        <is>
-          <t>https://fujitora.com/catalog/ginekologiya</t>
-        </is>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" t="inlineStr">
-        <is>
-          <t>rusmedcompany.ru</t>
-        </is>
-      </c>
-      <c r="B37" t="n">
-        <v>37</v>
-      </c>
-      <c r="C37" t="n">
-        <v>1</v>
-      </c>
-      <c r="D37" t="n">
-        <v>0</v>
-      </c>
-      <c r="E37" t="n">
-        <v>12</v>
-      </c>
-      <c r="F37" t="n">
-        <v>108</v>
-      </c>
-      <c r="G37" t="n">
-        <v>357</v>
-      </c>
-      <c r="H37" t="n">
-        <v>7086</v>
-      </c>
-      <c r="I37" t="inlineStr">
-        <is>
-          <t>https://rusmedcompany.ru/catalog/ginekologiya</t>
-        </is>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" t="inlineStr">
-        <is>
-          <t>gsmedicine.ru</t>
-        </is>
-      </c>
-      <c r="B38" t="n">
-        <v>23</v>
-      </c>
-      <c r="C38" t="n">
-        <v>1</v>
-      </c>
-      <c r="D38" t="n">
-        <v>0</v>
-      </c>
-      <c r="E38" t="n">
-        <v>5</v>
-      </c>
-      <c r="F38" t="n">
-        <v>33</v>
-      </c>
-      <c r="G38" t="n">
-        <v>87</v>
-      </c>
-      <c r="H38" t="n">
-        <v>722</v>
-      </c>
-      <c r="I38" t="inlineStr">
-        <is>
-          <t>https://gsmedicine.ru/product/ginekologicheskoe-oborudovanie</t>
-        </is>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" t="inlineStr">
-        <is>
-          <t>eurotech.ru</t>
-        </is>
-      </c>
-      <c r="B39" t="n">
-        <v>39</v>
-      </c>
-      <c r="C39" t="n">
-        <v>1</v>
-      </c>
-      <c r="D39" t="n">
-        <v>0</v>
-      </c>
-      <c r="E39" t="n">
-        <v>1</v>
-      </c>
-      <c r="F39" t="n">
-        <v>17</v>
-      </c>
-      <c r="G39" t="n">
-        <v>33</v>
-      </c>
-      <c r="H39" t="n">
-        <v>216</v>
-      </c>
-      <c r="I39" t="inlineStr">
-        <is>
-          <t>https://eurotech.ru/catalog/ginekologicheskoe-i-akusherskoe-oborudovanie</t>
-        </is>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" t="inlineStr">
-        <is>
-          <t>ro-med.ru</t>
-        </is>
-      </c>
-      <c r="B40" t="n">
-        <v>41</v>
-      </c>
-      <c r="C40" t="n">
-        <v>1</v>
-      </c>
-      <c r="D40" t="n">
-        <v>0</v>
-      </c>
-      <c r="E40" t="n">
-        <v>0</v>
-      </c>
-      <c r="F40" t="n">
-        <v>2</v>
-      </c>
-      <c r="G40" t="n">
-        <v>8</v>
-      </c>
-      <c r="H40" t="n">
-        <v>324</v>
-      </c>
-      <c r="I40" t="inlineStr">
-        <is>
-          <t>https://msk.ro-med.ru/catalog/gynecology</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add fotek.ru and medgrade.pro, keep 20 competitors
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01GGxzKXyeNbw77cRhpGHusQ
</commit_message>
<xml_diff>
--- a/out/analiz_konkurentov_reiginmed.xlsx
+++ b/out/analiz_konkurentov_reiginmed.xlsx
@@ -4069,7 +4069,7 @@
       </c>
       <c r="B18" s="28" t="inlineStr">
         <is>
-          <t>https://ambimed.ru/</t>
+          <t>https://intelmed.ru/</t>
         </is>
       </c>
       <c r="C18" s="31">
@@ -4089,12 +4089,8 @@
       <c r="K18" s="131" t="n"/>
       <c r="L18" s="40" t="n"/>
       <c r="M18" s="41" t="n"/>
-      <c r="N18" s="42" t="n">
-        <v>1194</v>
-      </c>
-      <c r="O18" s="255" t="n">
-        <v>21325</v>
-      </c>
+      <c r="N18" s="42" t="n"/>
+      <c r="O18" s="255" t="n"/>
       <c r="P18" s="44" t="n"/>
       <c r="Q18" s="311" t="n"/>
       <c r="R18" s="46">
@@ -4114,7 +4110,7 @@
       <c r="W18" s="50" t="n"/>
       <c r="X18" s="262" t="inlineStr">
         <is>
-          <t>Слабый конкурент</t>
+          <t>Более широкий конкурент</t>
         </is>
       </c>
     </row>
@@ -4125,7 +4121,7 @@
       </c>
       <c r="B19" s="28" t="inlineStr">
         <is>
-          <t>https://eurosmed.ru/</t>
+          <t>https://kriptomed.ru/</t>
         </is>
       </c>
       <c r="C19" s="31">
@@ -4145,12 +4141,8 @@
       <c r="K19" s="131" t="n"/>
       <c r="L19" s="40" t="n"/>
       <c r="M19" s="41" t="n"/>
-      <c r="N19" s="42" t="n">
-        <v>971</v>
-      </c>
-      <c r="O19" s="255" t="n">
-        <v>17394</v>
-      </c>
+      <c r="N19" s="42" t="n"/>
+      <c r="O19" s="255" t="n"/>
       <c r="P19" s="44" t="n"/>
       <c r="Q19" s="311" t="n"/>
       <c r="R19" s="46">
@@ -4170,7 +4162,7 @@
       <c r="W19" s="50" t="n"/>
       <c r="X19" s="262" t="inlineStr">
         <is>
-          <t>Слабый конкурент</t>
+          <t>Более широкий конкурент</t>
         </is>
       </c>
     </row>
@@ -4181,7 +4173,7 @@
       </c>
       <c r="B20" s="28" t="inlineStr">
         <is>
-          <t>https://intelmed.ru/</t>
+          <t>https://fotek.ru/</t>
         </is>
       </c>
       <c r="C20" s="31">
@@ -4233,7 +4225,7 @@
       </c>
       <c r="B21" s="28" t="inlineStr">
         <is>
-          <t>https://kriptomed.ru/</t>
+          <t>https://medgrade.pro/</t>
         </is>
       </c>
       <c r="C21" s="31">
@@ -4694,7 +4686,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I19"/>
+  <dimension ref="A1:I17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" style="354" min="1" max="1"/>
@@ -5280,72 +5272,6 @@
       <c r="I17" t="inlineStr">
         <is>
           <t>https://uromed-m.ru/ginekologicheskoe-oborudovanie</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="inlineStr">
-        <is>
-          <t>ambimed.ru</t>
-        </is>
-      </c>
-      <c r="B18" t="n">
-        <v>17</v>
-      </c>
-      <c r="C18" t="n">
-        <v>1</v>
-      </c>
-      <c r="D18" t="n">
-        <v>3</v>
-      </c>
-      <c r="E18" t="n">
-        <v>170</v>
-      </c>
-      <c r="F18" t="n">
-        <v>1194</v>
-      </c>
-      <c r="G18" t="n">
-        <v>3211</v>
-      </c>
-      <c r="H18" t="n">
-        <v>21325</v>
-      </c>
-      <c r="I18" t="inlineStr">
-        <is>
-          <t>https://ambimed.ru/product/akusherstvo-i-ginekologiya</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" t="inlineStr">
-        <is>
-          <t>eurosmed.ru</t>
-        </is>
-      </c>
-      <c r="B19" t="n">
-        <v>13</v>
-      </c>
-      <c r="C19" t="n">
-        <v>2</v>
-      </c>
-      <c r="D19" t="n">
-        <v>1</v>
-      </c>
-      <c r="E19" t="n">
-        <v>87</v>
-      </c>
-      <c r="F19" t="n">
-        <v>971</v>
-      </c>
-      <c r="G19" t="n">
-        <v>2980</v>
-      </c>
-      <c r="H19" t="n">
-        <v>17394</v>
-      </c>
-      <c r="I19" t="inlineStr">
-        <is>
-          <t>https://eurosmed.ru/catalog/ginekologicheskoe_oborudovanie</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Fill Yandex/Google positions, visibility and link metrics from exports
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01GGxzKXyeNbw77cRhpGHusQ
</commit_message>
<xml_diff>
--- a/out/analiz_konkurentov_reiginmed.xlsx
+++ b/out/analiz_konkurentov_reiginmed.xlsx
@@ -5,10 +5,11 @@
   <sheets>
     <sheet name="Анализ конкурентов" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Данные Simple.top" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Описание метрик" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Сводная таблица лидеров" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Инструкция" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="Технический лист" sheetId="6" state="hidden" r:id="rId6"/>
+    <sheet name="Доп. метрики" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Описание метрик" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Сводная таблица лидеров" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Инструкция" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Технический лист" sheetId="7" state="hidden" r:id="rId7"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Анализ конкурентов'!$A$1:$V$23</definedName>
@@ -3189,9 +3190,13 @@
       <c r="G2" s="35" t="n"/>
       <c r="H2" s="36" t="n"/>
       <c r="I2" s="37" t="n"/>
-      <c r="J2" s="38" t="n"/>
+      <c r="J2" s="38" t="n">
+        <v>895089</v>
+      </c>
       <c r="K2" s="131" t="n"/>
-      <c r="L2" s="40" t="n"/>
+      <c r="L2" s="40" t="n">
+        <v>333910</v>
+      </c>
       <c r="M2" s="41" t="n"/>
       <c r="N2" s="42" t="n">
         <v>34000</v>
@@ -3199,8 +3204,12 @@
       <c r="O2" s="255" t="n">
         <v>139372</v>
       </c>
-      <c r="P2" s="44" t="n"/>
-      <c r="Q2" s="311" t="n"/>
+      <c r="P2" s="44" t="n">
+        <v>12702</v>
+      </c>
+      <c r="Q2" s="311" t="n">
+        <v>82276</v>
+      </c>
       <c r="R2" s="46">
         <f>IFERROR(N2/O2,"")</f>
         <v/>
@@ -3209,13 +3218,19 @@
         <f>IFERROR(P2/Q2,"")</f>
         <v/>
       </c>
-      <c r="T2" s="47" t="n"/>
-      <c r="U2" s="48" t="n"/>
+      <c r="T2" s="47" t="n">
+        <v>632</v>
+      </c>
+      <c r="U2" s="48" t="n">
+        <v>4780</v>
+      </c>
       <c r="V2" s="49">
         <f>IFERROR(U2/T2,"")</f>
         <v/>
       </c>
-      <c r="W2" s="50" t="n"/>
+      <c r="W2" s="50" t="n">
+        <v>35</v>
+      </c>
       <c r="X2" s="64" t="inlineStr">
         <is>
           <t xml:space="preserve"> Лидер</t>
@@ -3245,9 +3260,13 @@
       <c r="G3" s="35" t="n"/>
       <c r="H3" s="36" t="n"/>
       <c r="I3" s="37" t="n"/>
-      <c r="J3" s="38" t="n"/>
+      <c r="J3" s="38" t="n">
+        <v>227153</v>
+      </c>
       <c r="K3" s="131" t="n"/>
-      <c r="L3" s="40" t="n"/>
+      <c r="L3" s="40" t="n">
+        <v>532882</v>
+      </c>
       <c r="M3" s="41" t="n"/>
       <c r="N3" s="42" t="n">
         <v>12027</v>
@@ -3255,8 +3274,12 @@
       <c r="O3" s="255" t="n">
         <v>42378</v>
       </c>
-      <c r="P3" s="44" t="n"/>
-      <c r="Q3" s="311" t="n"/>
+      <c r="P3" s="44" t="n">
+        <v>14364</v>
+      </c>
+      <c r="Q3" s="311" t="n">
+        <v>42983</v>
+      </c>
       <c r="R3" s="46">
         <f>IFERROR(N3/O3,"")</f>
         <v/>
@@ -3265,13 +3288,19 @@
         <f>IFERROR(P3/Q3,"")</f>
         <v/>
       </c>
-      <c r="T3" s="47" t="n"/>
-      <c r="U3" s="48" t="n"/>
+      <c r="T3" s="47" t="n">
+        <v>490</v>
+      </c>
+      <c r="U3" s="48" t="n">
+        <v>8330</v>
+      </c>
       <c r="V3" s="49">
         <f>IFERROR(U3/T3,"")</f>
         <v/>
       </c>
-      <c r="W3" s="50" t="n"/>
+      <c r="W3" s="50" t="n">
+        <v>34</v>
+      </c>
       <c r="X3" s="64" t="inlineStr">
         <is>
           <t xml:space="preserve"> Лидер</t>
@@ -3301,9 +3330,13 @@
       <c r="G4" s="35" t="n"/>
       <c r="H4" s="36" t="n"/>
       <c r="I4" s="37" t="n"/>
-      <c r="J4" s="38" t="n"/>
+      <c r="J4" s="38" t="n">
+        <v>150351</v>
+      </c>
       <c r="K4" s="131" t="n"/>
-      <c r="L4" s="40" t="n"/>
+      <c r="L4" s="40" t="n">
+        <v>103519</v>
+      </c>
       <c r="M4" s="41" t="n"/>
       <c r="N4" s="42" t="n">
         <v>8912</v>
@@ -3311,8 +3344,12 @@
       <c r="O4" s="255" t="n">
         <v>17944</v>
       </c>
-      <c r="P4" s="44" t="n"/>
-      <c r="Q4" s="311" t="n"/>
+      <c r="P4" s="44" t="n">
+        <v>5014</v>
+      </c>
+      <c r="Q4" s="311" t="n">
+        <v>17355</v>
+      </c>
       <c r="R4" s="46">
         <f>IFERROR(N4/O4,"")</f>
         <v/>
@@ -3321,13 +3358,19 @@
         <f>IFERROR(P4/Q4,"")</f>
         <v/>
       </c>
-      <c r="T4" s="47" t="n"/>
-      <c r="U4" s="48" t="n"/>
+      <c r="T4" s="47" t="n">
+        <v>566</v>
+      </c>
+      <c r="U4" s="48" t="n">
+        <v>23306</v>
+      </c>
       <c r="V4" s="49">
         <f>IFERROR(U4/T4,"")</f>
         <v/>
       </c>
-      <c r="W4" s="50" t="n"/>
+      <c r="W4" s="50" t="n">
+        <v>36</v>
+      </c>
       <c r="X4" s="64" t="inlineStr">
         <is>
           <t xml:space="preserve"> Лидер</t>
@@ -3357,9 +3400,13 @@
       <c r="G5" s="35" t="n"/>
       <c r="H5" s="36" t="n"/>
       <c r="I5" s="37" t="n"/>
-      <c r="J5" s="38" t="n"/>
+      <c r="J5" s="38" t="n">
+        <v>81164</v>
+      </c>
       <c r="K5" s="131" t="n"/>
-      <c r="L5" s="40" t="n"/>
+      <c r="L5" s="40" t="n">
+        <v>88676</v>
+      </c>
       <c r="M5" s="41" t="n"/>
       <c r="N5" s="42" t="n">
         <v>6795</v>
@@ -3367,8 +3414,12 @@
       <c r="O5" s="255" t="n">
         <v>80522</v>
       </c>
-      <c r="P5" s="44" t="n"/>
-      <c r="Q5" s="311" t="n"/>
+      <c r="P5" s="44" t="n">
+        <v>4490</v>
+      </c>
+      <c r="Q5" s="311" t="n">
+        <v>61946</v>
+      </c>
       <c r="R5" s="46">
         <f>IFERROR(N5/O5,"")</f>
         <v/>
@@ -3377,13 +3428,19 @@
         <f>IFERROR(P5/Q5,"")</f>
         <v/>
       </c>
-      <c r="T5" s="47" t="n"/>
-      <c r="U5" s="48" t="n"/>
+      <c r="T5" s="47" t="n">
+        <v>392</v>
+      </c>
+      <c r="U5" s="48" t="n">
+        <v>2986</v>
+      </c>
       <c r="V5" s="49">
         <f>IFERROR(U5/T5,"")</f>
         <v/>
       </c>
-      <c r="W5" s="50" t="n"/>
+      <c r="W5" s="50" t="n">
+        <v>29</v>
+      </c>
       <c r="X5" s="64" t="inlineStr">
         <is>
           <t xml:space="preserve"> Лидер</t>
@@ -3413,9 +3470,13 @@
       <c r="G6" s="35" t="n"/>
       <c r="H6" s="36" t="n"/>
       <c r="I6" s="37" t="n"/>
-      <c r="J6" s="38" t="n"/>
+      <c r="J6" s="38" t="n">
+        <v>95974</v>
+      </c>
       <c r="K6" s="131" t="n"/>
-      <c r="L6" s="40" t="n"/>
+      <c r="L6" s="40" t="n">
+        <v>21858</v>
+      </c>
       <c r="M6" s="41" t="n"/>
       <c r="N6" s="42" t="n">
         <v>6373</v>
@@ -3423,8 +3484,12 @@
       <c r="O6" s="255" t="n">
         <v>24331</v>
       </c>
-      <c r="P6" s="44" t="n"/>
-      <c r="Q6" s="311" t="n"/>
+      <c r="P6" s="44" t="n">
+        <v>1403</v>
+      </c>
+      <c r="Q6" s="311" t="n">
+        <v>16059</v>
+      </c>
       <c r="R6" s="46">
         <f>IFERROR(N6/O6,"")</f>
         <v/>
@@ -3433,13 +3498,19 @@
         <f>IFERROR(P6/Q6,"")</f>
         <v/>
       </c>
-      <c r="T6" s="47" t="n"/>
-      <c r="U6" s="48" t="n"/>
+      <c r="T6" s="47" t="n">
+        <v>79</v>
+      </c>
+      <c r="U6" s="48" t="n">
+        <v>394</v>
+      </c>
       <c r="V6" s="49">
         <f>IFERROR(U6/T6,"")</f>
         <v/>
       </c>
-      <c r="W6" s="50" t="n"/>
+      <c r="W6" s="50" t="n">
+        <v>25</v>
+      </c>
       <c r="X6" s="64" t="inlineStr">
         <is>
           <t xml:space="preserve"> Лидер</t>
@@ -3469,9 +3540,13 @@
       <c r="G7" s="35" t="n"/>
       <c r="H7" s="36" t="n"/>
       <c r="I7" s="37" t="n"/>
-      <c r="J7" s="38" t="n"/>
+      <c r="J7" s="38" t="n">
+        <v>70465</v>
+      </c>
       <c r="K7" s="131" t="n"/>
-      <c r="L7" s="40" t="n"/>
+      <c r="L7" s="40" t="n">
+        <v>8117</v>
+      </c>
       <c r="M7" s="41" t="n"/>
       <c r="N7" s="42" t="n">
         <v>6043</v>
@@ -3479,8 +3554,12 @@
       <c r="O7" s="255" t="n">
         <v>19713</v>
       </c>
-      <c r="P7" s="44" t="n"/>
-      <c r="Q7" s="311" t="n"/>
+      <c r="P7" s="44" t="n">
+        <v>440</v>
+      </c>
+      <c r="Q7" s="311" t="n">
+        <v>7340</v>
+      </c>
       <c r="R7" s="46">
         <f>IFERROR(N7/O7,"")</f>
         <v/>
@@ -3489,13 +3568,19 @@
         <f>IFERROR(P7/Q7,"")</f>
         <v/>
       </c>
-      <c r="T7" s="47" t="n"/>
-      <c r="U7" s="48" t="n"/>
+      <c r="T7" s="47" t="n">
+        <v>322</v>
+      </c>
+      <c r="U7" s="48" t="n">
+        <v>1962</v>
+      </c>
       <c r="V7" s="49">
         <f>IFERROR(U7/T7,"")</f>
         <v/>
       </c>
-      <c r="W7" s="50" t="n"/>
+      <c r="W7" s="50" t="n">
+        <v>35</v>
+      </c>
       <c r="X7" s="64" t="inlineStr">
         <is>
           <t xml:space="preserve"> Лидер</t>
@@ -3525,9 +3610,13 @@
       <c r="G8" s="35" t="n"/>
       <c r="H8" s="36" t="n"/>
       <c r="I8" s="37" t="n"/>
-      <c r="J8" s="38" t="n"/>
+      <c r="J8" s="38" t="n">
+        <v>72336</v>
+      </c>
       <c r="K8" s="131" t="n"/>
-      <c r="L8" s="40" t="n"/>
+      <c r="L8" s="40" t="n">
+        <v>29067</v>
+      </c>
       <c r="M8" s="41" t="n"/>
       <c r="N8" s="42" t="n">
         <v>4514</v>
@@ -3535,8 +3624,12 @@
       <c r="O8" s="255" t="n">
         <v>17901</v>
       </c>
-      <c r="P8" s="44" t="n"/>
-      <c r="Q8" s="311" t="n"/>
+      <c r="P8" s="44" t="n">
+        <v>1277</v>
+      </c>
+      <c r="Q8" s="311" t="n">
+        <v>7205</v>
+      </c>
       <c r="R8" s="46">
         <f>IFERROR(N8/O8,"")</f>
         <v/>
@@ -3545,13 +3638,19 @@
         <f>IFERROR(P8/Q8,"")</f>
         <v/>
       </c>
-      <c r="T8" s="47" t="n"/>
-      <c r="U8" s="48" t="n"/>
+      <c r="T8" s="47" t="n">
+        <v>69</v>
+      </c>
+      <c r="U8" s="48" t="n">
+        <v>182</v>
+      </c>
       <c r="V8" s="49">
         <f>IFERROR(U8/T8,"")</f>
         <v/>
       </c>
-      <c r="W8" s="50" t="n"/>
+      <c r="W8" s="50" t="n">
+        <v>31</v>
+      </c>
       <c r="X8" s="64" t="inlineStr">
         <is>
           <t xml:space="preserve"> Лидер</t>
@@ -3581,9 +3680,13 @@
       <c r="G9" s="35" t="n"/>
       <c r="H9" s="36" t="n"/>
       <c r="I9" s="37" t="n"/>
-      <c r="J9" s="38" t="n"/>
+      <c r="J9" s="38" t="n">
+        <v>21573</v>
+      </c>
       <c r="K9" s="131" t="n"/>
-      <c r="L9" s="40" t="n"/>
+      <c r="L9" s="40" t="n">
+        <v>83848</v>
+      </c>
       <c r="M9" s="41" t="n"/>
       <c r="N9" s="42" t="n">
         <v>2687</v>
@@ -3591,8 +3694,12 @@
       <c r="O9" s="255" t="n">
         <v>18562</v>
       </c>
-      <c r="P9" s="44" t="n"/>
-      <c r="Q9" s="311" t="n"/>
+      <c r="P9" s="44" t="n">
+        <v>3791</v>
+      </c>
+      <c r="Q9" s="311" t="n">
+        <v>22596</v>
+      </c>
       <c r="R9" s="46">
         <f>IFERROR(N9/O9,"")</f>
         <v/>
@@ -3601,13 +3708,19 @@
         <f>IFERROR(P9/Q9,"")</f>
         <v/>
       </c>
-      <c r="T9" s="47" t="n"/>
-      <c r="U9" s="48" t="n"/>
+      <c r="T9" s="47" t="n">
+        <v>292</v>
+      </c>
+      <c r="U9" s="48" t="n">
+        <v>2803</v>
+      </c>
       <c r="V9" s="49">
         <f>IFERROR(U9/T9,"")</f>
         <v/>
       </c>
-      <c r="W9" s="50" t="n"/>
+      <c r="W9" s="50" t="n">
+        <v>31</v>
+      </c>
       <c r="X9" s="262" t="inlineStr">
         <is>
           <t>Слабый конкурент</t>
@@ -3637,9 +3750,13 @@
       <c r="G10" s="35" t="n"/>
       <c r="H10" s="36" t="n"/>
       <c r="I10" s="37" t="n"/>
-      <c r="J10" s="38" t="n"/>
+      <c r="J10" s="38" t="n">
+        <v>27185</v>
+      </c>
       <c r="K10" s="131" t="n"/>
-      <c r="L10" s="40" t="n"/>
+      <c r="L10" s="40" t="n">
+        <v>107840</v>
+      </c>
       <c r="M10" s="41" t="n"/>
       <c r="N10" s="42" t="n">
         <v>2671</v>
@@ -3647,8 +3764,12 @@
       <c r="O10" s="255" t="n">
         <v>39793</v>
       </c>
-      <c r="P10" s="44" t="n"/>
-      <c r="Q10" s="311" t="n"/>
+      <c r="P10" s="44" t="n">
+        <v>4726</v>
+      </c>
+      <c r="Q10" s="311" t="n">
+        <v>32743</v>
+      </c>
       <c r="R10" s="46">
         <f>IFERROR(N10/O10,"")</f>
         <v/>
@@ -3657,13 +3778,19 @@
         <f>IFERROR(P10/Q10,"")</f>
         <v/>
       </c>
-      <c r="T10" s="47" t="n"/>
-      <c r="U10" s="48" t="n"/>
+      <c r="T10" s="47" t="n">
+        <v>712</v>
+      </c>
+      <c r="U10" s="48" t="n">
+        <v>8628</v>
+      </c>
       <c r="V10" s="49">
         <f>IFERROR(U10/T10,"")</f>
         <v/>
       </c>
-      <c r="W10" s="50" t="n"/>
+      <c r="W10" s="50" t="n">
+        <v>33</v>
+      </c>
       <c r="X10" s="262" t="inlineStr">
         <is>
           <t>Слабый конкурент</t>
@@ -3693,9 +3820,13 @@
       <c r="G11" s="35" t="n"/>
       <c r="H11" s="36" t="n"/>
       <c r="I11" s="37" t="n"/>
-      <c r="J11" s="38" t="n"/>
+      <c r="J11" s="38" t="n">
+        <v>39613</v>
+      </c>
       <c r="K11" s="131" t="n"/>
-      <c r="L11" s="40" t="n"/>
+      <c r="L11" s="40" t="n">
+        <v>13726</v>
+      </c>
       <c r="M11" s="41" t="n"/>
       <c r="N11" s="42" t="n">
         <v>2595</v>
@@ -3703,8 +3834,12 @@
       <c r="O11" s="255" t="n">
         <v>12635</v>
       </c>
-      <c r="P11" s="44" t="n"/>
-      <c r="Q11" s="311" t="n"/>
+      <c r="P11" s="44" t="n">
+        <v>874</v>
+      </c>
+      <c r="Q11" s="311" t="n">
+        <v>8113</v>
+      </c>
       <c r="R11" s="46">
         <f>IFERROR(N11/O11,"")</f>
         <v/>
@@ -3713,13 +3848,19 @@
         <f>IFERROR(P11/Q11,"")</f>
         <v/>
       </c>
-      <c r="T11" s="47" t="n"/>
-      <c r="U11" s="48" t="n"/>
+      <c r="T11" s="47" t="n">
+        <v>107</v>
+      </c>
+      <c r="U11" s="48" t="n">
+        <v>363</v>
+      </c>
       <c r="V11" s="49">
         <f>IFERROR(U11/T11,"")</f>
         <v/>
       </c>
-      <c r="W11" s="50" t="n"/>
+      <c r="W11" s="50" t="n">
+        <v>27</v>
+      </c>
       <c r="X11" s="262" t="inlineStr">
         <is>
           <t>Слабый конкурент</t>
@@ -3749,9 +3890,13 @@
       <c r="G12" s="35" t="n"/>
       <c r="H12" s="36" t="n"/>
       <c r="I12" s="37" t="n"/>
-      <c r="J12" s="38" t="n"/>
+      <c r="J12" s="38" t="n">
+        <v>21474</v>
+      </c>
       <c r="K12" s="131" t="n"/>
-      <c r="L12" s="40" t="n"/>
+      <c r="L12" s="40" t="n">
+        <v>2035</v>
+      </c>
       <c r="M12" s="41" t="n"/>
       <c r="N12" s="42" t="n">
         <v>2067</v>
@@ -3759,8 +3904,12 @@
       <c r="O12" s="255" t="n">
         <v>17494</v>
       </c>
-      <c r="P12" s="44" t="n"/>
-      <c r="Q12" s="311" t="n"/>
+      <c r="P12" s="44" t="n">
+        <v>151</v>
+      </c>
+      <c r="Q12" s="311" t="n">
+        <v>4310</v>
+      </c>
       <c r="R12" s="46">
         <f>IFERROR(N12/O12,"")</f>
         <v/>
@@ -3769,13 +3918,19 @@
         <f>IFERROR(P12/Q12,"")</f>
         <v/>
       </c>
-      <c r="T12" s="47" t="n"/>
-      <c r="U12" s="48" t="n"/>
+      <c r="T12" s="47" t="n">
+        <v>121</v>
+      </c>
+      <c r="U12" s="48" t="n">
+        <v>248</v>
+      </c>
       <c r="V12" s="49">
         <f>IFERROR(U12/T12,"")</f>
         <v/>
       </c>
-      <c r="W12" s="50" t="n"/>
+      <c r="W12" s="50" t="n">
+        <v>28</v>
+      </c>
       <c r="X12" s="262" t="inlineStr">
         <is>
           <t>Слабый конкурент</t>
@@ -3805,9 +3960,13 @@
       <c r="G13" s="35" t="n"/>
       <c r="H13" s="36" t="n"/>
       <c r="I13" s="37" t="n"/>
-      <c r="J13" s="38" t="n"/>
+      <c r="J13" s="38" t="n">
+        <v>21260</v>
+      </c>
       <c r="K13" s="131" t="n"/>
-      <c r="L13" s="40" t="n"/>
+      <c r="L13" s="40" t="n">
+        <v>5156</v>
+      </c>
       <c r="M13" s="41" t="n"/>
       <c r="N13" s="42" t="n">
         <v>1973</v>
@@ -3815,8 +3974,12 @@
       <c r="O13" s="255" t="n">
         <v>19233</v>
       </c>
-      <c r="P13" s="44" t="n"/>
-      <c r="Q13" s="311" t="n"/>
+      <c r="P13" s="44" t="n">
+        <v>249</v>
+      </c>
+      <c r="Q13" s="311" t="n">
+        <v>6835</v>
+      </c>
       <c r="R13" s="46">
         <f>IFERROR(N13/O13,"")</f>
         <v/>
@@ -3825,13 +3988,19 @@
         <f>IFERROR(P13/Q13,"")</f>
         <v/>
       </c>
-      <c r="T13" s="47" t="n"/>
-      <c r="U13" s="48" t="n"/>
+      <c r="T13" s="47" t="n">
+        <v>262</v>
+      </c>
+      <c r="U13" s="48" t="n">
+        <v>1037</v>
+      </c>
       <c r="V13" s="49">
         <f>IFERROR(U13/T13,"")</f>
         <v/>
       </c>
-      <c r="W13" s="50" t="n"/>
+      <c r="W13" s="50" t="n">
+        <v>22</v>
+      </c>
       <c r="X13" s="262" t="inlineStr">
         <is>
           <t>Слабый конкурент</t>
@@ -3861,9 +4030,13 @@
       <c r="G14" s="35" t="n"/>
       <c r="H14" s="36" t="n"/>
       <c r="I14" s="37" t="n"/>
-      <c r="J14" s="38" t="n"/>
+      <c r="J14" s="38" t="n">
+        <v>32260</v>
+      </c>
       <c r="K14" s="131" t="n"/>
-      <c r="L14" s="40" t="n"/>
+      <c r="L14" s="40" t="n">
+        <v>33398</v>
+      </c>
       <c r="M14" s="41" t="n"/>
       <c r="N14" s="42" t="n">
         <v>1826</v>
@@ -3871,8 +4044,12 @@
       <c r="O14" s="255" t="n">
         <v>16120</v>
       </c>
-      <c r="P14" s="44" t="n"/>
-      <c r="Q14" s="311" t="n"/>
+      <c r="P14" s="44" t="n">
+        <v>1321</v>
+      </c>
+      <c r="Q14" s="311" t="n">
+        <v>10167</v>
+      </c>
       <c r="R14" s="46">
         <f>IFERROR(N14/O14,"")</f>
         <v/>
@@ -3881,13 +4058,19 @@
         <f>IFERROR(P14/Q14,"")</f>
         <v/>
       </c>
-      <c r="T14" s="47" t="n"/>
-      <c r="U14" s="48" t="n"/>
+      <c r="T14" s="47" t="n">
+        <v>269</v>
+      </c>
+      <c r="U14" s="48" t="n">
+        <v>1446</v>
+      </c>
       <c r="V14" s="49">
         <f>IFERROR(U14/T14,"")</f>
         <v/>
       </c>
-      <c r="W14" s="50" t="n"/>
+      <c r="W14" s="50" t="n">
+        <v>32</v>
+      </c>
       <c r="X14" s="262" t="inlineStr">
         <is>
           <t>Слабый конкурент</t>
@@ -3917,9 +4100,13 @@
       <c r="G15" s="35" t="n"/>
       <c r="H15" s="36" t="n"/>
       <c r="I15" s="37" t="n"/>
-      <c r="J15" s="38" t="n"/>
+      <c r="J15" s="38" t="n">
+        <v>37751</v>
+      </c>
       <c r="K15" s="131" t="n"/>
-      <c r="L15" s="40" t="n"/>
+      <c r="L15" s="40" t="n">
+        <v>22013</v>
+      </c>
       <c r="M15" s="41" t="n"/>
       <c r="N15" s="42" t="n">
         <v>1795</v>
@@ -3927,8 +4114,12 @@
       <c r="O15" s="255" t="n">
         <v>31655</v>
       </c>
-      <c r="P15" s="44" t="n"/>
-      <c r="Q15" s="311" t="n"/>
+      <c r="P15" s="44" t="n">
+        <v>1242</v>
+      </c>
+      <c r="Q15" s="311" t="n">
+        <v>15963</v>
+      </c>
       <c r="R15" s="46">
         <f>IFERROR(N15/O15,"")</f>
         <v/>
@@ -3937,13 +4128,19 @@
         <f>IFERROR(P15/Q15,"")</f>
         <v/>
       </c>
-      <c r="T15" s="47" t="n"/>
-      <c r="U15" s="48" t="n"/>
+      <c r="T15" s="47" t="n">
+        <v>256</v>
+      </c>
+      <c r="U15" s="48" t="n">
+        <v>7606</v>
+      </c>
       <c r="V15" s="49">
         <f>IFERROR(U15/T15,"")</f>
         <v/>
       </c>
-      <c r="W15" s="50" t="n"/>
+      <c r="W15" s="50" t="n">
+        <v>29</v>
+      </c>
       <c r="X15" s="262" t="inlineStr">
         <is>
           <t>Слабый конкурент</t>
@@ -3973,9 +4170,13 @@
       <c r="G16" s="35" t="n"/>
       <c r="H16" s="36" t="n"/>
       <c r="I16" s="37" t="n"/>
-      <c r="J16" s="38" t="n"/>
+      <c r="J16" s="38" t="n">
+        <v>15955</v>
+      </c>
       <c r="K16" s="131" t="n"/>
-      <c r="L16" s="40" t="n"/>
+      <c r="L16" s="40" t="n">
+        <v>102730</v>
+      </c>
       <c r="M16" s="41" t="n"/>
       <c r="N16" s="42" t="n">
         <v>1753</v>
@@ -3983,8 +4184,12 @@
       <c r="O16" s="255" t="n">
         <v>14459</v>
       </c>
-      <c r="P16" s="44" t="n"/>
-      <c r="Q16" s="311" t="n"/>
+      <c r="P16" s="44" t="n">
+        <v>3342</v>
+      </c>
+      <c r="Q16" s="311" t="n">
+        <v>12922</v>
+      </c>
       <c r="R16" s="46">
         <f>IFERROR(N16/O16,"")</f>
         <v/>
@@ -3993,13 +4198,19 @@
         <f>IFERROR(P16/Q16,"")</f>
         <v/>
       </c>
-      <c r="T16" s="47" t="n"/>
-      <c r="U16" s="48" t="n"/>
+      <c r="T16" s="47" t="n">
+        <v>337</v>
+      </c>
+      <c r="U16" s="48" t="n">
+        <v>1791</v>
+      </c>
       <c r="V16" s="49">
         <f>IFERROR(U16/T16,"")</f>
         <v/>
       </c>
-      <c r="W16" s="50" t="n"/>
+      <c r="W16" s="50" t="n">
+        <v>31</v>
+      </c>
       <c r="X16" s="262" t="inlineStr">
         <is>
           <t>Слабый конкурент</t>
@@ -4029,9 +4240,13 @@
       <c r="G17" s="35" t="n"/>
       <c r="H17" s="36" t="n"/>
       <c r="I17" s="37" t="n"/>
-      <c r="J17" s="38" t="n"/>
+      <c r="J17" s="38" t="n">
+        <v>21301</v>
+      </c>
       <c r="K17" s="131" t="n"/>
-      <c r="L17" s="40" t="n"/>
+      <c r="L17" s="40" t="n">
+        <v>92887</v>
+      </c>
       <c r="M17" s="41" t="n"/>
       <c r="N17" s="42" t="n">
         <v>1209</v>
@@ -4039,8 +4254,12 @@
       <c r="O17" s="255" t="n">
         <v>8364</v>
       </c>
-      <c r="P17" s="44" t="n"/>
-      <c r="Q17" s="311" t="n"/>
+      <c r="P17" s="44" t="n">
+        <v>2275</v>
+      </c>
+      <c r="Q17" s="311" t="n">
+        <v>11370</v>
+      </c>
       <c r="R17" s="46">
         <f>IFERROR(N17/O17,"")</f>
         <v/>
@@ -4049,13 +4268,19 @@
         <f>IFERROR(P17/Q17,"")</f>
         <v/>
       </c>
-      <c r="T17" s="47" t="n"/>
-      <c r="U17" s="48" t="n"/>
+      <c r="T17" s="47" t="n">
+        <v>287</v>
+      </c>
+      <c r="U17" s="48" t="n">
+        <v>750</v>
+      </c>
       <c r="V17" s="49">
         <f>IFERROR(U17/T17,"")</f>
         <v/>
       </c>
-      <c r="W17" s="50" t="n"/>
+      <c r="W17" s="50" t="n">
+        <v>34</v>
+      </c>
       <c r="X17" s="262" t="inlineStr">
         <is>
           <t>Слабый конкурент</t>
@@ -4085,14 +4310,26 @@
       <c r="G18" s="35" t="n"/>
       <c r="H18" s="36" t="n"/>
       <c r="I18" s="37" t="n"/>
-      <c r="J18" s="38" t="n"/>
+      <c r="J18" s="38" t="n">
+        <v>2545</v>
+      </c>
       <c r="K18" s="131" t="n"/>
-      <c r="L18" s="40" t="n"/>
+      <c r="L18" s="40" t="n">
+        <v>47773</v>
+      </c>
       <c r="M18" s="41" t="n"/>
-      <c r="N18" s="42" t="n"/>
-      <c r="O18" s="255" t="n"/>
-      <c r="P18" s="44" t="n"/>
-      <c r="Q18" s="311" t="n"/>
+      <c r="N18" s="42" t="n">
+        <v>264</v>
+      </c>
+      <c r="O18" s="255" t="n">
+        <v>5081</v>
+      </c>
+      <c r="P18" s="44" t="n">
+        <v>1499</v>
+      </c>
+      <c r="Q18" s="311" t="n">
+        <v>7622</v>
+      </c>
       <c r="R18" s="46">
         <f>IFERROR(N18/O18,"")</f>
         <v/>
@@ -4101,16 +4338,22 @@
         <f>IFERROR(P18/Q18,"")</f>
         <v/>
       </c>
-      <c r="T18" s="47" t="n"/>
-      <c r="U18" s="48" t="n"/>
+      <c r="T18" s="47" t="n">
+        <v>214</v>
+      </c>
+      <c r="U18" s="48" t="n">
+        <v>479</v>
+      </c>
       <c r="V18" s="49">
         <f>IFERROR(U18/T18,"")</f>
         <v/>
       </c>
-      <c r="W18" s="50" t="n"/>
+      <c r="W18" s="50" t="n">
+        <v>24</v>
+      </c>
       <c r="X18" s="262" t="inlineStr">
         <is>
-          <t>Более широкий конкурент</t>
+          <t>Слабый конкурент</t>
         </is>
       </c>
     </row>
@@ -4137,14 +4380,26 @@
       <c r="G19" s="35" t="n"/>
       <c r="H19" s="36" t="n"/>
       <c r="I19" s="37" t="n"/>
-      <c r="J19" s="38" t="n"/>
+      <c r="J19" s="38" t="n">
+        <v>17437</v>
+      </c>
       <c r="K19" s="131" t="n"/>
-      <c r="L19" s="40" t="n"/>
+      <c r="L19" s="40" t="n">
+        <v>38052</v>
+      </c>
       <c r="M19" s="41" t="n"/>
-      <c r="N19" s="42" t="n"/>
-      <c r="O19" s="255" t="n"/>
-      <c r="P19" s="44" t="n"/>
-      <c r="Q19" s="311" t="n"/>
+      <c r="N19" s="42" t="n">
+        <v>1086</v>
+      </c>
+      <c r="O19" s="255" t="n">
+        <v>9184</v>
+      </c>
+      <c r="P19" s="44" t="n">
+        <v>1224</v>
+      </c>
+      <c r="Q19" s="311" t="n">
+        <v>6996</v>
+      </c>
       <c r="R19" s="46">
         <f>IFERROR(N19/O19,"")</f>
         <v/>
@@ -4153,16 +4408,22 @@
         <f>IFERROR(P19/Q19,"")</f>
         <v/>
       </c>
-      <c r="T19" s="47" t="n"/>
-      <c r="U19" s="48" t="n"/>
+      <c r="T19" s="47" t="n">
+        <v>127</v>
+      </c>
+      <c r="U19" s="48" t="n">
+        <v>253</v>
+      </c>
       <c r="V19" s="49">
         <f>IFERROR(U19/T19,"")</f>
         <v/>
       </c>
-      <c r="W19" s="50" t="n"/>
+      <c r="W19" s="50" t="n">
+        <v>26</v>
+      </c>
       <c r="X19" s="262" t="inlineStr">
         <is>
-          <t>Более широкий конкурент</t>
+          <t>Слабый конкурент</t>
         </is>
       </c>
     </row>
@@ -4189,14 +4450,26 @@
       <c r="G20" s="35" t="n"/>
       <c r="H20" s="36" t="n"/>
       <c r="I20" s="37" t="n"/>
-      <c r="J20" s="38" t="n"/>
+      <c r="J20" s="38" t="n">
+        <v>4906</v>
+      </c>
       <c r="K20" s="131" t="n"/>
-      <c r="L20" s="40" t="n"/>
+      <c r="L20" s="40" t="n">
+        <v>9862</v>
+      </c>
       <c r="M20" s="41" t="n"/>
-      <c r="N20" s="42" t="n"/>
-      <c r="O20" s="255" t="n"/>
-      <c r="P20" s="44" t="n"/>
-      <c r="Q20" s="311" t="n"/>
+      <c r="N20" s="42" t="n">
+        <v>319</v>
+      </c>
+      <c r="O20" s="255" t="n">
+        <v>2549</v>
+      </c>
+      <c r="P20" s="44" t="n">
+        <v>468</v>
+      </c>
+      <c r="Q20" s="311" t="n">
+        <v>2338</v>
+      </c>
       <c r="R20" s="46">
         <f>IFERROR(N20/O20,"")</f>
         <v/>
@@ -4205,16 +4478,22 @@
         <f>IFERROR(P20/Q20,"")</f>
         <v/>
       </c>
-      <c r="T20" s="47" t="n"/>
-      <c r="U20" s="48" t="n"/>
+      <c r="T20" s="47" t="n">
+        <v>197</v>
+      </c>
+      <c r="U20" s="48" t="n">
+        <v>1911</v>
+      </c>
       <c r="V20" s="49">
         <f>IFERROR(U20/T20,"")</f>
         <v/>
       </c>
-      <c r="W20" s="50" t="n"/>
+      <c r="W20" s="50" t="n">
+        <v>25</v>
+      </c>
       <c r="X20" s="262" t="inlineStr">
         <is>
-          <t>Более широкий конкурент</t>
+          <t>Слабый конкурент</t>
         </is>
       </c>
     </row>
@@ -4241,14 +4520,26 @@
       <c r="G21" s="35" t="n"/>
       <c r="H21" s="36" t="n"/>
       <c r="I21" s="37" t="n"/>
-      <c r="J21" s="38" t="n"/>
+      <c r="J21" s="38" t="n">
+        <v>16895</v>
+      </c>
       <c r="K21" s="131" t="n"/>
-      <c r="L21" s="40" t="n"/>
+      <c r="L21" s="40" t="n">
+        <v>13916</v>
+      </c>
       <c r="M21" s="41" t="n"/>
-      <c r="N21" s="42" t="n"/>
-      <c r="O21" s="255" t="n"/>
-      <c r="P21" s="44" t="n"/>
-      <c r="Q21" s="311" t="n"/>
+      <c r="N21" s="42" t="n">
+        <v>1115</v>
+      </c>
+      <c r="O21" s="255" t="n">
+        <v>8209</v>
+      </c>
+      <c r="P21" s="44" t="n">
+        <v>957</v>
+      </c>
+      <c r="Q21" s="311" t="n">
+        <v>6995</v>
+      </c>
       <c r="R21" s="46">
         <f>IFERROR(N21/O21,"")</f>
         <v/>
@@ -4257,16 +4548,22 @@
         <f>IFERROR(P21/Q21,"")</f>
         <v/>
       </c>
-      <c r="T21" s="47" t="n"/>
-      <c r="U21" s="48" t="n"/>
+      <c r="T21" s="47" t="n">
+        <v>103</v>
+      </c>
+      <c r="U21" s="48" t="n">
+        <v>253</v>
+      </c>
       <c r="V21" s="49">
         <f>IFERROR(U21/T21,"")</f>
         <v/>
       </c>
-      <c r="W21" s="50" t="n"/>
+      <c r="W21" s="50" t="n">
+        <v>26</v>
+      </c>
       <c r="X21" s="262" t="inlineStr">
         <is>
-          <t>Более широкий конкурент</t>
+          <t>Слабый конкурент</t>
         </is>
       </c>
     </row>
@@ -4321,11 +4618,11 @@
         <v/>
       </c>
       <c r="P22" s="337">
-        <f>IFERROR(MEDIAN(P2:P21),"")</f>
+        <f t="array" ref="P22">MEDIAN(IF(X2:X21=" Лидер",P2:P21))</f>
         <v/>
       </c>
       <c r="Q22" s="337">
-        <f>IFERROR(MEDIAN(Q2:Q21),"")</f>
+        <f t="array" ref="Q22">MEDIAN(IF(X2:X21=" Лидер",Q2:Q21))</f>
         <v/>
       </c>
       <c r="R22" s="341">
@@ -4333,7 +4630,7 @@
         <v/>
       </c>
       <c r="S22" s="341">
-        <f>IFERROR(MEDIAN(S2:S21),"")</f>
+        <f>P22/Q22</f>
         <v/>
       </c>
       <c r="T22" s="336">
@@ -4377,12 +4674,18 @@
       <c r="G23" s="345" t="n"/>
       <c r="H23" s="344" t="n"/>
       <c r="I23" s="346" t="n"/>
-      <c r="J23" s="348" t="n"/>
+      <c r="J23" s="348" t="n">
+        <v>0</v>
+      </c>
       <c r="K23" s="131" t="n"/>
       <c r="L23" s="348" t="n"/>
       <c r="M23" s="131" t="n"/>
-      <c r="N23" s="348" t="n"/>
-      <c r="O23" s="348" t="n"/>
+      <c r="N23" s="348" t="n">
+        <v>0</v>
+      </c>
+      <c r="O23" s="348" t="n">
+        <v>1</v>
+      </c>
       <c r="P23" s="348" t="n"/>
       <c r="Q23" s="348" t="n"/>
       <c r="R23" s="46">
@@ -4393,13 +4696,19 @@
         <f>IFERROR(P23/Q23,"")</f>
         <v/>
       </c>
-      <c r="T23" s="349" t="n"/>
-      <c r="U23" s="350" t="n"/>
+      <c r="T23" s="349" t="n">
+        <v>0</v>
+      </c>
+      <c r="U23" s="350" t="n">
+        <v>0</v>
+      </c>
       <c r="V23" s="351">
         <f>IFERROR(U23/T23,"")</f>
         <v/>
       </c>
-      <c r="W23" s="352" t="n"/>
+      <c r="W23" s="352" t="n">
+        <v>6</v>
+      </c>
       <c r="X23" s="353" t="inlineStr">
         <is>
           <t>Наш сайт</t>
@@ -4748,528 +5057,528 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
+      <c r="A2" s="0" t="inlineStr">
         <is>
           <t>dealmed.ru</t>
         </is>
       </c>
-      <c r="B2" t="n">
+      <c r="B2" s="0" t="n">
         <v>1</v>
       </c>
-      <c r="C2" t="n">
+      <c r="C2" s="0" t="n">
         <v>3</v>
       </c>
-      <c r="D2" t="n">
+      <c r="D2" s="0" t="n">
         <v>111</v>
       </c>
-      <c r="E2" t="n">
+      <c r="E2" s="0" t="n">
         <v>8095</v>
       </c>
-      <c r="F2" t="n">
+      <c r="F2" s="0" t="n">
         <v>34000</v>
       </c>
-      <c r="G2" t="n">
+      <c r="G2" s="0" t="n">
         <v>57843</v>
       </c>
-      <c r="H2" t="n">
+      <c r="H2" s="0" t="n">
         <v>139372</v>
       </c>
-      <c r="I2" t="inlineStr">
+      <c r="I2" s="0" t="inlineStr">
         <is>
           <t>https://dealmed.ru/ginekologicheskoe_oborudovanie.html</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr">
+      <c r="A3" s="0" t="inlineStr">
         <is>
           <t>medcomp.ru</t>
         </is>
       </c>
-      <c r="B3" t="n">
+      <c r="B3" s="0" t="n">
         <v>3</v>
       </c>
-      <c r="C3" t="n">
+      <c r="C3" s="0" t="n">
         <v>1</v>
       </c>
-      <c r="D3" t="n">
+      <c r="D3" s="0" t="n">
         <v>28</v>
       </c>
-      <c r="E3" t="n">
+      <c r="E3" s="0" t="n">
         <v>3014</v>
       </c>
-      <c r="F3" t="n">
+      <c r="F3" s="0" t="n">
         <v>12027</v>
       </c>
-      <c r="G3" t="n">
+      <c r="G3" s="0" t="n">
         <v>18818</v>
       </c>
-      <c r="H3" t="n">
+      <c r="H3" s="0" t="n">
         <v>42378</v>
       </c>
-      <c r="I3" t="inlineStr">
+      <c r="I3" s="0" t="inlineStr">
         <is>
           <t>https://medcomp.ru/catalog/oborudovanie/akusherstvo-i-ginekologiya</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr">
+      <c r="A4" s="0" t="inlineStr">
         <is>
           <t>medliga.ru</t>
         </is>
       </c>
-      <c r="B4" t="n">
+      <c r="B4" s="0" t="n">
         <v>2</v>
       </c>
-      <c r="C4" t="n">
+      <c r="C4" s="0" t="n">
         <v>1</v>
       </c>
-      <c r="D4" t="n">
+      <c r="D4" s="0" t="n">
         <v>19</v>
       </c>
-      <c r="E4" t="n">
+      <c r="E4" s="0" t="n">
         <v>4333</v>
       </c>
-      <c r="F4" t="n">
+      <c r="F4" s="0" t="n">
         <v>8912</v>
       </c>
-      <c r="G4" t="n">
+      <c r="G4" s="0" t="n">
         <v>11043</v>
       </c>
-      <c r="H4" t="n">
+      <c r="H4" s="0" t="n">
         <v>17944</v>
       </c>
-      <c r="I4" t="inlineStr">
+      <c r="I4" s="0" t="inlineStr">
         <is>
           <t>https://medliga.ru/catalog/ginekologiya</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="inlineStr">
+      <c r="A5" s="0" t="inlineStr">
         <is>
           <t>almamed.su</t>
         </is>
       </c>
-      <c r="B5" t="n">
+      <c r="B5" s="0" t="n">
         <v>4</v>
       </c>
-      <c r="C5" t="n">
+      <c r="C5" s="0" t="n">
         <v>1</v>
       </c>
-      <c r="D5" t="n">
+      <c r="D5" s="0" t="n">
         <v>10</v>
       </c>
-      <c r="E5" t="n">
+      <c r="E5" s="0" t="n">
         <v>672</v>
       </c>
-      <c r="F5" t="n">
+      <c r="F5" s="0" t="n">
         <v>6795</v>
       </c>
-      <c r="G5" t="n">
+      <c r="G5" s="0" t="n">
         <v>17379</v>
       </c>
-      <c r="H5" t="n">
+      <c r="H5" s="0" t="n">
         <v>80522</v>
       </c>
-      <c r="I5" t="inlineStr">
+      <c r="I5" s="0" t="inlineStr">
         <is>
           <t>https://almamed.su/category/ginekologiya</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" t="inlineStr">
+      <c r="A6" s="0" t="inlineStr">
         <is>
           <t>medcub.ru</t>
         </is>
       </c>
-      <c r="B6" t="n">
+      <c r="B6" s="0" t="n">
         <v>18</v>
       </c>
-      <c r="C6" t="n">
+      <c r="C6" s="0" t="n">
         <v>1</v>
       </c>
-      <c r="D6" t="n">
+      <c r="D6" s="0" t="n">
         <v>12</v>
       </c>
-      <c r="E6" t="n">
+      <c r="E6" s="0" t="n">
         <v>1297</v>
       </c>
-      <c r="F6" t="n">
+      <c r="F6" s="0" t="n">
         <v>6373</v>
       </c>
-      <c r="G6" t="n">
+      <c r="G6" s="0" t="n">
         <v>10031</v>
       </c>
-      <c r="H6" t="n">
+      <c r="H6" s="0" t="n">
         <v>24331</v>
       </c>
-      <c r="I6" t="inlineStr">
+      <c r="I6" s="0" t="inlineStr">
         <is>
           <t>https://medcub.ru/catalog/akusherstvo_i_ginekologiya</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" t="inlineStr">
+      <c r="A7" s="0" t="inlineStr">
         <is>
           <t>global-mt.ru</t>
         </is>
       </c>
-      <c r="B7" t="n">
+      <c r="B7" s="0" t="n">
         <v>31</v>
       </c>
-      <c r="C7" t="n">
+      <c r="C7" s="0" t="n">
         <v>1</v>
       </c>
-      <c r="D7" t="n">
+      <c r="D7" s="0" t="n">
         <v>9</v>
       </c>
-      <c r="E7" t="n">
+      <c r="E7" s="0" t="n">
         <v>1361</v>
       </c>
-      <c r="F7" t="n">
+      <c r="F7" s="0" t="n">
         <v>6043</v>
       </c>
-      <c r="G7" t="n">
+      <c r="G7" s="0" t="n">
         <v>9645</v>
       </c>
-      <c r="H7" t="n">
+      <c r="H7" s="0" t="n">
         <v>19713</v>
       </c>
-      <c r="I7" t="inlineStr">
+      <c r="I7" s="0" t="inlineStr">
         <is>
           <t>https://global-mt.ru/catalog/ginekologiya</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" t="inlineStr">
+      <c r="A8" s="0" t="inlineStr">
         <is>
           <t>gmk-kiel.ru</t>
         </is>
       </c>
-      <c r="B8" t="n">
+      <c r="B8" s="0" t="n">
         <v>6</v>
       </c>
-      <c r="C8" t="n">
+      <c r="C8" s="0" t="n">
         <v>1</v>
       </c>
-      <c r="D8" t="n">
+      <c r="D8" s="0" t="n">
         <v>9</v>
       </c>
-      <c r="E8" t="n">
+      <c r="E8" s="0" t="n">
         <v>907</v>
       </c>
-      <c r="F8" t="n">
+      <c r="F8" s="0" t="n">
         <v>4514</v>
       </c>
-      <c r="G8" t="n">
+      <c r="G8" s="0" t="n">
         <v>8074</v>
       </c>
-      <c r="H8" t="n">
+      <c r="H8" s="0" t="n">
         <v>17901</v>
       </c>
-      <c r="I8" t="inlineStr">
+      <c r="I8" s="0" t="inlineStr">
         <is>
           <t>https://gmk-kiel.ru/catalog/oborudovanie/akusherstvo-i-ginekologiya</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" t="inlineStr">
+      <c r="A9" s="0" t="inlineStr">
         <is>
           <t>cordismed.ru</t>
         </is>
       </c>
-      <c r="B9" t="n">
+      <c r="B9" s="0" t="n">
         <v>5</v>
       </c>
-      <c r="C9" t="n">
+      <c r="C9" s="0" t="n">
         <v>1</v>
       </c>
-      <c r="D9" t="n">
+      <c r="D9" s="0" t="n">
         <v>3</v>
       </c>
-      <c r="E9" t="n">
+      <c r="E9" s="0" t="n">
         <v>486</v>
       </c>
-      <c r="F9" t="n">
+      <c r="F9" s="0" t="n">
         <v>2687</v>
       </c>
-      <c r="G9" t="n">
+      <c r="G9" s="0" t="n">
         <v>5627</v>
       </c>
-      <c r="H9" t="n">
+      <c r="H9" s="0" t="n">
         <v>18562</v>
       </c>
-      <c r="I9" t="inlineStr">
+      <c r="I9" s="0" t="inlineStr">
         <is>
           <t>https://cordismed.ru/ginekologiya</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" t="inlineStr">
+      <c r="A10" s="0" t="inlineStr">
         <is>
           <t>medrk.ru</t>
         </is>
       </c>
-      <c r="B10" t="n">
+      <c r="B10" s="0" t="n">
         <v>26</v>
       </c>
-      <c r="C10" t="n">
+      <c r="C10" s="0" t="n">
         <v>1</v>
       </c>
-      <c r="D10" t="n">
+      <c r="D10" s="0" t="n">
         <v>3</v>
       </c>
-      <c r="E10" t="n">
+      <c r="E10" s="0" t="n">
         <v>421</v>
       </c>
-      <c r="F10" t="n">
+      <c r="F10" s="0" t="n">
         <v>2671</v>
       </c>
-      <c r="G10" t="n">
+      <c r="G10" s="0" t="n">
         <v>6184</v>
       </c>
-      <c r="H10" t="n">
+      <c r="H10" s="0" t="n">
         <v>39793</v>
       </c>
-      <c r="I10" t="inlineStr">
+      <c r="I10" s="0" t="inlineStr">
         <is>
           <t>https://medrk.ru/shop/ginekologiya</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" t="inlineStr">
+      <c r="A11" s="0" t="inlineStr">
         <is>
           <t>sterimed.ru</t>
         </is>
       </c>
-      <c r="B11" t="n">
+      <c r="B11" s="0" t="n">
         <v>10</v>
       </c>
-      <c r="C11" t="n">
+      <c r="C11" s="0" t="n">
         <v>1</v>
       </c>
-      <c r="D11" t="n">
+      <c r="D11" s="0" t="n">
         <v>5</v>
       </c>
-      <c r="E11" t="n">
+      <c r="E11" s="0" t="n">
         <v>282</v>
       </c>
-      <c r="F11" t="n">
+      <c r="F11" s="0" t="n">
         <v>2595</v>
       </c>
-      <c r="G11" t="n">
+      <c r="G11" s="0" t="n">
         <v>5515</v>
       </c>
-      <c r="H11" t="n">
+      <c r="H11" s="0" t="n">
         <v>12635</v>
       </c>
-      <c r="I11" t="inlineStr">
+      <c r="I11" s="0" t="inlineStr">
         <is>
           <t>https://sterimed.ru/catalog/akusherstvo_i_ginekologiya</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" t="inlineStr">
+      <c r="A12" s="0" t="inlineStr">
         <is>
           <t>ivlabmed.ru</t>
         </is>
       </c>
-      <c r="B12" t="n">
+      <c r="B12" s="0" t="n">
         <v>12</v>
       </c>
-      <c r="C12" t="n">
+      <c r="C12" s="0" t="n">
         <v>1</v>
       </c>
-      <c r="D12" t="n">
+      <c r="D12" s="0" t="n">
         <v>3</v>
       </c>
-      <c r="E12" t="n">
+      <c r="E12" s="0" t="n">
         <v>233</v>
       </c>
-      <c r="F12" t="n">
+      <c r="F12" s="0" t="n">
         <v>2067</v>
       </c>
-      <c r="G12" t="n">
+      <c r="G12" s="0" t="n">
         <v>5313</v>
       </c>
-      <c r="H12" t="n">
+      <c r="H12" s="0" t="n">
         <v>17494</v>
       </c>
-      <c r="I12" t="inlineStr">
+      <c r="I12" s="0" t="inlineStr">
         <is>
           <t>https://ivlabmed.ru/catalog/ginekologiya</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" t="inlineStr">
+      <c r="A13" s="0" t="inlineStr">
         <is>
           <t>medbuy.ru</t>
         </is>
       </c>
-      <c r="B13" t="n">
+      <c r="B13" s="0" t="n">
         <v>15</v>
       </c>
-      <c r="C13" t="n">
+      <c r="C13" s="0" t="n">
         <v>1</v>
       </c>
-      <c r="D13" t="n">
+      <c r="D13" s="0" t="n">
         <v>3</v>
       </c>
-      <c r="E13" t="n">
+      <c r="E13" s="0" t="n">
         <v>352</v>
       </c>
-      <c r="F13" t="n">
+      <c r="F13" s="0" t="n">
         <v>1973</v>
       </c>
-      <c r="G13" t="n">
+      <c r="G13" s="0" t="n">
         <v>4266</v>
       </c>
-      <c r="H13" t="n">
+      <c r="H13" s="0" t="n">
         <v>19233</v>
       </c>
-      <c r="I13" t="inlineStr">
+      <c r="I13" s="0" t="inlineStr">
         <is>
           <t>https://medbuy.ru/catalog/akusherskoe-i-ginekologicheskoe-oborudovanie</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" t="inlineStr">
+      <c r="A14" s="0" t="inlineStr">
         <is>
           <t>medpribor.pro</t>
         </is>
       </c>
-      <c r="B14" t="n">
+      <c r="B14" s="0" t="n">
         <v>22</v>
       </c>
-      <c r="C14" t="n">
+      <c r="C14" s="0" t="n">
         <v>1</v>
       </c>
-      <c r="D14" t="n">
+      <c r="D14" s="0" t="n">
         <v>4</v>
       </c>
-      <c r="E14" t="n">
+      <c r="E14" s="0" t="n">
         <v>317</v>
       </c>
-      <c r="F14" t="n">
+      <c r="F14" s="0" t="n">
         <v>1826</v>
       </c>
-      <c r="G14" t="n">
+      <c r="G14" s="0" t="n">
         <v>3899</v>
       </c>
-      <c r="H14" t="n">
+      <c r="H14" s="0" t="n">
         <v>16120</v>
       </c>
-      <c r="I14" t="inlineStr">
+      <c r="I14" s="0" t="inlineStr">
         <is>
           <t>https://medpribor.pro/pc/lpu/gynecological</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" t="inlineStr">
+      <c r="A15" s="0" t="inlineStr">
         <is>
           <t>medeq.ru</t>
         </is>
       </c>
-      <c r="B15" t="n">
+      <c r="B15" s="0" t="n">
         <v>7</v>
       </c>
-      <c r="C15" t="n">
+      <c r="C15" s="0" t="n">
         <v>1</v>
       </c>
-      <c r="D15" t="n">
+      <c r="D15" s="0" t="n">
         <v>5</v>
       </c>
-      <c r="E15" t="n">
+      <c r="E15" s="0" t="n">
         <v>237</v>
       </c>
-      <c r="F15" t="n">
+      <c r="F15" s="0" t="n">
         <v>1795</v>
       </c>
-      <c r="G15" t="n">
+      <c r="G15" s="0" t="n">
         <v>5100</v>
       </c>
-      <c r="H15" t="n">
+      <c r="H15" s="0" t="n">
         <v>31655</v>
       </c>
-      <c r="I15" t="inlineStr">
+      <c r="I15" s="0" t="inlineStr">
         <is>
           <t>https://medeq.ru/store/akusherstvo-i-ginekologiya</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" t="inlineStr">
+      <c r="A16" s="0" t="inlineStr">
         <is>
           <t>farm-invest.ru</t>
         </is>
       </c>
-      <c r="B16" t="n">
+      <c r="B16" s="0" t="n">
         <v>16</v>
       </c>
-      <c r="C16" t="n">
+      <c r="C16" s="0" t="n">
         <v>1</v>
       </c>
-      <c r="D16" t="n">
+      <c r="D16" s="0" t="n">
         <v>2</v>
       </c>
-      <c r="E16" t="n">
+      <c r="E16" s="0" t="n">
         <v>274</v>
       </c>
-      <c r="F16" t="n">
+      <c r="F16" s="0" t="n">
         <v>1753</v>
       </c>
-      <c r="G16" t="n">
+      <c r="G16" s="0" t="n">
         <v>3889</v>
       </c>
-      <c r="H16" t="n">
+      <c r="H16" s="0" t="n">
         <v>14459</v>
       </c>
-      <c r="I16" t="inlineStr">
+      <c r="I16" s="0" t="inlineStr">
         <is>
           <t>https://farm-invest.ru/catalog/akusherstvo-i-ginekologiya</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" t="inlineStr">
+      <c r="A17" s="0" t="inlineStr">
         <is>
           <t>uromed-m.ru</t>
         </is>
       </c>
-      <c r="B17" t="n">
+      <c r="B17" s="0" t="n">
         <v>8</v>
       </c>
-      <c r="C17" t="n">
+      <c r="C17" s="0" t="n">
         <v>1</v>
       </c>
-      <c r="D17" t="n">
+      <c r="D17" s="0" t="n">
         <v>3</v>
       </c>
-      <c r="E17" t="n">
+      <c r="E17" s="0" t="n">
         <v>224</v>
       </c>
-      <c r="F17" t="n">
+      <c r="F17" s="0" t="n">
         <v>1209</v>
       </c>
-      <c r="G17" t="n">
+      <c r="G17" s="0" t="n">
         <v>2427</v>
       </c>
-      <c r="H17" t="n">
+      <c r="H17" s="0" t="n">
         <v>8364</v>
       </c>
-      <c r="I17" t="inlineStr">
+      <c r="I17" s="0" t="inlineStr">
         <is>
           <t>https://uromed-m.ru/ginekologicheskoe-oborudovanie</t>
         </is>
@@ -5281,6 +5590,858 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:K22"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="22" customWidth="1" style="354" min="1" max="1"/>
+    <col width="15" customWidth="1" style="354" min="2" max="2"/>
+    <col width="15" customWidth="1" style="354" min="3" max="3"/>
+    <col width="15" customWidth="1" style="354" min="4" max="4"/>
+    <col width="15" customWidth="1" style="354" min="5" max="5"/>
+    <col width="15" customWidth="1" style="354" min="6" max="6"/>
+    <col width="15" customWidth="1" style="354" min="7" max="7"/>
+    <col width="15" customWidth="1" style="354" min="8" max="8"/>
+    <col width="15" customWidth="1" style="354" min="9" max="9"/>
+    <col width="15" customWidth="1" style="354" min="10" max="10"/>
+    <col width="15" customWidth="1" style="354" min="11" max="11"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="48" customHeight="1" s="354">
+      <c r="A1" s="355" t="inlineStr">
+        <is>
+          <t>Домен</t>
+        </is>
+      </c>
+      <c r="B1" s="355" t="inlineStr">
+        <is>
+          <t>Трафик Яндекс</t>
+        </is>
+      </c>
+      <c r="C1" s="355" t="inlineStr">
+        <is>
+          <t>Трафик Google</t>
+        </is>
+      </c>
+      <c r="D1" s="355" t="inlineStr">
+        <is>
+          <t>Упоминания в Алисе</t>
+        </is>
+      </c>
+      <c r="E1" s="355" t="inlineStr">
+        <is>
+          <t>Ключей в топ 1 (Ya)</t>
+        </is>
+      </c>
+      <c r="F1" s="355" t="inlineStr">
+        <is>
+          <t>Ключей в топ 10 (Ya)</t>
+        </is>
+      </c>
+      <c r="G1" s="355" t="inlineStr">
+        <is>
+          <t>Ключей в топ 1 (G)</t>
+        </is>
+      </c>
+      <c r="H1" s="355" t="inlineStr">
+        <is>
+          <t>Ключей в топ 10 (G)</t>
+        </is>
+      </c>
+      <c r="I1" s="355" t="inlineStr">
+        <is>
+          <t>Ссылающихся IP</t>
+        </is>
+      </c>
+      <c r="J1" s="355" t="inlineStr">
+        <is>
+          <t>Исходящих доменов</t>
+        </is>
+      </c>
+      <c r="K1" s="355" t="inlineStr">
+        <is>
+          <t>Трафик в контексте (Ya), запросов</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>dealmed.ru</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>9945</v>
+      </c>
+      <c r="C2" t="n">
+        <v>3710</v>
+      </c>
+      <c r="D2" t="n">
+        <v>12572</v>
+      </c>
+      <c r="E2" t="n">
+        <v>8095</v>
+      </c>
+      <c r="F2" t="n">
+        <v>57843</v>
+      </c>
+      <c r="G2" t="n">
+        <v>2003</v>
+      </c>
+      <c r="H2" t="n">
+        <v>26401</v>
+      </c>
+      <c r="I2" t="n">
+        <v>1576</v>
+      </c>
+      <c r="J2" t="n">
+        <v>38</v>
+      </c>
+      <c r="K2" t="n">
+        <v>14338</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>medcomp.ru</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>2524</v>
+      </c>
+      <c r="C3" t="n">
+        <v>5921</v>
+      </c>
+      <c r="D3" t="n">
+        <v>6520</v>
+      </c>
+      <c r="E3" t="n">
+        <v>3014</v>
+      </c>
+      <c r="F3" t="n">
+        <v>18818</v>
+      </c>
+      <c r="G3" t="n">
+        <v>4610</v>
+      </c>
+      <c r="H3" t="n">
+        <v>20602</v>
+      </c>
+      <c r="I3" t="n">
+        <v>1266</v>
+      </c>
+      <c r="J3" t="n">
+        <v>15</v>
+      </c>
+      <c r="K3" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>medliga.ru</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>1671</v>
+      </c>
+      <c r="C4" t="n">
+        <v>1150</v>
+      </c>
+      <c r="D4" t="n">
+        <v>2702</v>
+      </c>
+      <c r="E4" t="n">
+        <v>4333</v>
+      </c>
+      <c r="F4" t="n">
+        <v>11043</v>
+      </c>
+      <c r="G4" t="n">
+        <v>912</v>
+      </c>
+      <c r="H4" t="n">
+        <v>7865</v>
+      </c>
+      <c r="I4" t="n">
+        <v>702</v>
+      </c>
+      <c r="J4" t="n">
+        <v>44</v>
+      </c>
+      <c r="K4" t="n">
+        <v>3053</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>almamed.su</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>902</v>
+      </c>
+      <c r="C5" t="n">
+        <v>985</v>
+      </c>
+      <c r="D5" t="n">
+        <v>6877</v>
+      </c>
+      <c r="E5" t="n">
+        <v>672</v>
+      </c>
+      <c r="F5" t="n">
+        <v>17379</v>
+      </c>
+      <c r="G5" t="n">
+        <v>445</v>
+      </c>
+      <c r="H5" t="n">
+        <v>11282</v>
+      </c>
+      <c r="I5" t="n">
+        <v>1150</v>
+      </c>
+      <c r="J5" t="n">
+        <v>41</v>
+      </c>
+      <c r="K5" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>medcub.ru</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>1066</v>
+      </c>
+      <c r="C6" t="n">
+        <v>243</v>
+      </c>
+      <c r="D6" t="n">
+        <v>4240</v>
+      </c>
+      <c r="E6" t="n">
+        <v>1297</v>
+      </c>
+      <c r="F6" t="n">
+        <v>10031</v>
+      </c>
+      <c r="G6" t="n">
+        <v>94</v>
+      </c>
+      <c r="H6" t="n">
+        <v>3521</v>
+      </c>
+      <c r="I6" t="n">
+        <v>255</v>
+      </c>
+      <c r="J6" t="n">
+        <v>6</v>
+      </c>
+      <c r="K6" t="n">
+        <v>6299</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>global-mt.ru</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>783</v>
+      </c>
+      <c r="C7" t="n">
+        <v>90</v>
+      </c>
+      <c r="D7" t="n">
+        <v>2054</v>
+      </c>
+      <c r="E7" t="n">
+        <v>1361</v>
+      </c>
+      <c r="F7" t="n">
+        <v>9645</v>
+      </c>
+      <c r="G7" t="n">
+        <v>42</v>
+      </c>
+      <c r="H7" t="n">
+        <v>1226</v>
+      </c>
+      <c r="I7" t="n">
+        <v>211</v>
+      </c>
+      <c r="J7" t="n">
+        <v>246</v>
+      </c>
+      <c r="K7" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>gmk-kiel.ru</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>804</v>
+      </c>
+      <c r="C8" t="n">
+        <v>323</v>
+      </c>
+      <c r="D8" t="n">
+        <v>2250</v>
+      </c>
+      <c r="E8" t="n">
+        <v>907</v>
+      </c>
+      <c r="F8" t="n">
+        <v>8074</v>
+      </c>
+      <c r="G8" t="n">
+        <v>75</v>
+      </c>
+      <c r="H8" t="n">
+        <v>2688</v>
+      </c>
+      <c r="I8" t="n">
+        <v>132</v>
+      </c>
+      <c r="J8" t="n">
+        <v>20</v>
+      </c>
+      <c r="K8" t="n">
+        <v>172</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>cordismed.ru</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>240</v>
+      </c>
+      <c r="C9" t="n">
+        <v>932</v>
+      </c>
+      <c r="D9" t="n">
+        <v>3242</v>
+      </c>
+      <c r="E9" t="n">
+        <v>486</v>
+      </c>
+      <c r="F9" t="n">
+        <v>5627</v>
+      </c>
+      <c r="G9" t="n">
+        <v>959</v>
+      </c>
+      <c r="H9" t="n">
+        <v>7004</v>
+      </c>
+      <c r="I9" t="n">
+        <v>401</v>
+      </c>
+      <c r="J9" t="n">
+        <v>24</v>
+      </c>
+      <c r="K9" t="n">
+        <v>286</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>medrk.ru</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>302</v>
+      </c>
+      <c r="C10" t="n">
+        <v>1198</v>
+      </c>
+      <c r="D10" t="n">
+        <v>3539</v>
+      </c>
+      <c r="E10" t="n">
+        <v>421</v>
+      </c>
+      <c r="F10" t="n">
+        <v>6184</v>
+      </c>
+      <c r="G10" t="n">
+        <v>671</v>
+      </c>
+      <c r="H10" t="n">
+        <v>9501</v>
+      </c>
+      <c r="I10" t="n">
+        <v>1354</v>
+      </c>
+      <c r="J10" t="n">
+        <v>24</v>
+      </c>
+      <c r="K10" t="n">
+        <v>888</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>sterimed.ru</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>440</v>
+      </c>
+      <c r="C11" t="n">
+        <v>153</v>
+      </c>
+      <c r="D11" t="n">
+        <v>1584</v>
+      </c>
+      <c r="E11" t="n">
+        <v>282</v>
+      </c>
+      <c r="F11" t="n">
+        <v>5515</v>
+      </c>
+      <c r="G11" t="n">
+        <v>77</v>
+      </c>
+      <c r="H11" t="n">
+        <v>2431</v>
+      </c>
+      <c r="I11" t="n">
+        <v>165</v>
+      </c>
+      <c r="J11" t="n">
+        <v>22</v>
+      </c>
+      <c r="K11" t="n">
+        <v>2142</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>ivlabmed.ru</t>
+        </is>
+      </c>
+      <c r="B12" t="n">
+        <v>239</v>
+      </c>
+      <c r="C12" t="n">
+        <v>23</v>
+      </c>
+      <c r="D12" t="n">
+        <v>1096</v>
+      </c>
+      <c r="E12" t="n">
+        <v>233</v>
+      </c>
+      <c r="F12" t="n">
+        <v>5313</v>
+      </c>
+      <c r="G12" t="n">
+        <v>23</v>
+      </c>
+      <c r="H12" t="n">
+        <v>363</v>
+      </c>
+      <c r="I12" t="n">
+        <v>172</v>
+      </c>
+      <c r="J12" t="n">
+        <v>11</v>
+      </c>
+      <c r="K12" t="n">
+        <v>376</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>medbuy.ru</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>236</v>
+      </c>
+      <c r="C13" t="n">
+        <v>57</v>
+      </c>
+      <c r="D13" t="n">
+        <v>636</v>
+      </c>
+      <c r="E13" t="n">
+        <v>352</v>
+      </c>
+      <c r="F13" t="n">
+        <v>4266</v>
+      </c>
+      <c r="G13" t="n">
+        <v>21</v>
+      </c>
+      <c r="H13" t="n">
+        <v>833</v>
+      </c>
+      <c r="I13" t="n">
+        <v>545</v>
+      </c>
+      <c r="J13" t="n">
+        <v>870</v>
+      </c>
+      <c r="K13" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>medpribor.pro</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>358</v>
+      </c>
+      <c r="C14" t="n">
+        <v>371</v>
+      </c>
+      <c r="D14" t="n">
+        <v>939</v>
+      </c>
+      <c r="E14" t="n">
+        <v>317</v>
+      </c>
+      <c r="F14" t="n">
+        <v>3899</v>
+      </c>
+      <c r="G14" t="n">
+        <v>182</v>
+      </c>
+      <c r="H14" t="n">
+        <v>2575</v>
+      </c>
+      <c r="I14" t="n">
+        <v>460</v>
+      </c>
+      <c r="J14" t="n">
+        <v>14</v>
+      </c>
+      <c r="K14" t="n">
+        <v>685</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>medeq.ru</t>
+        </is>
+      </c>
+      <c r="B15" t="n">
+        <v>419</v>
+      </c>
+      <c r="C15" t="n">
+        <v>245</v>
+      </c>
+      <c r="D15" t="n">
+        <v>1223</v>
+      </c>
+      <c r="E15" t="n">
+        <v>237</v>
+      </c>
+      <c r="F15" t="n">
+        <v>5100</v>
+      </c>
+      <c r="G15" t="n">
+        <v>138</v>
+      </c>
+      <c r="H15" t="n">
+        <v>2911</v>
+      </c>
+      <c r="I15" t="n">
+        <v>792</v>
+      </c>
+      <c r="J15" t="n">
+        <v>14</v>
+      </c>
+      <c r="K15" t="n">
+        <v>1287</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>farm-invest.ru</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>177</v>
+      </c>
+      <c r="C16" t="n">
+        <v>1141</v>
+      </c>
+      <c r="D16" t="n">
+        <v>1506</v>
+      </c>
+      <c r="E16" t="n">
+        <v>274</v>
+      </c>
+      <c r="F16" t="n">
+        <v>3889</v>
+      </c>
+      <c r="G16" t="n">
+        <v>570</v>
+      </c>
+      <c r="H16" t="n">
+        <v>5330</v>
+      </c>
+      <c r="I16" t="n">
+        <v>583</v>
+      </c>
+      <c r="J16" t="n">
+        <v>14</v>
+      </c>
+      <c r="K16" t="n">
+        <v>303</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>uromed-m.ru</t>
+        </is>
+      </c>
+      <c r="B17" t="n">
+        <v>237</v>
+      </c>
+      <c r="C17" t="n">
+        <v>1032</v>
+      </c>
+      <c r="D17" t="n">
+        <v>1492</v>
+      </c>
+      <c r="E17" t="n">
+        <v>224</v>
+      </c>
+      <c r="F17" t="n">
+        <v>2427</v>
+      </c>
+      <c r="G17" t="n">
+        <v>475</v>
+      </c>
+      <c r="H17" t="n">
+        <v>3955</v>
+      </c>
+      <c r="I17" t="n">
+        <v>348</v>
+      </c>
+      <c r="J17" t="n">
+        <v>43</v>
+      </c>
+      <c r="K17" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>intelmed.ru</t>
+        </is>
+      </c>
+      <c r="B18" t="n">
+        <v>28</v>
+      </c>
+      <c r="C18" t="n">
+        <v>531</v>
+      </c>
+      <c r="D18" t="n">
+        <v>699</v>
+      </c>
+      <c r="E18" t="n">
+        <v>53</v>
+      </c>
+      <c r="F18" t="n">
+        <v>644</v>
+      </c>
+      <c r="G18" t="n">
+        <v>182</v>
+      </c>
+      <c r="H18" t="n">
+        <v>2912</v>
+      </c>
+      <c r="I18" t="n">
+        <v>240</v>
+      </c>
+      <c r="J18" t="n">
+        <v>37</v>
+      </c>
+      <c r="K18" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>kriptomed.ru</t>
+        </is>
+      </c>
+      <c r="B19" t="n">
+        <v>194</v>
+      </c>
+      <c r="C19" t="n">
+        <v>423</v>
+      </c>
+      <c r="D19" t="n">
+        <v>870</v>
+      </c>
+      <c r="E19" t="n">
+        <v>250</v>
+      </c>
+      <c r="F19" t="n">
+        <v>2137</v>
+      </c>
+      <c r="G19" t="n">
+        <v>311</v>
+      </c>
+      <c r="H19" t="n">
+        <v>2020</v>
+      </c>
+      <c r="I19" t="n">
+        <v>156</v>
+      </c>
+      <c r="J19" t="n">
+        <v>45</v>
+      </c>
+      <c r="K19" t="n">
+        <v>5092</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>fotek.ru</t>
+        </is>
+      </c>
+      <c r="B20" t="n">
+        <v>55</v>
+      </c>
+      <c r="C20" t="n">
+        <v>110</v>
+      </c>
+      <c r="D20" t="n">
+        <v>575</v>
+      </c>
+      <c r="E20" t="n">
+        <v>73</v>
+      </c>
+      <c r="F20" t="n">
+        <v>734</v>
+      </c>
+      <c r="G20" t="n">
+        <v>139</v>
+      </c>
+      <c r="H20" t="n">
+        <v>790</v>
+      </c>
+      <c r="I20" t="n">
+        <v>601</v>
+      </c>
+      <c r="J20" t="n">
+        <v>33</v>
+      </c>
+      <c r="K20" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>medgrade.pro</t>
+        </is>
+      </c>
+      <c r="B21" t="n">
+        <v>188</v>
+      </c>
+      <c r="C21" t="n">
+        <v>155</v>
+      </c>
+      <c r="D21" t="n">
+        <v>3483</v>
+      </c>
+      <c r="E21" t="n">
+        <v>287</v>
+      </c>
+      <c r="F21" t="n">
+        <v>2044</v>
+      </c>
+      <c r="G21" t="n">
+        <v>133</v>
+      </c>
+      <c r="H21" t="n">
+        <v>2183</v>
+      </c>
+      <c r="I21" t="n">
+        <v>152</v>
+      </c>
+      <c r="J21" t="n">
+        <v>112</v>
+      </c>
+      <c r="K21" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>reiginmed.ru</t>
+        </is>
+      </c>
+      <c r="B22" t="n">
+        <v>0</v>
+      </c>
+      <c r="D22" t="n">
+        <v>0</v>
+      </c>
+      <c r="E22" t="n">
+        <v>0</v>
+      </c>
+      <c r="F22" t="n">
+        <v>0</v>
+      </c>
+      <c r="I22" t="n">
+        <v>0</v>
+      </c>
+      <c r="J22" t="n">
+        <v>5</v>
+      </c>
+      <c r="K22" t="n">
+        <v>0</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
@@ -5493,7 +6654,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
@@ -5572,7 +6733,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
@@ -5672,7 +6833,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>

</xml_diff>

<commit_message>
Add pr-cy metrics: index, age, IKS, reviews, Ahrefs DR
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01GGxzKXyeNbw77cRhpGHusQ
</commit_message>
<xml_diff>
--- a/out/analiz_konkurentov_reiginmed.xlsx
+++ b/out/analiz_konkurentov_reiginmed.xlsx
@@ -3185,11 +3185,21 @@
         <f>"https://a.pr-cy.ru/"&amp;IF(ISERROR(FIND("//www.",B2)),MID(B2,FIND(":",B2,4)+3,FIND("/",B2,9)-FIND(":",B2,4)-3),MID(B2,FIND(":",B2,4)+7,FIND("/",B2,9)-FIND(":",B2,4)-7))&amp;"/"</f>
         <v/>
       </c>
-      <c r="E2" s="33" t="n"/>
-      <c r="F2" s="34" t="n"/>
-      <c r="G2" s="35" t="n"/>
-      <c r="H2" s="36" t="n"/>
-      <c r="I2" s="37" t="n"/>
+      <c r="E2" s="33" t="n">
+        <v>44000</v>
+      </c>
+      <c r="F2" s="34" t="n">
+        <v>118000</v>
+      </c>
+      <c r="G2" s="35" t="n">
+        <v>16.1</v>
+      </c>
+      <c r="H2" s="36" t="n">
+        <v>1170</v>
+      </c>
+      <c r="I2" s="37" t="n">
+        <v>82</v>
+      </c>
       <c r="J2" s="38" t="n">
         <v>895089</v>
       </c>
@@ -3229,7 +3239,7 @@
         <v/>
       </c>
       <c r="W2" s="50" t="n">
-        <v>35</v>
+        <v>58</v>
       </c>
       <c r="X2" s="64" t="inlineStr">
         <is>
@@ -3255,11 +3265,21 @@
         <f>"https://a.pr-cy.ru/"&amp;IF(ISERROR(FIND("//www.",B3)),MID(B3,FIND(":",B3,4)+3,FIND("/",B3,9)-FIND(":",B3,4)-3),MID(B3,FIND(":",B3,4)+7,FIND("/",B3,9)-FIND(":",B3,4)-7))&amp;"/"</f>
         <v/>
       </c>
-      <c r="E3" s="33" t="n"/>
-      <c r="F3" s="34" t="n"/>
-      <c r="G3" s="35" t="n"/>
-      <c r="H3" s="36" t="n"/>
-      <c r="I3" s="37" t="n"/>
+      <c r="E3" s="33" t="n">
+        <v>4000</v>
+      </c>
+      <c r="F3" s="34" t="n">
+        <v>27100</v>
+      </c>
+      <c r="G3" s="35" t="n">
+        <v>25.9</v>
+      </c>
+      <c r="H3" s="36" t="n">
+        <v>1170</v>
+      </c>
+      <c r="I3" s="37" t="n">
+        <v>49</v>
+      </c>
       <c r="J3" s="38" t="n">
         <v>227153</v>
       </c>
@@ -3299,7 +3319,7 @@
         <v/>
       </c>
       <c r="W3" s="50" t="n">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="X3" s="64" t="inlineStr">
         <is>
@@ -3325,11 +3345,21 @@
         <f>"https://a.pr-cy.ru/"&amp;IF(ISERROR(FIND("//www.",B4)),MID(B4,FIND(":",B4,4)+3,FIND("/",B4,9)-FIND(":",B4,4)-3),MID(B4,FIND(":",B4,4)+7,FIND("/",B4,9)-FIND(":",B4,4)-7))&amp;"/"</f>
         <v/>
       </c>
-      <c r="E4" s="33" t="n"/>
-      <c r="F4" s="34" t="n"/>
-      <c r="G4" s="35" t="n"/>
-      <c r="H4" s="36" t="n"/>
-      <c r="I4" s="37" t="n"/>
+      <c r="E4" s="33" t="n">
+        <v>36000</v>
+      </c>
+      <c r="F4" s="34" t="n">
+        <v>10200</v>
+      </c>
+      <c r="G4" s="35" t="n">
+        <v>6.3</v>
+      </c>
+      <c r="H4" s="36" t="n">
+        <v>410</v>
+      </c>
+      <c r="I4" s="37" t="n">
+        <v>24</v>
+      </c>
       <c r="J4" s="38" t="n">
         <v>150351</v>
       </c>
@@ -3369,7 +3399,7 @@
         <v/>
       </c>
       <c r="W4" s="50" t="n">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="X4" s="64" t="inlineStr">
         <is>
@@ -3395,11 +3425,21 @@
         <f>"https://a.pr-cy.ru/"&amp;IF(ISERROR(FIND("//www.",B5)),MID(B5,FIND(":",B5,4)+3,FIND("/",B5,9)-FIND(":",B5,4)-3),MID(B5,FIND(":",B5,4)+7,FIND("/",B5,9)-FIND(":",B5,4)-7))&amp;"/"</f>
         <v/>
       </c>
-      <c r="E5" s="33" t="n"/>
-      <c r="F5" s="34" t="n"/>
-      <c r="G5" s="35" t="n"/>
-      <c r="H5" s="36" t="n"/>
-      <c r="I5" s="37" t="n"/>
+      <c r="E5" s="33" t="n">
+        <v>35000</v>
+      </c>
+      <c r="F5" s="34" t="n">
+        <v>46700</v>
+      </c>
+      <c r="G5" s="35" t="n">
+        <v>11</v>
+      </c>
+      <c r="H5" s="36" t="n">
+        <v>370</v>
+      </c>
+      <c r="I5" s="37" t="n">
+        <v>22</v>
+      </c>
       <c r="J5" s="38" t="n">
         <v>81164</v>
       </c>
@@ -3439,7 +3479,7 @@
         <v/>
       </c>
       <c r="W5" s="50" t="n">
-        <v>29</v>
+        <v>25</v>
       </c>
       <c r="X5" s="64" t="inlineStr">
         <is>
@@ -3465,11 +3505,21 @@
         <f>"https://a.pr-cy.ru/"&amp;IF(ISERROR(FIND("//www.",B6)),MID(B6,FIND(":",B6,4)+3,FIND("/",B6,9)-FIND(":",B6,4)-3),MID(B6,FIND(":",B6,4)+7,FIND("/",B6,9)-FIND(":",B6,4)-7))&amp;"/"</f>
         <v/>
       </c>
-      <c r="E6" s="33" t="n"/>
-      <c r="F6" s="34" t="n"/>
-      <c r="G6" s="35" t="n"/>
-      <c r="H6" s="36" t="n"/>
-      <c r="I6" s="37" t="n"/>
+      <c r="E6" s="33" t="n">
+        <v>31000</v>
+      </c>
+      <c r="F6" s="34" t="n">
+        <v>173000</v>
+      </c>
+      <c r="G6" s="35" t="n">
+        <v>4.1</v>
+      </c>
+      <c r="H6" s="36" t="n">
+        <v>300</v>
+      </c>
+      <c r="I6" s="37" t="n">
+        <v>85</v>
+      </c>
       <c r="J6" s="38" t="n">
         <v>95974</v>
       </c>
@@ -3509,7 +3559,7 @@
         <v/>
       </c>
       <c r="W6" s="50" t="n">
-        <v>25</v>
+        <v>5</v>
       </c>
       <c r="X6" s="64" t="inlineStr">
         <is>
@@ -3535,11 +3585,21 @@
         <f>"https://a.pr-cy.ru/"&amp;IF(ISERROR(FIND("//www.",B7)),MID(B7,FIND(":",B7,4)+3,FIND("/",B7,9)-FIND(":",B7,4)-3),MID(B7,FIND(":",B7,4)+7,FIND("/",B7,9)-FIND(":",B7,4)-7))&amp;"/"</f>
         <v/>
       </c>
-      <c r="E7" s="33" t="n"/>
-      <c r="F7" s="34" t="n"/>
-      <c r="G7" s="35" t="n"/>
-      <c r="H7" s="36" t="n"/>
-      <c r="I7" s="37" t="n"/>
+      <c r="E7" s="33" t="n">
+        <v>12000</v>
+      </c>
+      <c r="F7" s="34" t="n">
+        <v>10400</v>
+      </c>
+      <c r="G7" s="35" t="n">
+        <v>10.1</v>
+      </c>
+      <c r="H7" s="36" t="n">
+        <v>240</v>
+      </c>
+      <c r="I7" s="37" t="n">
+        <v>1</v>
+      </c>
       <c r="J7" s="38" t="n">
         <v>70465</v>
       </c>
@@ -3579,7 +3639,7 @@
         <v/>
       </c>
       <c r="W7" s="50" t="n">
-        <v>35</v>
+        <v>15</v>
       </c>
       <c r="X7" s="64" t="inlineStr">
         <is>
@@ -3605,11 +3665,21 @@
         <f>"https://a.pr-cy.ru/"&amp;IF(ISERROR(FIND("//www.",B8)),MID(B8,FIND(":",B8,4)+3,FIND("/",B8,9)-FIND(":",B8,4)-3),MID(B8,FIND(":",B8,4)+7,FIND("/",B8,9)-FIND(":",B8,4)-7))&amp;"/"</f>
         <v/>
       </c>
-      <c r="E8" s="33" t="n"/>
-      <c r="F8" s="34" t="n"/>
-      <c r="G8" s="35" t="n"/>
-      <c r="H8" s="36" t="n"/>
-      <c r="I8" s="37" t="n"/>
+      <c r="E8" s="33" t="n">
+        <v>5000</v>
+      </c>
+      <c r="F8" s="34" t="n">
+        <v>5190</v>
+      </c>
+      <c r="G8" s="35" t="n">
+        <v>6.9</v>
+      </c>
+      <c r="H8" s="36" t="n">
+        <v>170</v>
+      </c>
+      <c r="I8" s="37" t="n">
+        <v>3</v>
+      </c>
       <c r="J8" s="38" t="n">
         <v>72336</v>
       </c>
@@ -3649,7 +3719,7 @@
         <v/>
       </c>
       <c r="W8" s="50" t="n">
-        <v>31</v>
+        <v>2</v>
       </c>
       <c r="X8" s="64" t="inlineStr">
         <is>
@@ -3675,11 +3745,21 @@
         <f>"https://a.pr-cy.ru/"&amp;IF(ISERROR(FIND("//www.",B9)),MID(B9,FIND(":",B9,4)+3,FIND("/",B9,9)-FIND(":",B9,4)-3),MID(B9,FIND(":",B9,4)+7,FIND("/",B9,9)-FIND(":",B9,4)-7))&amp;"/"</f>
         <v/>
       </c>
-      <c r="E9" s="33" t="n"/>
-      <c r="F9" s="34" t="n"/>
-      <c r="G9" s="35" t="n"/>
-      <c r="H9" s="36" t="n"/>
-      <c r="I9" s="37" t="n"/>
+      <c r="E9" s="33" t="n">
+        <v>4000</v>
+      </c>
+      <c r="F9" s="34" t="n">
+        <v>5440</v>
+      </c>
+      <c r="G9" s="35" t="n">
+        <v>8.5</v>
+      </c>
+      <c r="H9" s="36" t="n">
+        <v>230</v>
+      </c>
+      <c r="I9" s="37" t="n">
+        <v>3</v>
+      </c>
       <c r="J9" s="38" t="n">
         <v>21573</v>
       </c>
@@ -3719,7 +3799,7 @@
         <v/>
       </c>
       <c r="W9" s="50" t="n">
-        <v>31</v>
+        <v>22</v>
       </c>
       <c r="X9" s="262" t="inlineStr">
         <is>
@@ -3745,11 +3825,21 @@
         <f>"https://a.pr-cy.ru/"&amp;IF(ISERROR(FIND("//www.",B10)),MID(B10,FIND(":",B10,4)+3,FIND("/",B10,9)-FIND(":",B10,4)-3),MID(B10,FIND(":",B10,4)+7,FIND("/",B10,9)-FIND(":",B10,4)-7))&amp;"/"</f>
         <v/>
       </c>
-      <c r="E10" s="33" t="n"/>
-      <c r="F10" s="34" t="n"/>
-      <c r="G10" s="35" t="n"/>
-      <c r="H10" s="36" t="n"/>
-      <c r="I10" s="37" t="n"/>
+      <c r="E10" s="33" t="n">
+        <v>12000</v>
+      </c>
+      <c r="F10" s="34" t="n">
+        <v>12600</v>
+      </c>
+      <c r="G10" s="35" t="n">
+        <v>23.8</v>
+      </c>
+      <c r="H10" s="36" t="n">
+        <v>430</v>
+      </c>
+      <c r="I10" s="37" t="n">
+        <v>18</v>
+      </c>
       <c r="J10" s="38" t="n">
         <v>27185</v>
       </c>
@@ -3789,7 +3879,7 @@
         <v/>
       </c>
       <c r="W10" s="50" t="n">
-        <v>33</v>
+        <v>23</v>
       </c>
       <c r="X10" s="262" t="inlineStr">
         <is>
@@ -3815,11 +3905,21 @@
         <f>"https://a.pr-cy.ru/"&amp;IF(ISERROR(FIND("//www.",B11)),MID(B11,FIND(":",B11,4)+3,FIND("/",B11,9)-FIND(":",B11,4)-3),MID(B11,FIND(":",B11,4)+7,FIND("/",B11,9)-FIND(":",B11,4)-7))&amp;"/"</f>
         <v/>
       </c>
-      <c r="E11" s="33" t="n"/>
-      <c r="F11" s="34" t="n"/>
-      <c r="G11" s="35" t="n"/>
-      <c r="H11" s="36" t="n"/>
-      <c r="I11" s="37" t="n"/>
+      <c r="E11" s="33" t="n">
+        <v>3000</v>
+      </c>
+      <c r="F11" s="34" t="n">
+        <v>10500</v>
+      </c>
+      <c r="G11" s="35" t="n">
+        <v>19.4</v>
+      </c>
+      <c r="H11" s="36" t="n">
+        <v>330</v>
+      </c>
+      <c r="I11" s="37" t="n">
+        <v>7</v>
+      </c>
       <c r="J11" s="38" t="n">
         <v>39613</v>
       </c>
@@ -3859,7 +3959,7 @@
         <v/>
       </c>
       <c r="W11" s="50" t="n">
-        <v>27</v>
+        <v>21</v>
       </c>
       <c r="X11" s="262" t="inlineStr">
         <is>
@@ -3885,11 +3985,21 @@
         <f>"https://a.pr-cy.ru/"&amp;IF(ISERROR(FIND("//www.",B12)),MID(B12,FIND(":",B12,4)+3,FIND("/",B12,9)-FIND(":",B12,4)-3),MID(B12,FIND(":",B12,4)+7,FIND("/",B12,9)-FIND(":",B12,4)-7))&amp;"/"</f>
         <v/>
       </c>
-      <c r="E12" s="33" t="n"/>
-      <c r="F12" s="34" t="n"/>
-      <c r="G12" s="35" t="n"/>
-      <c r="H12" s="36" t="n"/>
-      <c r="I12" s="37" t="n"/>
+      <c r="E12" s="33" t="n">
+        <v>21000</v>
+      </c>
+      <c r="F12" s="34" t="n">
+        <v>2960</v>
+      </c>
+      <c r="G12" s="35" t="n">
+        <v>8.800000000000001</v>
+      </c>
+      <c r="H12" s="36" t="n">
+        <v>240</v>
+      </c>
+      <c r="I12" s="37" t="n">
+        <v>2</v>
+      </c>
       <c r="J12" s="38" t="n">
         <v>21474</v>
       </c>
@@ -3929,7 +4039,7 @@
         <v/>
       </c>
       <c r="W12" s="50" t="n">
-        <v>28</v>
+        <v>11</v>
       </c>
       <c r="X12" s="262" t="inlineStr">
         <is>
@@ -3955,11 +4065,21 @@
         <f>"https://a.pr-cy.ru/"&amp;IF(ISERROR(FIND("//www.",B13)),MID(B13,FIND(":",B13,4)+3,FIND("/",B13,9)-FIND(":",B13,4)-3),MID(B13,FIND(":",B13,4)+7,FIND("/",B13,9)-FIND(":",B13,4)-7))&amp;"/"</f>
         <v/>
       </c>
-      <c r="E13" s="33" t="n"/>
-      <c r="F13" s="34" t="n"/>
-      <c r="G13" s="35" t="n"/>
-      <c r="H13" s="36" t="n"/>
-      <c r="I13" s="37" t="n"/>
+      <c r="E13" s="33" t="n">
+        <v>9000</v>
+      </c>
+      <c r="F13" s="34" t="n">
+        <v>7120</v>
+      </c>
+      <c r="G13" s="35" t="n">
+        <v>15.3</v>
+      </c>
+      <c r="H13" s="36" t="n">
+        <v>210</v>
+      </c>
+      <c r="I13" s="37" t="n">
+        <v>23</v>
+      </c>
       <c r="J13" s="38" t="n">
         <v>21260</v>
       </c>
@@ -3999,7 +4119,7 @@
         <v/>
       </c>
       <c r="W13" s="50" t="n">
-        <v>22</v>
+        <v>32</v>
       </c>
       <c r="X13" s="262" t="inlineStr">
         <is>
@@ -4025,11 +4145,21 @@
         <f>"https://a.pr-cy.ru/"&amp;IF(ISERROR(FIND("//www.",B14)),MID(B14,FIND(":",B14,4)+3,FIND("/",B14,9)-FIND(":",B14,4)-3),MID(B14,FIND(":",B14,4)+7,FIND("/",B14,9)-FIND(":",B14,4)-7))&amp;"/"</f>
         <v/>
       </c>
-      <c r="E14" s="33" t="n"/>
-      <c r="F14" s="34" t="n"/>
-      <c r="G14" s="35" t="n"/>
-      <c r="H14" s="36" t="n"/>
-      <c r="I14" s="37" t="n"/>
+      <c r="E14" s="33" t="n">
+        <v>4000</v>
+      </c>
+      <c r="F14" s="34" t="n">
+        <v>4290</v>
+      </c>
+      <c r="G14" s="35" t="n">
+        <v>8.800000000000001</v>
+      </c>
+      <c r="H14" s="36" t="n">
+        <v>320</v>
+      </c>
+      <c r="I14" s="37" t="n">
+        <v>5</v>
+      </c>
       <c r="J14" s="38" t="n">
         <v>32260</v>
       </c>
@@ -4069,7 +4199,7 @@
         <v/>
       </c>
       <c r="W14" s="50" t="n">
-        <v>32</v>
+        <v>56</v>
       </c>
       <c r="X14" s="262" t="inlineStr">
         <is>
@@ -4095,11 +4225,21 @@
         <f>"https://a.pr-cy.ru/"&amp;IF(ISERROR(FIND("//www.",B15)),MID(B15,FIND(":",B15,4)+3,FIND("/",B15,9)-FIND(":",B15,4)-3),MID(B15,FIND(":",B15,4)+7,FIND("/",B15,9)-FIND(":",B15,4)-7))&amp;"/"</f>
         <v/>
       </c>
-      <c r="E15" s="33" t="n"/>
-      <c r="F15" s="34" t="n"/>
-      <c r="G15" s="35" t="n"/>
-      <c r="H15" s="36" t="n"/>
-      <c r="I15" s="37" t="n"/>
+      <c r="E15" s="33" t="n">
+        <v>13000</v>
+      </c>
+      <c r="F15" s="34" t="n">
+        <v>15300</v>
+      </c>
+      <c r="G15" s="35" t="n">
+        <v>9.9</v>
+      </c>
+      <c r="H15" s="36" t="n">
+        <v>300</v>
+      </c>
+      <c r="I15" s="37" t="n">
+        <v>21</v>
+      </c>
       <c r="J15" s="38" t="n">
         <v>37751</v>
       </c>
@@ -4139,7 +4279,7 @@
         <v/>
       </c>
       <c r="W15" s="50" t="n">
-        <v>29</v>
+        <v>34</v>
       </c>
       <c r="X15" s="262" t="inlineStr">
         <is>
@@ -4165,11 +4305,21 @@
         <f>"https://a.pr-cy.ru/"&amp;IF(ISERROR(FIND("//www.",B16)),MID(B16,FIND(":",B16,4)+3,FIND("/",B16,9)-FIND(":",B16,4)-3),MID(B16,FIND(":",B16,4)+7,FIND("/",B16,9)-FIND(":",B16,4)-7))&amp;"/"</f>
         <v/>
       </c>
-      <c r="E16" s="33" t="n"/>
-      <c r="F16" s="34" t="n"/>
-      <c r="G16" s="35" t="n"/>
-      <c r="H16" s="36" t="n"/>
-      <c r="I16" s="37" t="n"/>
+      <c r="E16" s="33" t="n">
+        <v>2000</v>
+      </c>
+      <c r="F16" s="34" t="n">
+        <v>100</v>
+      </c>
+      <c r="G16" s="35" t="n">
+        <v>22.2</v>
+      </c>
+      <c r="H16" s="36" t="n">
+        <v>320</v>
+      </c>
+      <c r="I16" s="37" t="n">
+        <v>4</v>
+      </c>
       <c r="J16" s="38" t="n">
         <v>15955</v>
       </c>
@@ -4209,7 +4359,7 @@
         <v/>
       </c>
       <c r="W16" s="50" t="n">
-        <v>31</v>
+        <v>14</v>
       </c>
       <c r="X16" s="262" t="inlineStr">
         <is>
@@ -4235,11 +4385,21 @@
         <f>"https://a.pr-cy.ru/"&amp;IF(ISERROR(FIND("//www.",B17)),MID(B17,FIND(":",B17,4)+3,FIND("/",B17,9)-FIND(":",B17,4)-3),MID(B17,FIND(":",B17,4)+7,FIND("/",B17,9)-FIND(":",B17,4)-7))&amp;"/"</f>
         <v/>
       </c>
-      <c r="E17" s="33" t="n"/>
-      <c r="F17" s="34" t="n"/>
-      <c r="G17" s="35" t="n"/>
-      <c r="H17" s="36" t="n"/>
-      <c r="I17" s="37" t="n"/>
+      <c r="E17" s="33" t="n">
+        <v>2000</v>
+      </c>
+      <c r="F17" s="34" t="n">
+        <v>2020</v>
+      </c>
+      <c r="G17" s="35" t="n">
+        <v>20.3</v>
+      </c>
+      <c r="H17" s="36" t="n">
+        <v>230</v>
+      </c>
+      <c r="I17" s="37" t="n">
+        <v>1</v>
+      </c>
       <c r="J17" s="38" t="n">
         <v>21301</v>
       </c>
@@ -4279,7 +4439,7 @@
         <v/>
       </c>
       <c r="W17" s="50" t="n">
-        <v>34</v>
+        <v>18</v>
       </c>
       <c r="X17" s="262" t="inlineStr">
         <is>
@@ -4305,11 +4465,21 @@
         <f>"https://a.pr-cy.ru/"&amp;IF(ISERROR(FIND("//www.",B18)),MID(B18,FIND(":",B18,4)+3,FIND("/",B18,9)-FIND(":",B18,4)-3),MID(B18,FIND(":",B18,4)+7,FIND("/",B18,9)-FIND(":",B18,4)-7))&amp;"/"</f>
         <v/>
       </c>
-      <c r="E18" s="33" t="n"/>
-      <c r="F18" s="34" t="n"/>
-      <c r="G18" s="35" t="n"/>
-      <c r="H18" s="36" t="n"/>
-      <c r="I18" s="37" t="n"/>
+      <c r="E18" s="33" t="n">
+        <v>778</v>
+      </c>
+      <c r="F18" s="34" t="n">
+        <v>1850</v>
+      </c>
+      <c r="G18" s="35" t="n">
+        <v>26.6</v>
+      </c>
+      <c r="H18" s="36" t="n">
+        <v>200</v>
+      </c>
+      <c r="I18" s="37" t="n">
+        <v>0</v>
+      </c>
       <c r="J18" s="38" t="n">
         <v>2545</v>
       </c>
@@ -4349,7 +4519,7 @@
         <v/>
       </c>
       <c r="W18" s="50" t="n">
-        <v>24</v>
+        <v>28</v>
       </c>
       <c r="X18" s="262" t="inlineStr">
         <is>
@@ -4375,11 +4545,21 @@
         <f>"https://a.pr-cy.ru/"&amp;IF(ISERROR(FIND("//www.",B19)),MID(B19,FIND(":",B19,4)+3,FIND("/",B19,9)-FIND(":",B19,4)-3),MID(B19,FIND(":",B19,4)+7,FIND("/",B19,9)-FIND(":",B19,4)-7))&amp;"/"</f>
         <v/>
       </c>
-      <c r="E19" s="33" t="n"/>
-      <c r="F19" s="34" t="n"/>
-      <c r="G19" s="35" t="n"/>
-      <c r="H19" s="36" t="n"/>
-      <c r="I19" s="37" t="n"/>
+      <c r="E19" s="33" t="n">
+        <v>3000</v>
+      </c>
+      <c r="F19" s="34" t="n">
+        <v>6200</v>
+      </c>
+      <c r="G19" s="35" t="n">
+        <v>19.8</v>
+      </c>
+      <c r="H19" s="36" t="n">
+        <v>340</v>
+      </c>
+      <c r="I19" s="37" t="n">
+        <v>4</v>
+      </c>
       <c r="J19" s="38" t="n">
         <v>17437</v>
       </c>
@@ -4419,7 +4599,7 @@
         <v/>
       </c>
       <c r="W19" s="50" t="n">
-        <v>26</v>
+        <v>12</v>
       </c>
       <c r="X19" s="262" t="inlineStr">
         <is>
@@ -4445,11 +4625,21 @@
         <f>"https://a.pr-cy.ru/"&amp;IF(ISERROR(FIND("//www.",B20)),MID(B20,FIND(":",B20,4)+3,FIND("/",B20,9)-FIND(":",B20,4)-3),MID(B20,FIND(":",B20,4)+7,FIND("/",B20,9)-FIND(":",B20,4)-7))&amp;"/"</f>
         <v/>
       </c>
-      <c r="E20" s="33" t="n"/>
-      <c r="F20" s="34" t="n"/>
-      <c r="G20" s="35" t="n"/>
-      <c r="H20" s="36" t="n"/>
-      <c r="I20" s="37" t="n"/>
+      <c r="E20" s="33" t="n">
+        <v>4000</v>
+      </c>
+      <c r="F20" s="34" t="n">
+        <v>2620</v>
+      </c>
+      <c r="G20" s="35" t="n">
+        <v>25.2</v>
+      </c>
+      <c r="H20" s="36" t="n">
+        <v>300</v>
+      </c>
+      <c r="I20" s="37" t="n">
+        <v>3</v>
+      </c>
       <c r="J20" s="38" t="n">
         <v>4906</v>
       </c>
@@ -4515,11 +4705,21 @@
         <f>"https://a.pr-cy.ru/"&amp;IF(ISERROR(FIND("//www.",B21)),MID(B21,FIND(":",B21,4)+3,FIND("/",B21,9)-FIND(":",B21,4)-3),MID(B21,FIND(":",B21,4)+7,FIND("/",B21,9)-FIND(":",B21,4)-7))&amp;"/"</f>
         <v/>
       </c>
-      <c r="E21" s="33" t="n"/>
-      <c r="F21" s="34" t="n"/>
-      <c r="G21" s="35" t="n"/>
-      <c r="H21" s="36" t="n"/>
-      <c r="I21" s="37" t="n"/>
+      <c r="E21" s="33" t="n">
+        <v>1000</v>
+      </c>
+      <c r="F21" s="34" t="n">
+        <v>1100</v>
+      </c>
+      <c r="G21" s="35" t="n">
+        <v>9</v>
+      </c>
+      <c r="H21" s="36" t="n">
+        <v>150</v>
+      </c>
+      <c r="I21" s="37" t="n">
+        <v>10</v>
+      </c>
       <c r="J21" s="38" t="n">
         <v>16895</v>
       </c>
@@ -4669,11 +4869,21 @@
         <f>"https://a.pr-cy.ru/"&amp;IF(ISERROR(FIND("//www.",B23)),MID(B23,FIND(":",B23,4)+3,FIND("/",B23,9)-FIND(":",B23,4)-3),MID(B23,FIND(":",B23,4)+7,FIND("/",B23,9)-FIND(":",B23,4)-7))&amp;"/"</f>
         <v/>
       </c>
-      <c r="E23" s="343" t="n"/>
-      <c r="F23" s="344" t="n"/>
-      <c r="G23" s="345" t="n"/>
-      <c r="H23" s="344" t="n"/>
-      <c r="I23" s="346" t="n"/>
+      <c r="E23" s="343" t="n">
+        <v>1</v>
+      </c>
+      <c r="F23" s="344" t="n">
+        <v>0</v>
+      </c>
+      <c r="G23" s="345" t="n">
+        <v>1.2</v>
+      </c>
+      <c r="H23" s="344" t="n">
+        <v>10</v>
+      </c>
+      <c r="I23" s="346" t="n">
+        <v>0</v>
+      </c>
       <c r="J23" s="348" t="n">
         <v>0</v>
       </c>
@@ -5595,7 +5805,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K22"/>
+  <dimension ref="A1:P22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" style="354" min="1" max="1"/>
@@ -5609,6 +5819,11 @@
     <col width="15" customWidth="1" style="354" min="9" max="9"/>
     <col width="15" customWidth="1" style="354" min="10" max="10"/>
     <col width="15" customWidth="1" style="354" min="11" max="11"/>
+    <col width="15" customWidth="1" style="354" min="12" max="12"/>
+    <col width="15" customWidth="1" style="354" min="13" max="13"/>
+    <col width="15" customWidth="1" style="354" min="14" max="14"/>
+    <col width="15" customWidth="1" style="354" min="15" max="15"/>
+    <col width="15" customWidth="1" style="354" min="16" max="16"/>
   </cols>
   <sheetData>
     <row r="1" ht="48" customHeight="1" s="354">
@@ -5667,773 +5882,1188 @@
           <t>Трафик в контексте (Ya), запросов</t>
         </is>
       </c>
+      <c r="L1" s="355" t="inlineStr">
+        <is>
+          <t>Посетители в месяц (pr-cy)</t>
+        </is>
+      </c>
+      <c r="M1" s="355" t="inlineStr">
+        <is>
+          <t>Поисковые системы, %</t>
+        </is>
+      </c>
+      <c r="N1" s="355" t="inlineStr">
+        <is>
+          <t>Отказы, %</t>
+        </is>
+      </c>
+      <c r="O1" s="355" t="inlineStr">
+        <is>
+          <t>Категория (pr-cy)</t>
+        </is>
+      </c>
+      <c r="P1" s="355" t="inlineStr">
+        <is>
+          <t>Обновление pr-cy</t>
+        </is>
+      </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
+      <c r="A2" s="0" t="inlineStr">
         <is>
           <t>dealmed.ru</t>
         </is>
       </c>
-      <c r="B2" t="n">
+      <c r="B2" s="0" t="n">
         <v>9945</v>
       </c>
-      <c r="C2" t="n">
+      <c r="C2" s="0" t="n">
         <v>3710</v>
       </c>
-      <c r="D2" t="n">
+      <c r="D2" s="0" t="n">
         <v>12572</v>
       </c>
-      <c r="E2" t="n">
+      <c r="E2" s="0" t="n">
         <v>8095</v>
       </c>
-      <c r="F2" t="n">
+      <c r="F2" s="0" t="n">
         <v>57843</v>
       </c>
-      <c r="G2" t="n">
+      <c r="G2" s="0" t="n">
         <v>2003</v>
       </c>
-      <c r="H2" t="n">
+      <c r="H2" s="0" t="n">
         <v>26401</v>
       </c>
-      <c r="I2" t="n">
+      <c r="I2" s="0" t="n">
         <v>1576</v>
       </c>
-      <c r="J2" t="n">
+      <c r="J2" s="0" t="n">
         <v>38</v>
       </c>
-      <c r="K2" t="n">
+      <c r="K2" s="0" t="n">
         <v>14338</v>
       </c>
+      <c r="L2" t="n">
+        <v>195000</v>
+      </c>
+      <c r="M2" t="n">
+        <v>30</v>
+      </c>
+      <c r="N2" t="n">
+        <v>52</v>
+      </c>
+      <c r="O2" t="inlineStr">
+        <is>
+          <t>Здоровье</t>
+        </is>
+      </c>
+      <c r="P2" t="inlineStr">
+        <is>
+          <t>23.09.2026</t>
+        </is>
+      </c>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr">
+      <c r="A3" s="0" t="inlineStr">
         <is>
           <t>medcomp.ru</t>
         </is>
       </c>
-      <c r="B3" t="n">
+      <c r="B3" s="0" t="n">
         <v>2524</v>
       </c>
-      <c r="C3" t="n">
+      <c r="C3" s="0" t="n">
         <v>5921</v>
       </c>
-      <c r="D3" t="n">
+      <c r="D3" s="0" t="n">
         <v>6520</v>
       </c>
-      <c r="E3" t="n">
+      <c r="E3" s="0" t="n">
         <v>3014</v>
       </c>
-      <c r="F3" t="n">
+      <c r="F3" s="0" t="n">
         <v>18818</v>
       </c>
-      <c r="G3" t="n">
+      <c r="G3" s="0" t="n">
         <v>4610</v>
       </c>
-      <c r="H3" t="n">
+      <c r="H3" s="0" t="n">
         <v>20602</v>
       </c>
-      <c r="I3" t="n">
+      <c r="I3" s="0" t="n">
         <v>1266</v>
       </c>
-      <c r="J3" t="n">
+      <c r="J3" s="0" t="n">
         <v>15</v>
       </c>
-      <c r="K3" t="n">
+      <c r="K3" s="0" t="n">
         <v>5</v>
       </c>
+      <c r="L3" t="n">
+        <v>141000</v>
+      </c>
+      <c r="M3" t="n">
+        <v>33</v>
+      </c>
+      <c r="N3" t="n">
+        <v>48</v>
+      </c>
+      <c r="O3" t="inlineStr">
+        <is>
+          <t>Здоровье</t>
+        </is>
+      </c>
+      <c r="P3" t="inlineStr">
+        <is>
+          <t>26.09.2026</t>
+        </is>
+      </c>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr">
+      <c r="A4" s="0" t="inlineStr">
         <is>
           <t>medliga.ru</t>
         </is>
       </c>
-      <c r="B4" t="n">
+      <c r="B4" s="0" t="n">
         <v>1671</v>
       </c>
-      <c r="C4" t="n">
+      <c r="C4" s="0" t="n">
         <v>1150</v>
       </c>
-      <c r="D4" t="n">
+      <c r="D4" s="0" t="n">
         <v>2702</v>
       </c>
-      <c r="E4" t="n">
+      <c r="E4" s="0" t="n">
         <v>4333</v>
       </c>
-      <c r="F4" t="n">
+      <c r="F4" s="0" t="n">
         <v>11043</v>
       </c>
-      <c r="G4" t="n">
+      <c r="G4" s="0" t="n">
         <v>912</v>
       </c>
-      <c r="H4" t="n">
+      <c r="H4" s="0" t="n">
         <v>7865</v>
       </c>
-      <c r="I4" t="n">
+      <c r="I4" s="0" t="n">
         <v>702</v>
       </c>
-      <c r="J4" t="n">
+      <c r="J4" s="0" t="n">
         <v>44</v>
       </c>
-      <c r="K4" t="n">
+      <c r="K4" s="0" t="n">
         <v>3053</v>
       </c>
+      <c r="L4" t="n">
+        <v>49300</v>
+      </c>
+      <c r="M4" t="n">
+        <v>58</v>
+      </c>
+      <c r="N4" t="n">
+        <v>46</v>
+      </c>
+      <c r="O4" t="inlineStr">
+        <is>
+          <t>Здоровье</t>
+        </is>
+      </c>
+      <c r="P4" t="inlineStr">
+        <is>
+          <t>29.09.2026</t>
+        </is>
+      </c>
     </row>
     <row r="5">
-      <c r="A5" t="inlineStr">
+      <c r="A5" s="0" t="inlineStr">
         <is>
           <t>almamed.su</t>
         </is>
       </c>
-      <c r="B5" t="n">
+      <c r="B5" s="0" t="n">
         <v>902</v>
       </c>
-      <c r="C5" t="n">
+      <c r="C5" s="0" t="n">
         <v>985</v>
       </c>
-      <c r="D5" t="n">
+      <c r="D5" s="0" t="n">
         <v>6877</v>
       </c>
-      <c r="E5" t="n">
+      <c r="E5" s="0" t="n">
         <v>672</v>
       </c>
-      <c r="F5" t="n">
+      <c r="F5" s="0" t="n">
         <v>17379</v>
       </c>
-      <c r="G5" t="n">
+      <c r="G5" s="0" t="n">
         <v>445</v>
       </c>
-      <c r="H5" t="n">
+      <c r="H5" s="0" t="n">
         <v>11282</v>
       </c>
-      <c r="I5" t="n">
+      <c r="I5" s="0" t="n">
         <v>1150</v>
       </c>
-      <c r="J5" t="n">
+      <c r="J5" s="0" t="n">
         <v>41</v>
       </c>
-      <c r="K5" t="n">
+      <c r="K5" s="0" t="n">
         <v>0</v>
       </c>
+      <c r="L5" t="n">
+        <v>87800</v>
+      </c>
+      <c r="M5" t="n">
+        <v>65</v>
+      </c>
+      <c r="N5" t="n">
+        <v>46</v>
+      </c>
+      <c r="O5" t="inlineStr">
+        <is>
+          <t>Здоровье</t>
+        </is>
+      </c>
+      <c r="P5" t="inlineStr">
+        <is>
+          <t>24.09.2026</t>
+        </is>
+      </c>
     </row>
     <row r="6">
-      <c r="A6" t="inlineStr">
+      <c r="A6" s="0" t="inlineStr">
         <is>
           <t>medcub.ru</t>
         </is>
       </c>
-      <c r="B6" t="n">
+      <c r="B6" s="0" t="n">
         <v>1066</v>
       </c>
-      <c r="C6" t="n">
+      <c r="C6" s="0" t="n">
         <v>243</v>
       </c>
-      <c r="D6" t="n">
+      <c r="D6" s="0" t="n">
         <v>4240</v>
       </c>
-      <c r="E6" t="n">
+      <c r="E6" s="0" t="n">
         <v>1297</v>
       </c>
-      <c r="F6" t="n">
+      <c r="F6" s="0" t="n">
         <v>10031</v>
       </c>
-      <c r="G6" t="n">
+      <c r="G6" s="0" t="n">
         <v>94</v>
       </c>
-      <c r="H6" t="n">
+      <c r="H6" s="0" t="n">
         <v>3521</v>
       </c>
-      <c r="I6" t="n">
+      <c r="I6" s="0" t="n">
         <v>255</v>
       </c>
-      <c r="J6" t="n">
+      <c r="J6" s="0" t="n">
         <v>6</v>
       </c>
-      <c r="K6" t="n">
+      <c r="K6" s="0" t="n">
         <v>6299</v>
       </c>
+      <c r="L6" t="n">
+        <v>55700</v>
+      </c>
+      <c r="M6" t="n">
+        <v>29</v>
+      </c>
+      <c r="N6" t="n">
+        <v>58</v>
+      </c>
+      <c r="O6" t="inlineStr">
+        <is>
+          <t>Здоровье</t>
+        </is>
+      </c>
+      <c r="P6" t="inlineStr">
+        <is>
+          <t>25.08.2026</t>
+        </is>
+      </c>
     </row>
     <row r="7">
-      <c r="A7" t="inlineStr">
+      <c r="A7" s="0" t="inlineStr">
         <is>
           <t>global-mt.ru</t>
         </is>
       </c>
-      <c r="B7" t="n">
+      <c r="B7" s="0" t="n">
         <v>783</v>
       </c>
-      <c r="C7" t="n">
+      <c r="C7" s="0" t="n">
         <v>90</v>
       </c>
-      <c r="D7" t="n">
+      <c r="D7" s="0" t="n">
         <v>2054</v>
       </c>
-      <c r="E7" t="n">
+      <c r="E7" s="0" t="n">
         <v>1361</v>
       </c>
-      <c r="F7" t="n">
+      <c r="F7" s="0" t="n">
         <v>9645</v>
       </c>
-      <c r="G7" t="n">
+      <c r="G7" s="0" t="n">
         <v>42</v>
       </c>
-      <c r="H7" t="n">
+      <c r="H7" s="0" t="n">
         <v>1226</v>
       </c>
-      <c r="I7" t="n">
+      <c r="I7" s="0" t="n">
         <v>211</v>
       </c>
-      <c r="J7" t="n">
+      <c r="J7" s="0" t="n">
         <v>246</v>
       </c>
-      <c r="K7" t="n">
+      <c r="K7" s="0" t="n">
         <v>3</v>
       </c>
+      <c r="L7" t="n">
+        <v>32200</v>
+      </c>
+      <c r="M7" t="n">
+        <v>61</v>
+      </c>
+      <c r="N7" t="n">
+        <v>66</v>
+      </c>
+      <c r="O7" t="inlineStr">
+        <is>
+          <t>Здоровье</t>
+        </is>
+      </c>
+      <c r="P7" t="inlineStr">
+        <is>
+          <t>04.09.2026</t>
+        </is>
+      </c>
     </row>
     <row r="8">
-      <c r="A8" t="inlineStr">
+      <c r="A8" s="0" t="inlineStr">
         <is>
           <t>gmk-kiel.ru</t>
         </is>
       </c>
-      <c r="B8" t="n">
+      <c r="B8" s="0" t="n">
         <v>804</v>
       </c>
-      <c r="C8" t="n">
+      <c r="C8" s="0" t="n">
         <v>323</v>
       </c>
-      <c r="D8" t="n">
+      <c r="D8" s="0" t="n">
         <v>2250</v>
       </c>
-      <c r="E8" t="n">
+      <c r="E8" s="0" t="n">
         <v>907</v>
       </c>
-      <c r="F8" t="n">
+      <c r="F8" s="0" t="n">
         <v>8074</v>
       </c>
-      <c r="G8" t="n">
+      <c r="G8" s="0" t="n">
         <v>75</v>
       </c>
-      <c r="H8" t="n">
+      <c r="H8" s="0" t="n">
         <v>2688</v>
       </c>
-      <c r="I8" t="n">
+      <c r="I8" s="0" t="n">
         <v>132</v>
       </c>
-      <c r="J8" t="n">
+      <c r="J8" s="0" t="n">
         <v>20</v>
       </c>
-      <c r="K8" t="n">
+      <c r="K8" s="0" t="n">
         <v>172</v>
       </c>
+      <c r="L8" t="n">
+        <v>8740</v>
+      </c>
+      <c r="M8" t="n">
+        <v>44</v>
+      </c>
+      <c r="N8" t="n">
+        <v>49</v>
+      </c>
+      <c r="O8" t="inlineStr">
+        <is>
+          <t>Здоровье</t>
+        </is>
+      </c>
+      <c r="P8" t="inlineStr">
+        <is>
+          <t>21.07.2026</t>
+        </is>
+      </c>
     </row>
     <row r="9">
-      <c r="A9" t="inlineStr">
+      <c r="A9" s="0" t="inlineStr">
         <is>
           <t>cordismed.ru</t>
         </is>
       </c>
-      <c r="B9" t="n">
+      <c r="B9" s="0" t="n">
         <v>240</v>
       </c>
-      <c r="C9" t="n">
+      <c r="C9" s="0" t="n">
         <v>932</v>
       </c>
-      <c r="D9" t="n">
+      <c r="D9" s="0" t="n">
         <v>3242</v>
       </c>
-      <c r="E9" t="n">
+      <c r="E9" s="0" t="n">
         <v>486</v>
       </c>
-      <c r="F9" t="n">
+      <c r="F9" s="0" t="n">
         <v>5627</v>
       </c>
-      <c r="G9" t="n">
+      <c r="G9" s="0" t="n">
         <v>959</v>
       </c>
-      <c r="H9" t="n">
+      <c r="H9" s="0" t="n">
         <v>7004</v>
       </c>
-      <c r="I9" t="n">
+      <c r="I9" s="0" t="n">
         <v>401</v>
       </c>
-      <c r="J9" t="n">
+      <c r="J9" s="0" t="n">
         <v>24</v>
       </c>
-      <c r="K9" t="n">
+      <c r="K9" s="0" t="n">
         <v>286</v>
       </c>
+      <c r="L9" t="n">
+        <v>32700</v>
+      </c>
+      <c r="M9" t="n">
+        <v>20</v>
+      </c>
+      <c r="N9" t="n">
+        <v>52</v>
+      </c>
+      <c r="O9" t="inlineStr">
+        <is>
+          <t>Здоровье</t>
+        </is>
+      </c>
+      <c r="P9" t="inlineStr">
+        <is>
+          <t>21.07.2026</t>
+        </is>
+      </c>
     </row>
     <row r="10">
-      <c r="A10" t="inlineStr">
+      <c r="A10" s="0" t="inlineStr">
         <is>
           <t>medrk.ru</t>
         </is>
       </c>
-      <c r="B10" t="n">
+      <c r="B10" s="0" t="n">
         <v>302</v>
       </c>
-      <c r="C10" t="n">
+      <c r="C10" s="0" t="n">
         <v>1198</v>
       </c>
-      <c r="D10" t="n">
+      <c r="D10" s="0" t="n">
         <v>3539</v>
       </c>
-      <c r="E10" t="n">
+      <c r="E10" s="0" t="n">
         <v>421</v>
       </c>
-      <c r="F10" t="n">
+      <c r="F10" s="0" t="n">
         <v>6184</v>
       </c>
-      <c r="G10" t="n">
+      <c r="G10" s="0" t="n">
         <v>671</v>
       </c>
-      <c r="H10" t="n">
+      <c r="H10" s="0" t="n">
         <v>9501</v>
       </c>
-      <c r="I10" t="n">
+      <c r="I10" s="0" t="n">
         <v>1354</v>
       </c>
-      <c r="J10" t="n">
+      <c r="J10" s="0" t="n">
         <v>24</v>
       </c>
-      <c r="K10" t="n">
+      <c r="K10" s="0" t="n">
         <v>888</v>
       </c>
+      <c r="L10" t="n">
+        <v>42700</v>
+      </c>
+      <c r="M10" t="n">
+        <v>63</v>
+      </c>
+      <c r="N10" t="n">
+        <v>47</v>
+      </c>
+      <c r="O10" t="inlineStr">
+        <is>
+          <t>Здоровье</t>
+        </is>
+      </c>
+      <c r="P10" t="inlineStr">
+        <is>
+          <t>28.08.2026</t>
+        </is>
+      </c>
     </row>
     <row r="11">
-      <c r="A11" t="inlineStr">
+      <c r="A11" s="0" t="inlineStr">
         <is>
           <t>sterimed.ru</t>
         </is>
       </c>
-      <c r="B11" t="n">
+      <c r="B11" s="0" t="n">
         <v>440</v>
       </c>
-      <c r="C11" t="n">
+      <c r="C11" s="0" t="n">
         <v>153</v>
       </c>
-      <c r="D11" t="n">
+      <c r="D11" s="0" t="n">
         <v>1584</v>
       </c>
-      <c r="E11" t="n">
+      <c r="E11" s="0" t="n">
         <v>282</v>
       </c>
-      <c r="F11" t="n">
+      <c r="F11" s="0" t="n">
         <v>5515</v>
       </c>
-      <c r="G11" t="n">
+      <c r="G11" s="0" t="n">
         <v>77</v>
       </c>
-      <c r="H11" t="n">
+      <c r="H11" s="0" t="n">
         <v>2431</v>
       </c>
-      <c r="I11" t="n">
+      <c r="I11" s="0" t="n">
         <v>165</v>
       </c>
-      <c r="J11" t="n">
+      <c r="J11" s="0" t="n">
         <v>22</v>
       </c>
-      <c r="K11" t="n">
+      <c r="K11" s="0" t="n">
         <v>2142</v>
       </c>
+      <c r="L11" t="n">
+        <v>6570</v>
+      </c>
+      <c r="M11" t="n">
+        <v>34</v>
+      </c>
+      <c r="N11" t="n">
+        <v>43</v>
+      </c>
+      <c r="O11" t="inlineStr">
+        <is>
+          <t>Здоровье</t>
+        </is>
+      </c>
+      <c r="P11" t="inlineStr">
+        <is>
+          <t>22.09.2026</t>
+        </is>
+      </c>
     </row>
     <row r="12">
-      <c r="A12" t="inlineStr">
+      <c r="A12" s="0" t="inlineStr">
         <is>
           <t>ivlabmed.ru</t>
         </is>
       </c>
-      <c r="B12" t="n">
+      <c r="B12" s="0" t="n">
         <v>239</v>
       </c>
-      <c r="C12" t="n">
+      <c r="C12" s="0" t="n">
         <v>23</v>
       </c>
-      <c r="D12" t="n">
+      <c r="D12" s="0" t="n">
         <v>1096</v>
       </c>
-      <c r="E12" t="n">
+      <c r="E12" s="0" t="n">
         <v>233</v>
       </c>
-      <c r="F12" t="n">
+      <c r="F12" s="0" t="n">
         <v>5313</v>
       </c>
-      <c r="G12" t="n">
+      <c r="G12" s="0" t="n">
         <v>23</v>
       </c>
-      <c r="H12" t="n">
+      <c r="H12" s="0" t="n">
         <v>363</v>
       </c>
-      <c r="I12" t="n">
+      <c r="I12" s="0" t="n">
         <v>172</v>
       </c>
-      <c r="J12" t="n">
+      <c r="J12" s="0" t="n">
         <v>11</v>
       </c>
-      <c r="K12" t="n">
+      <c r="K12" s="0" t="n">
         <v>376</v>
       </c>
+      <c r="L12" t="n">
+        <v>11000</v>
+      </c>
+      <c r="M12" t="n">
+        <v>58</v>
+      </c>
+      <c r="N12" t="n">
+        <v>78</v>
+      </c>
+      <c r="O12" t="inlineStr">
+        <is>
+          <t>Здоровье</t>
+        </is>
+      </c>
+      <c r="P12" t="inlineStr">
+        <is>
+          <t>25.08.2026</t>
+        </is>
+      </c>
     </row>
     <row r="13">
-      <c r="A13" t="inlineStr">
+      <c r="A13" s="0" t="inlineStr">
         <is>
           <t>medbuy.ru</t>
         </is>
       </c>
-      <c r="B13" t="n">
+      <c r="B13" s="0" t="n">
         <v>236</v>
       </c>
-      <c r="C13" t="n">
+      <c r="C13" s="0" t="n">
         <v>57</v>
       </c>
-      <c r="D13" t="n">
+      <c r="D13" s="0" t="n">
         <v>636</v>
       </c>
-      <c r="E13" t="n">
+      <c r="E13" s="0" t="n">
         <v>352</v>
       </c>
-      <c r="F13" t="n">
+      <c r="F13" s="0" t="n">
         <v>4266</v>
       </c>
-      <c r="G13" t="n">
+      <c r="G13" s="0" t="n">
         <v>21</v>
       </c>
-      <c r="H13" t="n">
+      <c r="H13" s="0" t="n">
         <v>833</v>
       </c>
-      <c r="I13" t="n">
+      <c r="I13" s="0" t="n">
         <v>545</v>
       </c>
-      <c r="J13" t="n">
+      <c r="J13" s="0" t="n">
         <v>870</v>
       </c>
-      <c r="K13" t="n">
+      <c r="K13" s="0" t="n">
         <v>0</v>
       </c>
+      <c r="L13" t="n">
+        <v>14700</v>
+      </c>
+      <c r="M13" t="n">
+        <v>35</v>
+      </c>
+      <c r="N13" t="n">
+        <v>46</v>
+      </c>
+      <c r="O13" t="inlineStr">
+        <is>
+          <t>Здоровье</t>
+        </is>
+      </c>
+      <c r="P13" t="inlineStr">
+        <is>
+          <t>25.08.2026</t>
+        </is>
+      </c>
     </row>
     <row r="14">
-      <c r="A14" t="inlineStr">
+      <c r="A14" s="0" t="inlineStr">
         <is>
           <t>medpribor.pro</t>
         </is>
       </c>
-      <c r="B14" t="n">
+      <c r="B14" s="0" t="n">
         <v>358</v>
       </c>
-      <c r="C14" t="n">
+      <c r="C14" s="0" t="n">
         <v>371</v>
       </c>
-      <c r="D14" t="n">
+      <c r="D14" s="0" t="n">
         <v>939</v>
       </c>
-      <c r="E14" t="n">
+      <c r="E14" s="0" t="n">
         <v>317</v>
       </c>
-      <c r="F14" t="n">
+      <c r="F14" s="0" t="n">
         <v>3899</v>
       </c>
-      <c r="G14" t="n">
+      <c r="G14" s="0" t="n">
         <v>182</v>
       </c>
-      <c r="H14" t="n">
+      <c r="H14" s="0" t="n">
         <v>2575</v>
       </c>
-      <c r="I14" t="n">
+      <c r="I14" s="0" t="n">
         <v>460</v>
       </c>
-      <c r="J14" t="n">
+      <c r="J14" s="0" t="n">
         <v>14</v>
       </c>
-      <c r="K14" t="n">
+      <c r="K14" s="0" t="n">
         <v>685</v>
       </c>
+      <c r="L14" t="n">
+        <v>9880</v>
+      </c>
+      <c r="M14" t="n">
+        <v>23</v>
+      </c>
+      <c r="N14" t="n">
+        <v>45</v>
+      </c>
+      <c r="O14" t="inlineStr">
+        <is>
+          <t>Здоровье</t>
+        </is>
+      </c>
+      <c r="P14" t="inlineStr">
+        <is>
+          <t>16.09.2026</t>
+        </is>
+      </c>
     </row>
     <row r="15">
-      <c r="A15" t="inlineStr">
+      <c r="A15" s="0" t="inlineStr">
         <is>
           <t>medeq.ru</t>
         </is>
       </c>
-      <c r="B15" t="n">
+      <c r="B15" s="0" t="n">
         <v>419</v>
       </c>
-      <c r="C15" t="n">
+      <c r="C15" s="0" t="n">
         <v>245</v>
       </c>
-      <c r="D15" t="n">
+      <c r="D15" s="0" t="n">
         <v>1223</v>
       </c>
-      <c r="E15" t="n">
+      <c r="E15" s="0" t="n">
         <v>237</v>
       </c>
-      <c r="F15" t="n">
+      <c r="F15" s="0" t="n">
         <v>5100</v>
       </c>
-      <c r="G15" t="n">
+      <c r="G15" s="0" t="n">
         <v>138</v>
       </c>
-      <c r="H15" t="n">
+      <c r="H15" s="0" t="n">
         <v>2911</v>
       </c>
-      <c r="I15" t="n">
+      <c r="I15" s="0" t="n">
         <v>792</v>
       </c>
-      <c r="J15" t="n">
+      <c r="J15" s="0" t="n">
         <v>14</v>
       </c>
-      <c r="K15" t="n">
+      <c r="K15" s="0" t="n">
         <v>1287</v>
       </c>
+      <c r="L15" t="n">
+        <v>29300</v>
+      </c>
+      <c r="M15" t="n">
+        <v>4</v>
+      </c>
+      <c r="N15" t="n">
+        <v>58</v>
+      </c>
+      <c r="O15" t="inlineStr">
+        <is>
+          <t>Здоровье</t>
+        </is>
+      </c>
+      <c r="P15" t="inlineStr">
+        <is>
+          <t>29.09.2026</t>
+        </is>
+      </c>
     </row>
     <row r="16">
-      <c r="A16" t="inlineStr">
+      <c r="A16" s="0" t="inlineStr">
         <is>
           <t>farm-invest.ru</t>
         </is>
       </c>
-      <c r="B16" t="n">
+      <c r="B16" s="0" t="n">
         <v>177</v>
       </c>
-      <c r="C16" t="n">
+      <c r="C16" s="0" t="n">
         <v>1141</v>
       </c>
-      <c r="D16" t="n">
+      <c r="D16" s="0" t="n">
         <v>1506</v>
       </c>
-      <c r="E16" t="n">
+      <c r="E16" s="0" t="n">
         <v>274</v>
       </c>
-      <c r="F16" t="n">
+      <c r="F16" s="0" t="n">
         <v>3889</v>
       </c>
-      <c r="G16" t="n">
+      <c r="G16" s="0" t="n">
         <v>570</v>
       </c>
-      <c r="H16" t="n">
+      <c r="H16" s="0" t="n">
         <v>5330</v>
       </c>
-      <c r="I16" t="n">
+      <c r="I16" s="0" t="n">
         <v>583</v>
       </c>
-      <c r="J16" t="n">
+      <c r="J16" s="0" t="n">
         <v>14</v>
       </c>
-      <c r="K16" t="n">
+      <c r="K16" s="0" t="n">
         <v>303</v>
       </c>
+      <c r="L16" t="n">
+        <v>37000</v>
+      </c>
+      <c r="M16" t="n">
+        <v>17</v>
+      </c>
+      <c r="N16" t="n">
+        <v>59</v>
+      </c>
+      <c r="O16" t="inlineStr">
+        <is>
+          <t>Здоровье</t>
+        </is>
+      </c>
+      <c r="P16" t="inlineStr">
+        <is>
+          <t>14.09.2026</t>
+        </is>
+      </c>
     </row>
     <row r="17">
-      <c r="A17" t="inlineStr">
+      <c r="A17" s="0" t="inlineStr">
         <is>
           <t>uromed-m.ru</t>
         </is>
       </c>
-      <c r="B17" t="n">
+      <c r="B17" s="0" t="n">
         <v>237</v>
       </c>
-      <c r="C17" t="n">
+      <c r="C17" s="0" t="n">
         <v>1032</v>
       </c>
-      <c r="D17" t="n">
+      <c r="D17" s="0" t="n">
         <v>1492</v>
       </c>
-      <c r="E17" t="n">
+      <c r="E17" s="0" t="n">
         <v>224</v>
       </c>
-      <c r="F17" t="n">
+      <c r="F17" s="0" t="n">
         <v>2427</v>
       </c>
-      <c r="G17" t="n">
+      <c r="G17" s="0" t="n">
         <v>475</v>
       </c>
-      <c r="H17" t="n">
+      <c r="H17" s="0" t="n">
         <v>3955</v>
       </c>
-      <c r="I17" t="n">
+      <c r="I17" s="0" t="n">
         <v>348</v>
       </c>
-      <c r="J17" t="n">
+      <c r="J17" s="0" t="n">
         <v>43</v>
       </c>
-      <c r="K17" t="n">
+      <c r="K17" s="0" t="n">
         <v>0</v>
       </c>
+      <c r="L17" t="n">
+        <v>24800</v>
+      </c>
+      <c r="M17" t="n">
+        <v>78</v>
+      </c>
+      <c r="N17" t="n">
+        <v>47</v>
+      </c>
+      <c r="O17" t="inlineStr">
+        <is>
+          <t>Здоровье</t>
+        </is>
+      </c>
+      <c r="P17" t="inlineStr">
+        <is>
+          <t>20.07.2026</t>
+        </is>
+      </c>
     </row>
     <row r="18">
-      <c r="A18" t="inlineStr">
+      <c r="A18" s="0" t="inlineStr">
         <is>
           <t>intelmed.ru</t>
         </is>
       </c>
-      <c r="B18" t="n">
+      <c r="B18" s="0" t="n">
         <v>28</v>
       </c>
-      <c r="C18" t="n">
+      <c r="C18" s="0" t="n">
         <v>531</v>
       </c>
-      <c r="D18" t="n">
+      <c r="D18" s="0" t="n">
         <v>699</v>
       </c>
-      <c r="E18" t="n">
+      <c r="E18" s="0" t="n">
         <v>53</v>
       </c>
-      <c r="F18" t="n">
+      <c r="F18" s="0" t="n">
         <v>644</v>
       </c>
-      <c r="G18" t="n">
+      <c r="G18" s="0" t="n">
         <v>182</v>
       </c>
-      <c r="H18" t="n">
+      <c r="H18" s="0" t="n">
         <v>2912</v>
       </c>
-      <c r="I18" t="n">
+      <c r="I18" s="0" t="n">
         <v>240</v>
       </c>
-      <c r="J18" t="n">
+      <c r="J18" s="0" t="n">
         <v>37</v>
       </c>
-      <c r="K18" t="n">
+      <c r="K18" s="0" t="n">
         <v>0</v>
       </c>
+      <c r="L18" t="n">
+        <v>14700</v>
+      </c>
+      <c r="M18" t="n">
+        <v>60</v>
+      </c>
+      <c r="N18" t="n">
+        <v>48</v>
+      </c>
+      <c r="O18" t="inlineStr">
+        <is>
+          <t>Здоровье</t>
+        </is>
+      </c>
+      <c r="P18" t="inlineStr">
+        <is>
+          <t>25.08.2026</t>
+        </is>
+      </c>
     </row>
     <row r="19">
-      <c r="A19" t="inlineStr">
+      <c r="A19" s="0" t="inlineStr">
         <is>
           <t>kriptomed.ru</t>
         </is>
       </c>
-      <c r="B19" t="n">
+      <c r="B19" s="0" t="n">
         <v>194</v>
       </c>
-      <c r="C19" t="n">
+      <c r="C19" s="0" t="n">
         <v>423</v>
       </c>
-      <c r="D19" t="n">
+      <c r="D19" s="0" t="n">
         <v>870</v>
       </c>
-      <c r="E19" t="n">
+      <c r="E19" s="0" t="n">
         <v>250</v>
       </c>
-      <c r="F19" t="n">
+      <c r="F19" s="0" t="n">
         <v>2137</v>
       </c>
-      <c r="G19" t="n">
+      <c r="G19" s="0" t="n">
         <v>311</v>
       </c>
-      <c r="H19" t="n">
+      <c r="H19" s="0" t="n">
         <v>2020</v>
       </c>
-      <c r="I19" t="n">
+      <c r="I19" s="0" t="n">
         <v>156</v>
       </c>
-      <c r="J19" t="n">
+      <c r="J19" s="0" t="n">
         <v>45</v>
       </c>
-      <c r="K19" t="n">
+      <c r="K19" s="0" t="n">
         <v>5092</v>
       </c>
+      <c r="L19" t="n">
+        <v>7240</v>
+      </c>
+      <c r="M19" t="n">
+        <v>62</v>
+      </c>
+      <c r="N19" t="n">
+        <v>53</v>
+      </c>
+      <c r="O19" t="inlineStr">
+        <is>
+          <t>Здоровье</t>
+        </is>
+      </c>
+      <c r="P19" t="inlineStr">
+        <is>
+          <t>25.08.2026</t>
+        </is>
+      </c>
     </row>
     <row r="20">
-      <c r="A20" t="inlineStr">
+      <c r="A20" s="0" t="inlineStr">
         <is>
           <t>fotek.ru</t>
         </is>
       </c>
-      <c r="B20" t="n">
+      <c r="B20" s="0" t="n">
         <v>55</v>
       </c>
-      <c r="C20" t="n">
+      <c r="C20" s="0" t="n">
         <v>110</v>
       </c>
-      <c r="D20" t="n">
+      <c r="D20" s="0" t="n">
         <v>575</v>
       </c>
-      <c r="E20" t="n">
+      <c r="E20" s="0" t="n">
         <v>73</v>
       </c>
-      <c r="F20" t="n">
+      <c r="F20" s="0" t="n">
         <v>734</v>
       </c>
-      <c r="G20" t="n">
+      <c r="G20" s="0" t="n">
         <v>139</v>
       </c>
-      <c r="H20" t="n">
+      <c r="H20" s="0" t="n">
         <v>790</v>
       </c>
-      <c r="I20" t="n">
+      <c r="I20" s="0" t="n">
         <v>601</v>
       </c>
-      <c r="J20" t="n">
+      <c r="J20" s="0" t="n">
         <v>33</v>
       </c>
-      <c r="K20" t="n">
+      <c r="K20" s="0" t="n">
         <v>0</v>
       </c>
+      <c r="L20" t="n">
+        <v>6880</v>
+      </c>
+      <c r="M20" t="n">
+        <v>60</v>
+      </c>
+      <c r="N20" t="n">
+        <v>28</v>
+      </c>
+      <c r="O20" t="inlineStr">
+        <is>
+          <t>Здоровье</t>
+        </is>
+      </c>
+      <c r="P20" t="inlineStr">
+        <is>
+          <t>05.06.2026</t>
+        </is>
+      </c>
     </row>
     <row r="21">
-      <c r="A21" t="inlineStr">
+      <c r="A21" s="0" t="inlineStr">
         <is>
           <t>medgrade.pro</t>
         </is>
       </c>
-      <c r="B21" t="n">
+      <c r="B21" s="0" t="n">
         <v>188</v>
       </c>
-      <c r="C21" t="n">
+      <c r="C21" s="0" t="n">
         <v>155</v>
       </c>
-      <c r="D21" t="n">
+      <c r="D21" s="0" t="n">
         <v>3483</v>
       </c>
-      <c r="E21" t="n">
+      <c r="E21" s="0" t="n">
         <v>287</v>
       </c>
-      <c r="F21" t="n">
+      <c r="F21" s="0" t="n">
         <v>2044</v>
       </c>
-      <c r="G21" t="n">
+      <c r="G21" s="0" t="n">
         <v>133</v>
       </c>
-      <c r="H21" t="n">
+      <c r="H21" s="0" t="n">
         <v>2183</v>
       </c>
-      <c r="I21" t="n">
+      <c r="I21" s="0" t="n">
         <v>152</v>
       </c>
-      <c r="J21" t="n">
+      <c r="J21" s="0" t="n">
         <v>112</v>
       </c>
-      <c r="K21" t="n">
+      <c r="K21" s="0" t="n">
         <v>0</v>
       </c>
+      <c r="L21" t="n">
+        <v>11600</v>
+      </c>
+      <c r="M21" t="n">
+        <v>51</v>
+      </c>
+      <c r="N21" t="n">
+        <v>38</v>
+      </c>
+      <c r="O21" t="inlineStr">
+        <is>
+          <t>Здоровье</t>
+        </is>
+      </c>
+      <c r="P21" t="inlineStr">
+        <is>
+          <t>31.05.2026</t>
+        </is>
+      </c>
     </row>
     <row r="22">
-      <c r="A22" t="inlineStr">
+      <c r="A22" s="0" t="inlineStr">
         <is>
           <t>reiginmed.ru</t>
         </is>
       </c>
-      <c r="B22" t="n">
+      <c r="B22" s="0" t="n">
         <v>0</v>
       </c>
-      <c r="D22" t="n">
+      <c r="D22" s="0" t="n">
         <v>0</v>
       </c>
-      <c r="E22" t="n">
+      <c r="E22" s="0" t="n">
         <v>0</v>
       </c>
-      <c r="F22" t="n">
+      <c r="F22" s="0" t="n">
         <v>0</v>
       </c>
-      <c r="I22" t="n">
+      <c r="I22" s="0" t="n">
         <v>0</v>
       </c>
-      <c r="J22" t="n">
+      <c r="J22" s="0" t="n">
         <v>5</v>
       </c>
-      <c r="K22" t="n">
+      <c r="K22" s="0" t="n">
         <v>0</v>
+      </c>
+      <c r="O22" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="P22" t="inlineStr">
+        <is>
+          <t>29.04.2026</t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Write computed efficiency and links/donors values
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01GGxzKXyeNbw77cRhpGHusQ
</commit_message>
<xml_diff>
--- a/out/analiz_konkurentov_reiginmed.xlsx
+++ b/out/analiz_konkurentov_reiginmed.xlsx
@@ -20,7 +20,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="0.0"/>
+  </numFmts>
   <fonts count="12">
     <font>
       <name val="Arial"/>
@@ -1530,7 +1532,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="364">
+  <cellXfs count="367">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="bottom"/>
     </xf>
@@ -2581,6 +2583,15 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="7" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="10" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="6" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="bottom"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="227" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="bottom"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="24" borderId="11" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="bottom"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -3220,13 +3231,11 @@
       <c r="Q2" s="311" t="n">
         <v>82276</v>
       </c>
-      <c r="R2" s="46">
-        <f>IFERROR(N2/O2,"")</f>
-        <v/>
-      </c>
-      <c r="S2" s="46">
-        <f>IFERROR(P2/Q2,"")</f>
-        <v/>
+      <c r="R2" s="46" t="n">
+        <v>0.2439514393134919</v>
+      </c>
+      <c r="S2" s="46" t="n">
+        <v>0.1543828090816277</v>
       </c>
       <c r="T2" s="47" t="n">
         <v>632</v>
@@ -3234,9 +3243,8 @@
       <c r="U2" s="48" t="n">
         <v>4780</v>
       </c>
-      <c r="V2" s="49">
-        <f>IFERROR(U2/T2,"")</f>
-        <v/>
+      <c r="V2" s="364" t="n">
+        <v>7.563291139240507</v>
       </c>
       <c r="W2" s="50" t="n">
         <v>58</v>
@@ -3300,13 +3308,11 @@
       <c r="Q3" s="311" t="n">
         <v>42983</v>
       </c>
-      <c r="R3" s="46">
-        <f>IFERROR(N3/O3,"")</f>
-        <v/>
-      </c>
-      <c r="S3" s="46">
-        <f>IFERROR(P3/Q3,"")</f>
-        <v/>
+      <c r="R3" s="46" t="n">
+        <v>0.2838029166076738</v>
+      </c>
+      <c r="S3" s="46" t="n">
+        <v>0.3341786287602075</v>
       </c>
       <c r="T3" s="47" t="n">
         <v>490</v>
@@ -3314,9 +3320,8 @@
       <c r="U3" s="48" t="n">
         <v>8330</v>
       </c>
-      <c r="V3" s="49">
-        <f>IFERROR(U3/T3,"")</f>
-        <v/>
+      <c r="V3" s="364" t="n">
+        <v>17</v>
       </c>
       <c r="W3" s="50" t="n">
         <v>33</v>
@@ -3380,13 +3385,11 @@
       <c r="Q4" s="311" t="n">
         <v>17355</v>
       </c>
-      <c r="R4" s="46">
-        <f>IFERROR(N4/O4,"")</f>
-        <v/>
-      </c>
-      <c r="S4" s="46">
-        <f>IFERROR(P4/Q4,"")</f>
-        <v/>
+      <c r="R4" s="46" t="n">
+        <v>0.4966562639322336</v>
+      </c>
+      <c r="S4" s="46" t="n">
+        <v>0.2889080956496687</v>
       </c>
       <c r="T4" s="47" t="n">
         <v>566</v>
@@ -3394,9 +3397,8 @@
       <c r="U4" s="48" t="n">
         <v>23306</v>
       </c>
-      <c r="V4" s="49">
-        <f>IFERROR(U4/T4,"")</f>
-        <v/>
+      <c r="V4" s="364" t="n">
+        <v>41.17667844522968</v>
       </c>
       <c r="W4" s="50" t="n">
         <v>35</v>
@@ -3460,13 +3462,11 @@
       <c r="Q5" s="311" t="n">
         <v>61946</v>
       </c>
-      <c r="R5" s="46">
-        <f>IFERROR(N5/O5,"")</f>
-        <v/>
-      </c>
-      <c r="S5" s="46">
-        <f>IFERROR(P5/Q5,"")</f>
-        <v/>
+      <c r="R5" s="46" t="n">
+        <v>0.08438687563647201</v>
+      </c>
+      <c r="S5" s="46" t="n">
+        <v>0.07248248474477771</v>
       </c>
       <c r="T5" s="47" t="n">
         <v>392</v>
@@ -3474,9 +3474,8 @@
       <c r="U5" s="48" t="n">
         <v>2986</v>
       </c>
-      <c r="V5" s="49">
-        <f>IFERROR(U5/T5,"")</f>
-        <v/>
+      <c r="V5" s="364" t="n">
+        <v>7.61734693877551</v>
       </c>
       <c r="W5" s="50" t="n">
         <v>25</v>
@@ -3540,13 +3539,11 @@
       <c r="Q6" s="311" t="n">
         <v>16059</v>
       </c>
-      <c r="R6" s="46">
-        <f>IFERROR(N6/O6,"")</f>
-        <v/>
-      </c>
-      <c r="S6" s="46">
-        <f>IFERROR(P6/Q6,"")</f>
-        <v/>
+      <c r="R6" s="46" t="n">
+        <v>0.2619292260901731</v>
+      </c>
+      <c r="S6" s="46" t="n">
+        <v>0.08736534030761567</v>
       </c>
       <c r="T6" s="47" t="n">
         <v>79</v>
@@ -3554,9 +3551,8 @@
       <c r="U6" s="48" t="n">
         <v>394</v>
       </c>
-      <c r="V6" s="49">
-        <f>IFERROR(U6/T6,"")</f>
-        <v/>
+      <c r="V6" s="364" t="n">
+        <v>4.987341772151899</v>
       </c>
       <c r="W6" s="50" t="n">
         <v>5</v>
@@ -3620,13 +3616,11 @@
       <c r="Q7" s="311" t="n">
         <v>7340</v>
       </c>
-      <c r="R7" s="46">
-        <f>IFERROR(N7/O7,"")</f>
-        <v/>
-      </c>
-      <c r="S7" s="46">
-        <f>IFERROR(P7/Q7,"")</f>
-        <v/>
+      <c r="R7" s="46" t="n">
+        <v>0.3065489778318876</v>
+      </c>
+      <c r="S7" s="46" t="n">
+        <v>0.05994550408719346</v>
       </c>
       <c r="T7" s="47" t="n">
         <v>322</v>
@@ -3634,9 +3628,8 @@
       <c r="U7" s="48" t="n">
         <v>1962</v>
       </c>
-      <c r="V7" s="49">
-        <f>IFERROR(U7/T7,"")</f>
-        <v/>
+      <c r="V7" s="364" t="n">
+        <v>6.093167701863354</v>
       </c>
       <c r="W7" s="50" t="n">
         <v>15</v>
@@ -3700,13 +3693,11 @@
       <c r="Q8" s="311" t="n">
         <v>7205</v>
       </c>
-      <c r="R8" s="46">
-        <f>IFERROR(N8/O8,"")</f>
-        <v/>
-      </c>
-      <c r="S8" s="46">
-        <f>IFERROR(P8/Q8,"")</f>
-        <v/>
+      <c r="R8" s="46" t="n">
+        <v>0.2521646835372325</v>
+      </c>
+      <c r="S8" s="46" t="n">
+        <v>0.1772380291464261</v>
       </c>
       <c r="T8" s="47" t="n">
         <v>69</v>
@@ -3714,9 +3705,8 @@
       <c r="U8" s="48" t="n">
         <v>182</v>
       </c>
-      <c r="V8" s="49">
-        <f>IFERROR(U8/T8,"")</f>
-        <v/>
+      <c r="V8" s="364" t="n">
+        <v>2.63768115942029</v>
       </c>
       <c r="W8" s="50" t="n">
         <v>2</v>
@@ -3780,13 +3770,11 @@
       <c r="Q9" s="311" t="n">
         <v>22596</v>
       </c>
-      <c r="R9" s="46">
-        <f>IFERROR(N9/O9,"")</f>
-        <v/>
-      </c>
-      <c r="S9" s="46">
-        <f>IFERROR(P9/Q9,"")</f>
-        <v/>
+      <c r="R9" s="46" t="n">
+        <v>0.144758107962504</v>
+      </c>
+      <c r="S9" s="46" t="n">
+        <v>0.1677730571782616</v>
       </c>
       <c r="T9" s="47" t="n">
         <v>292</v>
@@ -3794,9 +3782,8 @@
       <c r="U9" s="48" t="n">
         <v>2803</v>
       </c>
-      <c r="V9" s="49">
-        <f>IFERROR(U9/T9,"")</f>
-        <v/>
+      <c r="V9" s="364" t="n">
+        <v>9.599315068493151</v>
       </c>
       <c r="W9" s="50" t="n">
         <v>22</v>
@@ -3860,13 +3847,11 @@
       <c r="Q10" s="311" t="n">
         <v>32743</v>
       </c>
-      <c r="R10" s="46">
-        <f>IFERROR(N10/O10,"")</f>
-        <v/>
-      </c>
-      <c r="S10" s="46">
-        <f>IFERROR(P10/Q10,"")</f>
-        <v/>
+      <c r="R10" s="46" t="n">
+        <v>0.06712235820370417</v>
+      </c>
+      <c r="S10" s="46" t="n">
+        <v>0.1443361939956632</v>
       </c>
       <c r="T10" s="47" t="n">
         <v>712</v>
@@ -3874,9 +3859,8 @@
       <c r="U10" s="48" t="n">
         <v>8628</v>
       </c>
-      <c r="V10" s="49">
-        <f>IFERROR(U10/T10,"")</f>
-        <v/>
+      <c r="V10" s="364" t="n">
+        <v>12.11797752808989</v>
       </c>
       <c r="W10" s="50" t="n">
         <v>23</v>
@@ -3940,13 +3924,11 @@
       <c r="Q11" s="311" t="n">
         <v>8113</v>
       </c>
-      <c r="R11" s="46">
-        <f>IFERROR(N11/O11,"")</f>
-        <v/>
-      </c>
-      <c r="S11" s="46">
-        <f>IFERROR(P11/Q11,"")</f>
-        <v/>
+      <c r="R11" s="46" t="n">
+        <v>0.2053818757419865</v>
+      </c>
+      <c r="S11" s="46" t="n">
+        <v>0.107728337236534</v>
       </c>
       <c r="T11" s="47" t="n">
         <v>107</v>
@@ -3954,9 +3936,8 @@
       <c r="U11" s="48" t="n">
         <v>363</v>
       </c>
-      <c r="V11" s="49">
-        <f>IFERROR(U11/T11,"")</f>
-        <v/>
+      <c r="V11" s="364" t="n">
+        <v>3.392523364485981</v>
       </c>
       <c r="W11" s="50" t="n">
         <v>21</v>
@@ -4020,13 +4001,11 @@
       <c r="Q12" s="311" t="n">
         <v>4310</v>
       </c>
-      <c r="R12" s="46">
-        <f>IFERROR(N12/O12,"")</f>
-        <v/>
-      </c>
-      <c r="S12" s="46">
-        <f>IFERROR(P12/Q12,"")</f>
-        <v/>
+      <c r="R12" s="46" t="n">
+        <v>0.1181547959300332</v>
+      </c>
+      <c r="S12" s="46" t="n">
+        <v>0.03503480278422274</v>
       </c>
       <c r="T12" s="47" t="n">
         <v>121</v>
@@ -4034,9 +4013,8 @@
       <c r="U12" s="48" t="n">
         <v>248</v>
       </c>
-      <c r="V12" s="49">
-        <f>IFERROR(U12/T12,"")</f>
-        <v/>
+      <c r="V12" s="364" t="n">
+        <v>2.049586776859504</v>
       </c>
       <c r="W12" s="50" t="n">
         <v>11</v>
@@ -4100,13 +4078,11 @@
       <c r="Q13" s="311" t="n">
         <v>6835</v>
       </c>
-      <c r="R13" s="46">
-        <f>IFERROR(N13/O13,"")</f>
-        <v/>
-      </c>
-      <c r="S13" s="46">
-        <f>IFERROR(P13/Q13,"")</f>
-        <v/>
+      <c r="R13" s="46" t="n">
+        <v>0.1025841002443717</v>
+      </c>
+      <c r="S13" s="46" t="n">
+        <v>0.03643013899049012</v>
       </c>
       <c r="T13" s="47" t="n">
         <v>262</v>
@@ -4114,9 +4090,8 @@
       <c r="U13" s="48" t="n">
         <v>1037</v>
       </c>
-      <c r="V13" s="49">
-        <f>IFERROR(U13/T13,"")</f>
-        <v/>
+      <c r="V13" s="364" t="n">
+        <v>3.958015267175572</v>
       </c>
       <c r="W13" s="50" t="n">
         <v>32</v>
@@ -4180,13 +4155,11 @@
       <c r="Q14" s="311" t="n">
         <v>10167</v>
       </c>
-      <c r="R14" s="46">
-        <f>IFERROR(N14/O14,"")</f>
-        <v/>
-      </c>
-      <c r="S14" s="46">
-        <f>IFERROR(P14/Q14,"")</f>
-        <v/>
+      <c r="R14" s="46" t="n">
+        <v>0.1132754342431762</v>
+      </c>
+      <c r="S14" s="46" t="n">
+        <v>0.1299301662240582</v>
       </c>
       <c r="T14" s="47" t="n">
         <v>269</v>
@@ -4194,9 +4167,8 @@
       <c r="U14" s="48" t="n">
         <v>1446</v>
       </c>
-      <c r="V14" s="49">
-        <f>IFERROR(U14/T14,"")</f>
-        <v/>
+      <c r="V14" s="364" t="n">
+        <v>5.37546468401487</v>
       </c>
       <c r="W14" s="50" t="n">
         <v>56</v>
@@ -4260,13 +4232,11 @@
       <c r="Q15" s="311" t="n">
         <v>15963</v>
       </c>
-      <c r="R15" s="46">
-        <f>IFERROR(N15/O15,"")</f>
-        <v/>
-      </c>
-      <c r="S15" s="46">
-        <f>IFERROR(P15/Q15,"")</f>
-        <v/>
+      <c r="R15" s="46" t="n">
+        <v>0.05670510187963987</v>
+      </c>
+      <c r="S15" s="46" t="n">
+        <v>0.07780492388648751</v>
       </c>
       <c r="T15" s="47" t="n">
         <v>256</v>
@@ -4274,9 +4244,8 @@
       <c r="U15" s="48" t="n">
         <v>7606</v>
       </c>
-      <c r="V15" s="49">
-        <f>IFERROR(U15/T15,"")</f>
-        <v/>
+      <c r="V15" s="364" t="n">
+        <v>29.7109375</v>
       </c>
       <c r="W15" s="50" t="n">
         <v>34</v>
@@ -4340,13 +4309,11 @@
       <c r="Q16" s="311" t="n">
         <v>12922</v>
       </c>
-      <c r="R16" s="46">
-        <f>IFERROR(N16/O16,"")</f>
-        <v/>
-      </c>
-      <c r="S16" s="46">
-        <f>IFERROR(P16/Q16,"")</f>
-        <v/>
+      <c r="R16" s="46" t="n">
+        <v>0.1212393664845425</v>
+      </c>
+      <c r="S16" s="46" t="n">
+        <v>0.2586286952484135</v>
       </c>
       <c r="T16" s="47" t="n">
         <v>337</v>
@@ -4354,9 +4321,8 @@
       <c r="U16" s="48" t="n">
         <v>1791</v>
       </c>
-      <c r="V16" s="49">
-        <f>IFERROR(U16/T16,"")</f>
-        <v/>
+      <c r="V16" s="364" t="n">
+        <v>5.314540059347181</v>
       </c>
       <c r="W16" s="50" t="n">
         <v>14</v>
@@ -4420,13 +4386,11 @@
       <c r="Q17" s="311" t="n">
         <v>11370</v>
       </c>
-      <c r="R17" s="46">
-        <f>IFERROR(N17/O17,"")</f>
-        <v/>
-      </c>
-      <c r="S17" s="46">
-        <f>IFERROR(P17/Q17,"")</f>
-        <v/>
+      <c r="R17" s="46" t="n">
+        <v>0.1445480631276901</v>
+      </c>
+      <c r="S17" s="46" t="n">
+        <v>0.2000879507475813</v>
       </c>
       <c r="T17" s="47" t="n">
         <v>287</v>
@@ -4434,9 +4398,8 @@
       <c r="U17" s="48" t="n">
         <v>750</v>
       </c>
-      <c r="V17" s="49">
-        <f>IFERROR(U17/T17,"")</f>
-        <v/>
+      <c r="V17" s="364" t="n">
+        <v>2.613240418118467</v>
       </c>
       <c r="W17" s="50" t="n">
         <v>18</v>
@@ -4500,13 +4463,11 @@
       <c r="Q18" s="311" t="n">
         <v>7622</v>
       </c>
-      <c r="R18" s="46">
-        <f>IFERROR(N18/O18,"")</f>
-        <v/>
-      </c>
-      <c r="S18" s="46">
-        <f>IFERROR(P18/Q18,"")</f>
-        <v/>
+      <c r="R18" s="46" t="n">
+        <v>0.05195827592993505</v>
+      </c>
+      <c r="S18" s="46" t="n">
+        <v>0.1966675413277355</v>
       </c>
       <c r="T18" s="47" t="n">
         <v>214</v>
@@ -4514,9 +4475,8 @@
       <c r="U18" s="48" t="n">
         <v>479</v>
       </c>
-      <c r="V18" s="49">
-        <f>IFERROR(U18/T18,"")</f>
-        <v/>
+      <c r="V18" s="364" t="n">
+        <v>2.238317757009346</v>
       </c>
       <c r="W18" s="50" t="n">
         <v>28</v>
@@ -4580,13 +4540,11 @@
       <c r="Q19" s="311" t="n">
         <v>6996</v>
       </c>
-      <c r="R19" s="46">
-        <f>IFERROR(N19/O19,"")</f>
-        <v/>
-      </c>
-      <c r="S19" s="46">
-        <f>IFERROR(P19/Q19,"")</f>
-        <v/>
+      <c r="R19" s="46" t="n">
+        <v>0.1182491289198606</v>
+      </c>
+      <c r="S19" s="46" t="n">
+        <v>0.1749571183533448</v>
       </c>
       <c r="T19" s="47" t="n">
         <v>127</v>
@@ -4594,9 +4552,8 @@
       <c r="U19" s="48" t="n">
         <v>253</v>
       </c>
-      <c r="V19" s="49">
-        <f>IFERROR(U19/T19,"")</f>
-        <v/>
+      <c r="V19" s="364" t="n">
+        <v>1.992125984251969</v>
       </c>
       <c r="W19" s="50" t="n">
         <v>12</v>
@@ -4660,13 +4617,11 @@
       <c r="Q20" s="311" t="n">
         <v>2338</v>
       </c>
-      <c r="R20" s="46">
-        <f>IFERROR(N20/O20,"")</f>
-        <v/>
-      </c>
-      <c r="S20" s="46">
-        <f>IFERROR(P20/Q20,"")</f>
-        <v/>
+      <c r="R20" s="46" t="n">
+        <v>0.1251471165162809</v>
+      </c>
+      <c r="S20" s="46" t="n">
+        <v>0.2001710863986313</v>
       </c>
       <c r="T20" s="47" t="n">
         <v>197</v>
@@ -4674,9 +4629,8 @@
       <c r="U20" s="48" t="n">
         <v>1911</v>
       </c>
-      <c r="V20" s="49">
-        <f>IFERROR(U20/T20,"")</f>
-        <v/>
+      <c r="V20" s="364" t="n">
+        <v>9.700507614213198</v>
       </c>
       <c r="W20" s="50" t="n">
         <v>25</v>
@@ -4740,13 +4694,11 @@
       <c r="Q21" s="311" t="n">
         <v>6995</v>
       </c>
-      <c r="R21" s="46">
-        <f>IFERROR(N21/O21,"")</f>
-        <v/>
-      </c>
-      <c r="S21" s="46">
-        <f>IFERROR(P21/Q21,"")</f>
-        <v/>
+      <c r="R21" s="46" t="n">
+        <v>0.1358265318552808</v>
+      </c>
+      <c r="S21" s="46" t="n">
+        <v>0.1368120085775554</v>
       </c>
       <c r="T21" s="47" t="n">
         <v>103</v>
@@ -4754,9 +4706,8 @@
       <c r="U21" s="48" t="n">
         <v>253</v>
       </c>
-      <c r="V21" s="49">
-        <f>IFERROR(U21/T21,"")</f>
-        <v/>
+      <c r="V21" s="364" t="n">
+        <v>2.45631067961165</v>
       </c>
       <c r="W21" s="50" t="n">
         <v>26</v>
@@ -4779,75 +4730,58 @@
       </c>
       <c r="C22" s="340" t="n"/>
       <c r="D22" s="340" t="n"/>
-      <c r="E22" s="336">
-        <f>IFERROR(MEDIAN(E2:E21),"")</f>
-        <v/>
-      </c>
-      <c r="F22" s="337">
-        <f>IFERROR(MEDIAN(F2:F21),"")</f>
-        <v/>
-      </c>
-      <c r="G22" s="337">
-        <f>IFERROR(MEDIAN(G2:G21),"")</f>
-        <v/>
-      </c>
-      <c r="H22" s="337">
-        <f>IFERROR(MEDIAN(H2:H21),"")</f>
-        <v/>
-      </c>
-      <c r="I22" s="338">
-        <f>IFERROR(MEDIAN(I2:I21),"")</f>
-        <v/>
-      </c>
-      <c r="J22" s="337">
-        <f>IFERROR(MEDIAN(J2:J21),"")</f>
-        <v/>
+      <c r="E22" s="336" t="n">
+        <v>4500</v>
+      </c>
+      <c r="F22" s="337" t="n">
+        <v>6660</v>
+      </c>
+      <c r="G22" s="337" t="n">
+        <v>13.15</v>
+      </c>
+      <c r="H22" s="337" t="n">
+        <v>300</v>
+      </c>
+      <c r="I22" s="338" t="n">
+        <v>6</v>
+      </c>
+      <c r="J22" s="337" t="n">
+        <v>29722.5</v>
       </c>
       <c r="K22" s="339" t="n"/>
-      <c r="L22" s="337">
-        <f>IFERROR(MEDIAN(L2:L21),"")</f>
-        <v/>
+      <c r="L22" s="337" t="n">
+        <v>35725</v>
       </c>
       <c r="M22" s="340" t="n"/>
-      <c r="N22" s="337">
-        <f t="array" ref="N22">MEDIAN(IF(X2:X21=" Лидер",N2:N21))</f>
-        <v/>
-      </c>
-      <c r="O22" s="337">
-        <f t="array" ref="O22">MEDIAN(IF(X2:X21=" Лидер",O2:O21))</f>
-        <v/>
-      </c>
-      <c r="P22" s="337">
-        <f t="array" ref="P22">MEDIAN(IF(X2:X21=" Лидер",P2:P21))</f>
-        <v/>
-      </c>
-      <c r="Q22" s="337">
-        <f t="array" ref="Q22">MEDIAN(IF(X2:X21=" Лидер",Q2:Q21))</f>
-        <v/>
-      </c>
-      <c r="R22" s="341">
-        <f>N22/O22</f>
-        <v/>
-      </c>
-      <c r="S22" s="341">
-        <f>P22/Q22</f>
-        <v/>
-      </c>
-      <c r="T22" s="336">
-        <f>IFERROR(MEDIAN(T2:T21),"")</f>
-        <v/>
-      </c>
-      <c r="U22" s="337">
-        <f>IFERROR(MEDIAN(U2:U21),"")</f>
-        <v/>
-      </c>
-      <c r="V22" s="337">
-        <f>IFERROR(MEDIAN(V2:V21),"")</f>
-        <v/>
-      </c>
-      <c r="W22" s="338">
-        <f>IFERROR(MEDIAN(W2:W21),"")</f>
-        <v/>
+      <c r="N22" s="337" t="n">
+        <v>6795</v>
+      </c>
+      <c r="O22" s="337" t="n">
+        <v>24331</v>
+      </c>
+      <c r="P22" s="337" t="n">
+        <v>4490</v>
+      </c>
+      <c r="Q22" s="337" t="n">
+        <v>17355</v>
+      </c>
+      <c r="R22" s="341" t="n">
+        <v>0.2792733549792446</v>
+      </c>
+      <c r="S22" s="341" t="n">
+        <v>0.2587150677038317</v>
+      </c>
+      <c r="T22" s="336" t="n">
+        <v>265.5</v>
+      </c>
+      <c r="U22" s="337" t="n">
+        <v>1618.5</v>
+      </c>
+      <c r="V22" s="365" t="n">
+        <v>5.345002371681026</v>
+      </c>
+      <c r="W22" s="338" t="n">
+        <v>24</v>
       </c>
       <c r="X22" s="340" t="n"/>
     </row>
@@ -4898,13 +4832,11 @@
       </c>
       <c r="P23" s="348" t="n"/>
       <c r="Q23" s="348" t="n"/>
-      <c r="R23" s="46">
-        <f>IFERROR(N23/O23,"")</f>
-        <v/>
-      </c>
-      <c r="S23" s="46">
-        <f>IFERROR(P23/Q23,"")</f>
-        <v/>
+      <c r="R23" s="46" t="n">
+        <v>0</v>
+      </c>
+      <c r="S23" s="46" t="n">
+        <v>0</v>
       </c>
       <c r="T23" s="349" t="n">
         <v>0</v>
@@ -4912,9 +4844,8 @@
       <c r="U23" s="350" t="n">
         <v>0</v>
       </c>
-      <c r="V23" s="351">
-        <f>IFERROR(U23/T23,"")</f>
-        <v/>
+      <c r="V23" s="366" t="n">
+        <v>0</v>
       </c>
       <c r="W23" s="352" t="n">
         <v>6</v>
@@ -5944,21 +5875,21 @@
       <c r="K2" s="0" t="n">
         <v>14338</v>
       </c>
-      <c r="L2" t="n">
+      <c r="L2" s="0" t="n">
         <v>195000</v>
       </c>
-      <c r="M2" t="n">
+      <c r="M2" s="0" t="n">
         <v>30</v>
       </c>
-      <c r="N2" t="n">
+      <c r="N2" s="0" t="n">
         <v>52</v>
       </c>
-      <c r="O2" t="inlineStr">
+      <c r="O2" s="0" t="inlineStr">
         <is>
           <t>Здоровье</t>
         </is>
       </c>
-      <c r="P2" t="inlineStr">
+      <c r="P2" s="0" t="inlineStr">
         <is>
           <t>23.09.2026</t>
         </is>
@@ -6000,21 +5931,21 @@
       <c r="K3" s="0" t="n">
         <v>5</v>
       </c>
-      <c r="L3" t="n">
+      <c r="L3" s="0" t="n">
         <v>141000</v>
       </c>
-      <c r="M3" t="n">
+      <c r="M3" s="0" t="n">
         <v>33</v>
       </c>
-      <c r="N3" t="n">
+      <c r="N3" s="0" t="n">
         <v>48</v>
       </c>
-      <c r="O3" t="inlineStr">
+      <c r="O3" s="0" t="inlineStr">
         <is>
           <t>Здоровье</t>
         </is>
       </c>
-      <c r="P3" t="inlineStr">
+      <c r="P3" s="0" t="inlineStr">
         <is>
           <t>26.09.2026</t>
         </is>
@@ -6056,21 +5987,21 @@
       <c r="K4" s="0" t="n">
         <v>3053</v>
       </c>
-      <c r="L4" t="n">
+      <c r="L4" s="0" t="n">
         <v>49300</v>
       </c>
-      <c r="M4" t="n">
+      <c r="M4" s="0" t="n">
         <v>58</v>
       </c>
-      <c r="N4" t="n">
+      <c r="N4" s="0" t="n">
         <v>46</v>
       </c>
-      <c r="O4" t="inlineStr">
+      <c r="O4" s="0" t="inlineStr">
         <is>
           <t>Здоровье</t>
         </is>
       </c>
-      <c r="P4" t="inlineStr">
+      <c r="P4" s="0" t="inlineStr">
         <is>
           <t>29.09.2026</t>
         </is>
@@ -6112,21 +6043,21 @@
       <c r="K5" s="0" t="n">
         <v>0</v>
       </c>
-      <c r="L5" t="n">
+      <c r="L5" s="0" t="n">
         <v>87800</v>
       </c>
-      <c r="M5" t="n">
+      <c r="M5" s="0" t="n">
         <v>65</v>
       </c>
-      <c r="N5" t="n">
+      <c r="N5" s="0" t="n">
         <v>46</v>
       </c>
-      <c r="O5" t="inlineStr">
+      <c r="O5" s="0" t="inlineStr">
         <is>
           <t>Здоровье</t>
         </is>
       </c>
-      <c r="P5" t="inlineStr">
+      <c r="P5" s="0" t="inlineStr">
         <is>
           <t>24.09.2026</t>
         </is>
@@ -6168,21 +6099,21 @@
       <c r="K6" s="0" t="n">
         <v>6299</v>
       </c>
-      <c r="L6" t="n">
+      <c r="L6" s="0" t="n">
         <v>55700</v>
       </c>
-      <c r="M6" t="n">
+      <c r="M6" s="0" t="n">
         <v>29</v>
       </c>
-      <c r="N6" t="n">
+      <c r="N6" s="0" t="n">
         <v>58</v>
       </c>
-      <c r="O6" t="inlineStr">
+      <c r="O6" s="0" t="inlineStr">
         <is>
           <t>Здоровье</t>
         </is>
       </c>
-      <c r="P6" t="inlineStr">
+      <c r="P6" s="0" t="inlineStr">
         <is>
           <t>25.08.2026</t>
         </is>
@@ -6224,21 +6155,21 @@
       <c r="K7" s="0" t="n">
         <v>3</v>
       </c>
-      <c r="L7" t="n">
+      <c r="L7" s="0" t="n">
         <v>32200</v>
       </c>
-      <c r="M7" t="n">
+      <c r="M7" s="0" t="n">
         <v>61</v>
       </c>
-      <c r="N7" t="n">
+      <c r="N7" s="0" t="n">
         <v>66</v>
       </c>
-      <c r="O7" t="inlineStr">
+      <c r="O7" s="0" t="inlineStr">
         <is>
           <t>Здоровье</t>
         </is>
       </c>
-      <c r="P7" t="inlineStr">
+      <c r="P7" s="0" t="inlineStr">
         <is>
           <t>04.09.2026</t>
         </is>
@@ -6280,21 +6211,21 @@
       <c r="K8" s="0" t="n">
         <v>172</v>
       </c>
-      <c r="L8" t="n">
+      <c r="L8" s="0" t="n">
         <v>8740</v>
       </c>
-      <c r="M8" t="n">
+      <c r="M8" s="0" t="n">
         <v>44</v>
       </c>
-      <c r="N8" t="n">
+      <c r="N8" s="0" t="n">
         <v>49</v>
       </c>
-      <c r="O8" t="inlineStr">
+      <c r="O8" s="0" t="inlineStr">
         <is>
           <t>Здоровье</t>
         </is>
       </c>
-      <c r="P8" t="inlineStr">
+      <c r="P8" s="0" t="inlineStr">
         <is>
           <t>21.07.2026</t>
         </is>
@@ -6336,21 +6267,21 @@
       <c r="K9" s="0" t="n">
         <v>286</v>
       </c>
-      <c r="L9" t="n">
+      <c r="L9" s="0" t="n">
         <v>32700</v>
       </c>
-      <c r="M9" t="n">
+      <c r="M9" s="0" t="n">
         <v>20</v>
       </c>
-      <c r="N9" t="n">
+      <c r="N9" s="0" t="n">
         <v>52</v>
       </c>
-      <c r="O9" t="inlineStr">
+      <c r="O9" s="0" t="inlineStr">
         <is>
           <t>Здоровье</t>
         </is>
       </c>
-      <c r="P9" t="inlineStr">
+      <c r="P9" s="0" t="inlineStr">
         <is>
           <t>21.07.2026</t>
         </is>
@@ -6392,21 +6323,21 @@
       <c r="K10" s="0" t="n">
         <v>888</v>
       </c>
-      <c r="L10" t="n">
+      <c r="L10" s="0" t="n">
         <v>42700</v>
       </c>
-      <c r="M10" t="n">
+      <c r="M10" s="0" t="n">
         <v>63</v>
       </c>
-      <c r="N10" t="n">
+      <c r="N10" s="0" t="n">
         <v>47</v>
       </c>
-      <c r="O10" t="inlineStr">
+      <c r="O10" s="0" t="inlineStr">
         <is>
           <t>Здоровье</t>
         </is>
       </c>
-      <c r="P10" t="inlineStr">
+      <c r="P10" s="0" t="inlineStr">
         <is>
           <t>28.08.2026</t>
         </is>
@@ -6448,21 +6379,21 @@
       <c r="K11" s="0" t="n">
         <v>2142</v>
       </c>
-      <c r="L11" t="n">
+      <c r="L11" s="0" t="n">
         <v>6570</v>
       </c>
-      <c r="M11" t="n">
+      <c r="M11" s="0" t="n">
         <v>34</v>
       </c>
-      <c r="N11" t="n">
+      <c r="N11" s="0" t="n">
         <v>43</v>
       </c>
-      <c r="O11" t="inlineStr">
+      <c r="O11" s="0" t="inlineStr">
         <is>
           <t>Здоровье</t>
         </is>
       </c>
-      <c r="P11" t="inlineStr">
+      <c r="P11" s="0" t="inlineStr">
         <is>
           <t>22.09.2026</t>
         </is>
@@ -6504,21 +6435,21 @@
       <c r="K12" s="0" t="n">
         <v>376</v>
       </c>
-      <c r="L12" t="n">
+      <c r="L12" s="0" t="n">
         <v>11000</v>
       </c>
-      <c r="M12" t="n">
+      <c r="M12" s="0" t="n">
         <v>58</v>
       </c>
-      <c r="N12" t="n">
+      <c r="N12" s="0" t="n">
         <v>78</v>
       </c>
-      <c r="O12" t="inlineStr">
+      <c r="O12" s="0" t="inlineStr">
         <is>
           <t>Здоровье</t>
         </is>
       </c>
-      <c r="P12" t="inlineStr">
+      <c r="P12" s="0" t="inlineStr">
         <is>
           <t>25.08.2026</t>
         </is>
@@ -6560,21 +6491,21 @@
       <c r="K13" s="0" t="n">
         <v>0</v>
       </c>
-      <c r="L13" t="n">
+      <c r="L13" s="0" t="n">
         <v>14700</v>
       </c>
-      <c r="M13" t="n">
+      <c r="M13" s="0" t="n">
         <v>35</v>
       </c>
-      <c r="N13" t="n">
+      <c r="N13" s="0" t="n">
         <v>46</v>
       </c>
-      <c r="O13" t="inlineStr">
+      <c r="O13" s="0" t="inlineStr">
         <is>
           <t>Здоровье</t>
         </is>
       </c>
-      <c r="P13" t="inlineStr">
+      <c r="P13" s="0" t="inlineStr">
         <is>
           <t>25.08.2026</t>
         </is>
@@ -6616,21 +6547,21 @@
       <c r="K14" s="0" t="n">
         <v>685</v>
       </c>
-      <c r="L14" t="n">
+      <c r="L14" s="0" t="n">
         <v>9880</v>
       </c>
-      <c r="M14" t="n">
+      <c r="M14" s="0" t="n">
         <v>23</v>
       </c>
-      <c r="N14" t="n">
+      <c r="N14" s="0" t="n">
         <v>45</v>
       </c>
-      <c r="O14" t="inlineStr">
+      <c r="O14" s="0" t="inlineStr">
         <is>
           <t>Здоровье</t>
         </is>
       </c>
-      <c r="P14" t="inlineStr">
+      <c r="P14" s="0" t="inlineStr">
         <is>
           <t>16.09.2026</t>
         </is>
@@ -6672,21 +6603,21 @@
       <c r="K15" s="0" t="n">
         <v>1287</v>
       </c>
-      <c r="L15" t="n">
+      <c r="L15" s="0" t="n">
         <v>29300</v>
       </c>
-      <c r="M15" t="n">
+      <c r="M15" s="0" t="n">
         <v>4</v>
       </c>
-      <c r="N15" t="n">
+      <c r="N15" s="0" t="n">
         <v>58</v>
       </c>
-      <c r="O15" t="inlineStr">
+      <c r="O15" s="0" t="inlineStr">
         <is>
           <t>Здоровье</t>
         </is>
       </c>
-      <c r="P15" t="inlineStr">
+      <c r="P15" s="0" t="inlineStr">
         <is>
           <t>29.09.2026</t>
         </is>
@@ -6728,21 +6659,21 @@
       <c r="K16" s="0" t="n">
         <v>303</v>
       </c>
-      <c r="L16" t="n">
+      <c r="L16" s="0" t="n">
         <v>37000</v>
       </c>
-      <c r="M16" t="n">
+      <c r="M16" s="0" t="n">
         <v>17</v>
       </c>
-      <c r="N16" t="n">
+      <c r="N16" s="0" t="n">
         <v>59</v>
       </c>
-      <c r="O16" t="inlineStr">
+      <c r="O16" s="0" t="inlineStr">
         <is>
           <t>Здоровье</t>
         </is>
       </c>
-      <c r="P16" t="inlineStr">
+      <c r="P16" s="0" t="inlineStr">
         <is>
           <t>14.09.2026</t>
         </is>
@@ -6784,21 +6715,21 @@
       <c r="K17" s="0" t="n">
         <v>0</v>
       </c>
-      <c r="L17" t="n">
+      <c r="L17" s="0" t="n">
         <v>24800</v>
       </c>
-      <c r="M17" t="n">
+      <c r="M17" s="0" t="n">
         <v>78</v>
       </c>
-      <c r="N17" t="n">
+      <c r="N17" s="0" t="n">
         <v>47</v>
       </c>
-      <c r="O17" t="inlineStr">
+      <c r="O17" s="0" t="inlineStr">
         <is>
           <t>Здоровье</t>
         </is>
       </c>
-      <c r="P17" t="inlineStr">
+      <c r="P17" s="0" t="inlineStr">
         <is>
           <t>20.07.2026</t>
         </is>
@@ -6840,21 +6771,21 @@
       <c r="K18" s="0" t="n">
         <v>0</v>
       </c>
-      <c r="L18" t="n">
+      <c r="L18" s="0" t="n">
         <v>14700</v>
       </c>
-      <c r="M18" t="n">
+      <c r="M18" s="0" t="n">
         <v>60</v>
       </c>
-      <c r="N18" t="n">
+      <c r="N18" s="0" t="n">
         <v>48</v>
       </c>
-      <c r="O18" t="inlineStr">
+      <c r="O18" s="0" t="inlineStr">
         <is>
           <t>Здоровье</t>
         </is>
       </c>
-      <c r="P18" t="inlineStr">
+      <c r="P18" s="0" t="inlineStr">
         <is>
           <t>25.08.2026</t>
         </is>
@@ -6896,21 +6827,21 @@
       <c r="K19" s="0" t="n">
         <v>5092</v>
       </c>
-      <c r="L19" t="n">
+      <c r="L19" s="0" t="n">
         <v>7240</v>
       </c>
-      <c r="M19" t="n">
+      <c r="M19" s="0" t="n">
         <v>62</v>
       </c>
-      <c r="N19" t="n">
+      <c r="N19" s="0" t="n">
         <v>53</v>
       </c>
-      <c r="O19" t="inlineStr">
+      <c r="O19" s="0" t="inlineStr">
         <is>
           <t>Здоровье</t>
         </is>
       </c>
-      <c r="P19" t="inlineStr">
+      <c r="P19" s="0" t="inlineStr">
         <is>
           <t>25.08.2026</t>
         </is>
@@ -6952,21 +6883,21 @@
       <c r="K20" s="0" t="n">
         <v>0</v>
       </c>
-      <c r="L20" t="n">
+      <c r="L20" s="0" t="n">
         <v>6880</v>
       </c>
-      <c r="M20" t="n">
+      <c r="M20" s="0" t="n">
         <v>60</v>
       </c>
-      <c r="N20" t="n">
+      <c r="N20" s="0" t="n">
         <v>28</v>
       </c>
-      <c r="O20" t="inlineStr">
+      <c r="O20" s="0" t="inlineStr">
         <is>
           <t>Здоровье</t>
         </is>
       </c>
-      <c r="P20" t="inlineStr">
+      <c r="P20" s="0" t="inlineStr">
         <is>
           <t>05.06.2026</t>
         </is>
@@ -7008,21 +6939,21 @@
       <c r="K21" s="0" t="n">
         <v>0</v>
       </c>
-      <c r="L21" t="n">
+      <c r="L21" s="0" t="n">
         <v>11600</v>
       </c>
-      <c r="M21" t="n">
+      <c r="M21" s="0" t="n">
         <v>51</v>
       </c>
-      <c r="N21" t="n">
+      <c r="N21" s="0" t="n">
         <v>38</v>
       </c>
-      <c r="O21" t="inlineStr">
+      <c r="O21" s="0" t="inlineStr">
         <is>
           <t>Здоровье</t>
         </is>
       </c>
-      <c r="P21" t="inlineStr">
+      <c r="P21" s="0" t="inlineStr">
         <is>
           <t>31.05.2026</t>
         </is>
@@ -7055,12 +6986,12 @@
       <c r="K22" s="0" t="n">
         <v>0</v>
       </c>
-      <c r="O22" t="inlineStr">
+      <c r="O22" s="0" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="P22" t="inlineStr">
+      <c r="P22" s="0" t="inlineStr">
         <is>
           <t>29.04.2026</t>
         </is>

</xml_diff>

<commit_message>
Set stagnation dynamics for reiginmed.ru
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01GGxzKXyeNbw77cRhpGHusQ
</commit_message>
<xml_diff>
--- a/out/analiz_konkurentov_reiginmed.xlsx
+++ b/out/analiz_konkurentov_reiginmed.xlsx
@@ -4821,9 +4821,17 @@
       <c r="J23" s="348" t="n">
         <v>0</v>
       </c>
-      <c r="K23" s="131" t="n"/>
+      <c r="K23" s="131" t="inlineStr">
+        <is>
+          <t>Стагнация</t>
+        </is>
+      </c>
       <c r="L23" s="348" t="n"/>
-      <c r="M23" s="131" t="n"/>
+      <c r="M23" s="131" t="inlineStr">
+        <is>
+          <t>Стагнация</t>
+        </is>
+      </c>
       <c r="N23" s="348" t="n">
         <v>0</v>
       </c>

</xml_diff>

<commit_message>
Add visibility dynamics for top competitors
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01GGxzKXyeNbw77cRhpGHusQ
</commit_message>
<xml_diff>
--- a/out/analiz_konkurentov_reiginmed.xlsx
+++ b/out/analiz_konkurentov_reiginmed.xlsx
@@ -3214,11 +3214,19 @@
       <c r="J2" s="38" t="n">
         <v>895089</v>
       </c>
-      <c r="K2" s="131" t="n"/>
+      <c r="K2" s="131" t="inlineStr">
+        <is>
+          <t>Сильный рост</t>
+        </is>
+      </c>
       <c r="L2" s="40" t="n">
         <v>333910</v>
       </c>
-      <c r="M2" s="41" t="n"/>
+      <c r="M2" s="41" t="inlineStr">
+        <is>
+          <t>Стагнация</t>
+        </is>
+      </c>
       <c r="N2" s="42" t="n">
         <v>34000</v>
       </c>
@@ -3291,11 +3299,19 @@
       <c r="J3" s="38" t="n">
         <v>227153</v>
       </c>
-      <c r="K3" s="131" t="n"/>
+      <c r="K3" s="131" t="inlineStr">
+        <is>
+          <t>Рост</t>
+        </is>
+      </c>
       <c r="L3" s="40" t="n">
         <v>532882</v>
       </c>
-      <c r="M3" s="41" t="n"/>
+      <c r="M3" s="41" t="inlineStr">
+        <is>
+          <t>Падение</t>
+        </is>
+      </c>
       <c r="N3" s="42" t="n">
         <v>12027</v>
       </c>
@@ -3368,7 +3384,11 @@
       <c r="J4" s="38" t="n">
         <v>150351</v>
       </c>
-      <c r="K4" s="131" t="n"/>
+      <c r="K4" s="131" t="inlineStr">
+        <is>
+          <t>Рост</t>
+        </is>
+      </c>
       <c r="L4" s="40" t="n">
         <v>103519</v>
       </c>

</xml_diff>

<commit_message>
Add dynamics for medliga, almamed, medcub
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01GGxzKXyeNbw77cRhpGHusQ
</commit_message>
<xml_diff>
--- a/out/analiz_konkurentov_reiginmed.xlsx
+++ b/out/analiz_konkurentov_reiginmed.xlsx
@@ -3392,7 +3392,11 @@
       <c r="L4" s="40" t="n">
         <v>103519</v>
       </c>
-      <c r="M4" s="41" t="n"/>
+      <c r="M4" s="41" t="inlineStr">
+        <is>
+          <t>Стагнация</t>
+        </is>
+      </c>
       <c r="N4" s="42" t="n">
         <v>8912</v>
       </c>
@@ -3465,11 +3469,19 @@
       <c r="J5" s="38" t="n">
         <v>81164</v>
       </c>
-      <c r="K5" s="131" t="n"/>
+      <c r="K5" s="131" t="inlineStr">
+        <is>
+          <t>Рост</t>
+        </is>
+      </c>
       <c r="L5" s="40" t="n">
         <v>88676</v>
       </c>
-      <c r="M5" s="41" t="n"/>
+      <c r="M5" s="41" t="inlineStr">
+        <is>
+          <t>Падение</t>
+        </is>
+      </c>
       <c r="N5" s="42" t="n">
         <v>6795</v>
       </c>
@@ -3542,11 +3554,19 @@
       <c r="J6" s="38" t="n">
         <v>95974</v>
       </c>
-      <c r="K6" s="131" t="n"/>
+      <c r="K6" s="131" t="inlineStr">
+        <is>
+          <t>Рост</t>
+        </is>
+      </c>
       <c r="L6" s="40" t="n">
         <v>21858</v>
       </c>
-      <c r="M6" s="41" t="n"/>
+      <c r="M6" s="41" t="inlineStr">
+        <is>
+          <t>Рост</t>
+        </is>
+      </c>
       <c r="N6" s="42" t="n">
         <v>6373</v>
       </c>

</xml_diff>

<commit_message>
Add dynamics for global-mt, gmk-kiel, cordismed
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01GGxzKXyeNbw77cRhpGHusQ
</commit_message>
<xml_diff>
--- a/out/analiz_konkurentov_reiginmed.xlsx
+++ b/out/analiz_konkurentov_reiginmed.xlsx
@@ -3639,11 +3639,19 @@
       <c r="J7" s="38" t="n">
         <v>70465</v>
       </c>
-      <c r="K7" s="131" t="n"/>
+      <c r="K7" s="131" t="inlineStr">
+        <is>
+          <t>Рост</t>
+        </is>
+      </c>
       <c r="L7" s="40" t="n">
         <v>8117</v>
       </c>
-      <c r="M7" s="41" t="n"/>
+      <c r="M7" s="41" t="inlineStr">
+        <is>
+          <t>Стагнация</t>
+        </is>
+      </c>
       <c r="N7" s="42" t="n">
         <v>6043</v>
       </c>
@@ -3716,11 +3724,19 @@
       <c r="J8" s="38" t="n">
         <v>72336</v>
       </c>
-      <c r="K8" s="131" t="n"/>
+      <c r="K8" s="131" t="inlineStr">
+        <is>
+          <t>Рост</t>
+        </is>
+      </c>
       <c r="L8" s="40" t="n">
         <v>29067</v>
       </c>
-      <c r="M8" s="41" t="n"/>
+      <c r="M8" s="41" t="inlineStr">
+        <is>
+          <t>Стагнация</t>
+        </is>
+      </c>
       <c r="N8" s="42" t="n">
         <v>4514</v>
       </c>
@@ -3797,7 +3813,11 @@
       <c r="L9" s="40" t="n">
         <v>83848</v>
       </c>
-      <c r="M9" s="41" t="n"/>
+      <c r="M9" s="41" t="inlineStr">
+        <is>
+          <t>Стагнация</t>
+        </is>
+      </c>
       <c r="N9" s="42" t="n">
         <v>2687</v>
       </c>

</xml_diff>

<commit_message>
Add dynamics for cordismed, medrk, sterimed
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01GGxzKXyeNbw77cRhpGHusQ
</commit_message>
<xml_diff>
--- a/out/analiz_konkurentov_reiginmed.xlsx
+++ b/out/analiz_konkurentov_reiginmed.xlsx
@@ -3809,7 +3809,11 @@
       <c r="J9" s="38" t="n">
         <v>21573</v>
       </c>
-      <c r="K9" s="131" t="n"/>
+      <c r="K9" s="131" t="inlineStr">
+        <is>
+          <t>Рост</t>
+        </is>
+      </c>
       <c r="L9" s="40" t="n">
         <v>83848</v>
       </c>
@@ -3890,11 +3894,19 @@
       <c r="J10" s="38" t="n">
         <v>27185</v>
       </c>
-      <c r="K10" s="131" t="n"/>
+      <c r="K10" s="131" t="inlineStr">
+        <is>
+          <t>Рост</t>
+        </is>
+      </c>
       <c r="L10" s="40" t="n">
         <v>107840</v>
       </c>
-      <c r="M10" s="41" t="n"/>
+      <c r="M10" s="41" t="inlineStr">
+        <is>
+          <t>Стагнация</t>
+        </is>
+      </c>
       <c r="N10" s="42" t="n">
         <v>2671</v>
       </c>
@@ -3967,11 +3979,19 @@
       <c r="J11" s="38" t="n">
         <v>39613</v>
       </c>
-      <c r="K11" s="131" t="n"/>
+      <c r="K11" s="131" t="inlineStr">
+        <is>
+          <t>Рост</t>
+        </is>
+      </c>
       <c r="L11" s="40" t="n">
         <v>13726</v>
       </c>
-      <c r="M11" s="41" t="n"/>
+      <c r="M11" s="41" t="inlineStr">
+        <is>
+          <t>Падение</t>
+        </is>
+      </c>
       <c r="N11" s="42" t="n">
         <v>2595</v>
       </c>

</xml_diff>

<commit_message>
Add dynamics for ivlabmed, medbuy, medpribor
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01GGxzKXyeNbw77cRhpGHusQ
</commit_message>
<xml_diff>
--- a/out/analiz_konkurentov_reiginmed.xlsx
+++ b/out/analiz_konkurentov_reiginmed.xlsx
@@ -4064,11 +4064,19 @@
       <c r="J12" s="38" t="n">
         <v>21474</v>
       </c>
-      <c r="K12" s="131" t="n"/>
+      <c r="K12" s="131" t="inlineStr">
+        <is>
+          <t>Рост</t>
+        </is>
+      </c>
       <c r="L12" s="40" t="n">
         <v>2035</v>
       </c>
-      <c r="M12" s="41" t="n"/>
+      <c r="M12" s="41" t="inlineStr">
+        <is>
+          <t>Стагнация</t>
+        </is>
+      </c>
       <c r="N12" s="42" t="n">
         <v>2067</v>
       </c>
@@ -4141,11 +4149,19 @@
       <c r="J13" s="38" t="n">
         <v>21260</v>
       </c>
-      <c r="K13" s="131" t="n"/>
+      <c r="K13" s="131" t="inlineStr">
+        <is>
+          <t>Сильный рост</t>
+        </is>
+      </c>
       <c r="L13" s="40" t="n">
         <v>5156</v>
       </c>
-      <c r="M13" s="41" t="n"/>
+      <c r="M13" s="41" t="inlineStr">
+        <is>
+          <t>Падение</t>
+        </is>
+      </c>
       <c r="N13" s="42" t="n">
         <v>1973</v>
       </c>
@@ -4218,7 +4234,11 @@
       <c r="J14" s="38" t="n">
         <v>32260</v>
       </c>
-      <c r="K14" s="131" t="n"/>
+      <c r="K14" s="131" t="inlineStr">
+        <is>
+          <t>Рост</t>
+        </is>
+      </c>
       <c r="L14" s="40" t="n">
         <v>33398</v>
       </c>

</xml_diff>

<commit_message>
Add dynamics for medpribor, medeq, farm-invest
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01GGxzKXyeNbw77cRhpGHusQ
</commit_message>
<xml_diff>
--- a/out/analiz_konkurentov_reiginmed.xlsx
+++ b/out/analiz_konkurentov_reiginmed.xlsx
@@ -4242,7 +4242,11 @@
       <c r="L14" s="40" t="n">
         <v>33398</v>
       </c>
-      <c r="M14" s="41" t="n"/>
+      <c r="M14" s="41" t="inlineStr">
+        <is>
+          <t>Падение</t>
+        </is>
+      </c>
       <c r="N14" s="42" t="n">
         <v>1826</v>
       </c>
@@ -4315,11 +4319,19 @@
       <c r="J15" s="38" t="n">
         <v>37751</v>
       </c>
-      <c r="K15" s="131" t="n"/>
+      <c r="K15" s="131" t="inlineStr">
+        <is>
+          <t>Рост</t>
+        </is>
+      </c>
       <c r="L15" s="40" t="n">
         <v>22013</v>
       </c>
-      <c r="M15" s="41" t="n"/>
+      <c r="M15" s="41" t="inlineStr">
+        <is>
+          <t>Падение</t>
+        </is>
+      </c>
       <c r="N15" s="42" t="n">
         <v>1795</v>
       </c>
@@ -4392,11 +4404,19 @@
       <c r="J16" s="38" t="n">
         <v>15955</v>
       </c>
-      <c r="K16" s="131" t="n"/>
+      <c r="K16" s="131" t="inlineStr">
+        <is>
+          <t>Рост</t>
+        </is>
+      </c>
       <c r="L16" s="40" t="n">
         <v>102730</v>
       </c>
-      <c r="M16" s="41" t="n"/>
+      <c r="M16" s="41" t="inlineStr">
+        <is>
+          <t>Падение</t>
+        </is>
+      </c>
       <c r="N16" s="42" t="n">
         <v>1753</v>
       </c>

</xml_diff>

<commit_message>
Add dynamics for uromed-m, intelmed, kriptomed
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01GGxzKXyeNbw77cRhpGHusQ
</commit_message>
<xml_diff>
--- a/out/analiz_konkurentov_reiginmed.xlsx
+++ b/out/analiz_konkurentov_reiginmed.xlsx
@@ -4489,11 +4489,19 @@
       <c r="J17" s="38" t="n">
         <v>21301</v>
       </c>
-      <c r="K17" s="131" t="n"/>
+      <c r="K17" s="131" t="inlineStr">
+        <is>
+          <t>Рост</t>
+        </is>
+      </c>
       <c r="L17" s="40" t="n">
         <v>92887</v>
       </c>
-      <c r="M17" s="41" t="n"/>
+      <c r="M17" s="41" t="inlineStr">
+        <is>
+          <t>Падение</t>
+        </is>
+      </c>
       <c r="N17" s="42" t="n">
         <v>1209</v>
       </c>
@@ -4566,11 +4574,19 @@
       <c r="J18" s="38" t="n">
         <v>2545</v>
       </c>
-      <c r="K18" s="131" t="n"/>
+      <c r="K18" s="131" t="inlineStr">
+        <is>
+          <t>Рост</t>
+        </is>
+      </c>
       <c r="L18" s="40" t="n">
         <v>47773</v>
       </c>
-      <c r="M18" s="41" t="n"/>
+      <c r="M18" s="41" t="inlineStr">
+        <is>
+          <t>Стагнация</t>
+        </is>
+      </c>
       <c r="N18" s="42" t="n">
         <v>264</v>
       </c>
@@ -4647,7 +4663,11 @@
       <c r="L19" s="40" t="n">
         <v>38052</v>
       </c>
-      <c r="M19" s="41" t="n"/>
+      <c r="M19" s="41" t="inlineStr">
+        <is>
+          <t>Стагнация</t>
+        </is>
+      </c>
       <c r="N19" s="42" t="n">
         <v>1086</v>
       </c>

</xml_diff>

<commit_message>
Add dynamics for kriptomed, fotek, medgrade
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01GGxzKXyeNbw77cRhpGHusQ
</commit_message>
<xml_diff>
--- a/out/analiz_konkurentov_reiginmed.xlsx
+++ b/out/analiz_konkurentov_reiginmed.xlsx
@@ -4659,7 +4659,11 @@
       <c r="J19" s="38" t="n">
         <v>17437</v>
       </c>
-      <c r="K19" s="131" t="n"/>
+      <c r="K19" s="131" t="inlineStr">
+        <is>
+          <t>Рост</t>
+        </is>
+      </c>
       <c r="L19" s="40" t="n">
         <v>38052</v>
       </c>
@@ -4740,11 +4744,19 @@
       <c r="J20" s="38" t="n">
         <v>4906</v>
       </c>
-      <c r="K20" s="131" t="n"/>
+      <c r="K20" s="131" t="inlineStr">
+        <is>
+          <t>Рост</t>
+        </is>
+      </c>
       <c r="L20" s="40" t="n">
         <v>9862</v>
       </c>
-      <c r="M20" s="41" t="n"/>
+      <c r="M20" s="41" t="inlineStr">
+        <is>
+          <t>Падение</t>
+        </is>
+      </c>
       <c r="N20" s="42" t="n">
         <v>319</v>
       </c>
@@ -4817,11 +4829,19 @@
       <c r="J21" s="38" t="n">
         <v>16895</v>
       </c>
-      <c r="K21" s="131" t="n"/>
+      <c r="K21" s="131" t="inlineStr">
+        <is>
+          <t>Рост</t>
+        </is>
+      </c>
       <c r="L21" s="40" t="n">
         <v>13916</v>
       </c>
-      <c r="M21" s="41" t="n"/>
+      <c r="M21" s="41" t="inlineStr">
+        <is>
+          <t>Рост</t>
+        </is>
+      </c>
       <c r="N21" s="42" t="n">
         <v>1115</v>
       </c>

</xml_diff>

<commit_message>
Set 6 leaders, add dark horse status, fix conditional formatting ranges
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01GGxzKXyeNbw77cRhpGHusQ
</commit_message>
<xml_diff>
--- a/out/analiz_konkurentov_reiginmed.xlsx
+++ b/out/analiz_konkurentov_reiginmed.xlsx
@@ -3769,7 +3769,7 @@
       </c>
       <c r="X8" s="64" t="inlineStr">
         <is>
-          <t xml:space="preserve"> Лидер</t>
+          <t xml:space="preserve"> Тёмная лошадка</t>
         </is>
       </c>
     </row>
@@ -3854,7 +3854,7 @@
       </c>
       <c r="X9" s="262" t="inlineStr">
         <is>
-          <t>Слабый конкурент</t>
+          <t xml:space="preserve"> Тёмная лошадка</t>
         </is>
       </c>
     </row>
@@ -4109,7 +4109,7 @@
       </c>
       <c r="X12" s="262" t="inlineStr">
         <is>
-          <t>Слабый конкурент</t>
+          <t xml:space="preserve"> Тёмная лошадка</t>
         </is>
       </c>
     </row>
@@ -4874,7 +4874,7 @@
       </c>
       <c r="X21" s="262" t="inlineStr">
         <is>
-          <t>Слабый конкурент</t>
+          <t xml:space="preserve"> Тёмная лошадка</t>
         </is>
       </c>
     </row>
@@ -4914,22 +4914,22 @@
       </c>
       <c r="M22" s="340" t="n"/>
       <c r="N22" s="337" t="n">
-        <v>6795</v>
+        <v>7853.5</v>
       </c>
       <c r="O22" s="337" t="n">
-        <v>24331</v>
+        <v>33354.5</v>
       </c>
       <c r="P22" s="337" t="n">
-        <v>4490</v>
+        <v>4752</v>
       </c>
       <c r="Q22" s="337" t="n">
-        <v>17355</v>
+        <v>30169</v>
       </c>
       <c r="R22" s="341" t="n">
-        <v>0.2792733549792446</v>
+        <v>0.2354554857665382</v>
       </c>
       <c r="S22" s="341" t="n">
-        <v>0.2587150677038317</v>
+        <v>0.1575126785773476</v>
       </c>
       <c r="T22" s="336" t="n">
         <v>265.5</v>
@@ -5026,7 +5026,7 @@
     </row>
   </sheetData>
   <autoFilter ref="A1:V23"/>
-  <conditionalFormatting sqref="K2:K31 M2:M31">
+  <conditionalFormatting sqref="K2:K23 M2:M23">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
       <formula>"Рост"</formula>
     </cfRule>
@@ -5043,7 +5043,7 @@
       <formula>"Сильное падение"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="K2:K31">
+  <conditionalFormatting sqref="K2:K23">
     <cfRule type="colorScale" priority="6">
       <colorScale>
         <cfvo type="min"/>
@@ -5055,7 +5055,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="H2:H29 H31">
+  <conditionalFormatting sqref="H2:H21 H23">
     <cfRule type="colorScale" priority="7">
       <colorScale>
         <cfvo type="min"/>
@@ -5067,7 +5067,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="E2:E29 E31">
+  <conditionalFormatting sqref="E2:E21 E23">
     <cfRule type="colorScale" priority="8">
       <colorScale>
         <cfvo type="min"/>
@@ -5079,7 +5079,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="U2:U29 U31">
+  <conditionalFormatting sqref="U2:U21 U23">
     <cfRule type="colorScale" priority="9">
       <colorScale>
         <cfvo type="min"/>
@@ -5091,7 +5091,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="S2:S29 S31">
+  <conditionalFormatting sqref="S2:S21 S23">
     <cfRule type="colorScale" priority="10">
       <colorScale>
         <cfvo type="min"/>
@@ -5103,7 +5103,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="T2:T29 T31">
+  <conditionalFormatting sqref="T2:T21 T23">
     <cfRule type="colorScale" priority="11">
       <colorScale>
         <cfvo type="min"/>
@@ -5115,7 +5115,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="V2:X31">
+  <conditionalFormatting sqref="V2:X23">
     <cfRule type="cellIs" priority="12" operator="equal" dxfId="0">
       <formula>" Лидер"</formula>
     </cfRule>
@@ -5132,7 +5132,7 @@
       <formula>NOT(ISERROR(SEARCH(("Более широкий"),(V2))))</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="J2:J29 J31">
+  <conditionalFormatting sqref="J2:J21 J23">
     <cfRule type="colorScale" priority="17">
       <colorScale>
         <cfvo type="min"/>
@@ -5154,7 +5154,7 @@
       <formula>LEN(TRIM(E4))&gt;0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="I2:I29 I31">
+  <conditionalFormatting sqref="I2:I21 I23">
     <cfRule type="colorScale" priority="20">
       <colorScale>
         <cfvo type="min"/>
@@ -5166,7 +5166,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="G2:G29 G31">
+  <conditionalFormatting sqref="G2:G21 G23">
     <cfRule type="colorScale" priority="21">
       <colorScale>
         <cfvo type="min"/>
@@ -5178,7 +5178,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="F2:F29 F31">
+  <conditionalFormatting sqref="F2:F21 F23">
     <cfRule type="colorScale" priority="22">
       <colorScale>
         <cfvo type="min"/>
@@ -5190,7 +5190,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="L2:L29 L31">
+  <conditionalFormatting sqref="L2:L21 L23">
     <cfRule type="colorScale" priority="23">
       <colorScale>
         <cfvo type="min"/>
@@ -5202,7 +5202,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="N2:N29 N31">
+  <conditionalFormatting sqref="N2:N21 N23">
     <cfRule type="colorScale" priority="24">
       <colorScale>
         <cfvo type="min"/>
@@ -5214,7 +5214,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="O2:O29 O31">
+  <conditionalFormatting sqref="O2:O21 O23">
     <cfRule type="colorScale" priority="25">
       <colorScale>
         <cfvo type="min"/>
@@ -5226,7 +5226,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="P2:P29 P31">
+  <conditionalFormatting sqref="P2:P21 P23">
     <cfRule type="colorScale" priority="26">
       <colorScale>
         <cfvo type="min"/>
@@ -5238,7 +5238,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="Q2:Q29 Q31">
+  <conditionalFormatting sqref="Q2:Q21 Q23">
     <cfRule type="colorScale" priority="27">
       <colorScale>
         <cfvo type="min"/>
@@ -5250,7 +5250,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="R2:R29 R31">
+  <conditionalFormatting sqref="R2:R21 R23">
     <cfRule type="colorScale" priority="28">
       <colorScale>
         <cfvo type="min"/>
@@ -5262,7 +5262,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="V2:V29 V31">
+  <conditionalFormatting sqref="V2:V21 V23">
     <cfRule type="colorScale" priority="29">
       <colorScale>
         <cfvo type="min"/>
@@ -5274,7 +5274,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="W2:W29 W31">
+  <conditionalFormatting sqref="W2:W21 W23">
     <cfRule type="colorScale" priority="30">
       <colorScale>
         <cfvo type="min"/>

</xml_diff>